<commit_message>
Simule et décompose Current policies
</commit_message>
<xml_diff>
--- a/results/Décomposition CP.xlsx
+++ b/results/Décomposition CP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flori\Documents\Github\ThreeME_V3-ADEME\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B9CA82-ADEA-4966-9542-A8629AEE2986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10942160-48B6-4095-893D-0557620857BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{64203D87-38B7-4BDD-A33D-820F861F4EFC}"/>
   </bookViews>
@@ -55,7 +55,7 @@
     <t>NZP</t>
   </si>
   <si>
-    <t>Net Zero</t>
+    <t>Current policies</t>
   </si>
 </sst>
 </file>
@@ -147,20 +147,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="fr-FR" sz="2400"/>
-              <a:t>Décomposition scénario Net Zero (% du PIB)</a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="2400"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="fr-FR" sz="1600"/>
-              <a:t>incluant</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="fr-FR" sz="1600" baseline="0"/>
-              <a:t> les risques physiques</a:t>
+              <a:t>Décomposition scénario Current policies (% du PIB)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -169,8 +156,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.20501902519546519"/>
-          <c:y val="2.9335174245866687E-2"/>
+          <c:x val="0.16677612924894331"/>
+          <c:y val="2.3053340517596718E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -201,7 +188,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="7.0272504293453358E-2"/>
+          <c:y val="0.11366458767098624"/>
+          <c:w val="0.91470350087041308"/>
+          <c:h val="0.72163232707480229"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="stacked"/>
@@ -522,238 +519,238 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-0.19694161232846064</c:v>
+                  <c:v>0.19161550315185405</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-0.32910460472266312</c:v>
+                  <c:v>0.31789887951911844</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-8.0637713317255333E-2</c:v>
+                  <c:v>6.7015030786099494E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.20258876617191834</c:v>
+                  <c:v>-0.21728167797012699</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.45424694424371914</c:v>
+                  <c:v>-0.46886133701437016</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.6611727771178133</c:v>
+                  <c:v>-0.67638884472317473</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.83719057505624583</c:v>
+                  <c:v>-0.85375889954031337</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.0028947161887292</c:v>
+                  <c:v>-1.0207112465597246</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1.1571750805414949</c:v>
+                  <c:v>-1.1759379933896641</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.2887400597361598</c:v>
+                  <c:v>-1.307531973432452</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1.3742398781701581</c:v>
+                  <c:v>-1.3941416492964653</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.4290171313425803</c:v>
+                  <c:v>-1.4508647654808193</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1.4675920150303501</c:v>
+                  <c:v>-1.4919916852337844</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.4991113762324426</c:v>
+                  <c:v>-1.5264967867797408</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.5278210019538108</c:v>
+                  <c:v>-1.5576296940993828</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.5537649183268609</c:v>
+                  <c:v>-1.5861667841999827</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.5768060907918269</c:v>
+                  <c:v>-1.6118588854758364</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.5965658939140592</c:v>
+                  <c:v>-1.6342925349397075</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.6125052003735707</c:v>
+                  <c:v>-1.6529130346936594</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1.6238872985003372</c:v>
+                  <c:v>-1.6664774336045296</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1.6292175777404383</c:v>
+                  <c:v>-1.6738659693794067</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1.6302196584468298</c:v>
+                  <c:v>-1.6767182125922653</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1.6294193971467585</c:v>
+                  <c:v>-1.677493043235545</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1.628626915129705</c:v>
+                  <c:v>-1.6779763018033189</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1.6291172996173886</c:v>
+                  <c:v>-1.6790908599914611</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1.6304594714892096</c:v>
+                  <c:v>-1.6807531170653367</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1.6346407218347014</c:v>
+                  <c:v>-1.6849090679153078</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1.6454229613436233</c:v>
+                  <c:v>-1.6952498621138901</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1.6696180039645014</c:v>
+                  <c:v>-1.7184393048263136</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>1.6889441686418261</c:v>
+                  <c:v>-1.7362029288578218</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>1.7078428405991497</c:v>
+                  <c:v>-1.7534246166071354</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>1.7236337283863978</c:v>
+                  <c:v>-1.7675856069250262</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>1.7349248053407429</c:v>
+                  <c:v>-1.7775623333425861</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>1.7411540936693504</c:v>
+                  <c:v>-1.7830030310172607</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>1.7428896953826323</c:v>
+                  <c:v>-1.7843857765953541</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>1.7398540828657216</c:v>
+                  <c:v>-1.7814809968153322</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>1.7329147309208093</c:v>
+                  <c:v>-1.7750230330517369</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>1.7230862359691956</c:v>
+                  <c:v>-1.7659091624286583</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>1.7113712076963328</c:v>
+                  <c:v>-1.7550687062752313</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>1.6991510984826208</c:v>
+                  <c:v>-1.7437581416538506</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>1.6866072217296857</c:v>
+                  <c:v>-1.7322399317636572</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>1.6742464005973456</c:v>
+                  <c:v>-1.7209837178788767</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>1.6623965816549013</c:v>
+                  <c:v>-1.7102969143967806</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>1.6512509308354018</c:v>
+                  <c:v>-1.7003514750675741</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>1.6524822554548013</c:v>
+                  <c:v>-1.7041717945534995</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>1.6450248394999534</c:v>
+                  <c:v>-1.6968611913178111</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>1.6348458928615806</c:v>
+                  <c:v>-1.6874204618492761</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>1.6242837620730421</c:v>
+                  <c:v>-1.6779987060296264</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>1.6146046053609364</c:v>
+                  <c:v>-1.6695997980133215</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>1.6075645605232003</c:v>
+                  <c:v>-1.6637538837163346</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>1.6016081837933793</c:v>
+                  <c:v>-1.6589740264339237</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>1.5966635898912562</c:v>
+                  <c:v>-1.6551568536300354</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>1.5925545300034649</c:v>
+                  <c:v>-1.6521136575608164</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>1.5891372665503889</c:v>
+                  <c:v>-1.6496961346720851</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>1.5863392639233309</c:v>
+                  <c:v>-1.647812183467412</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>1.5841510083471011</c:v>
+                  <c:v>-1.6464745156678506</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>1.5826012084538377</c:v>
+                  <c:v>-1.6457143828054077</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>1.5817315368870766</c:v>
+                  <c:v>-1.6455781760776222</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>1.5815791282935976</c:v>
+                  <c:v>-1.6461074372563056</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>1.5833859626567248</c:v>
+                  <c:v>-1.6484945595247713</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>1.585692472380229</c:v>
+                  <c:v>-1.6513493411040914</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>1.5886108369449925</c:v>
+                  <c:v>-1.6547799298626154</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>1.5921782276750784</c:v>
+                  <c:v>-1.6588215817661012</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>1.5963952313138297</c:v>
+                  <c:v>-1.663474348417826</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>1.6012455941350368</c:v>
+                  <c:v>-1.668749189340446</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>1.6067094578869234</c:v>
+                  <c:v>-1.6745957993986593</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>1.6127694246065971</c:v>
+                  <c:v>-1.6809976191283882</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>1.6194122415741141</c:v>
+                  <c:v>-1.6879396819433956</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>1.6266274009712811</c:v>
+                  <c:v>-1.6954091313694963</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>1.6354020493762667</c:v>
+                  <c:v>-1.7043809443399893</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>1.6445477994649904</c:v>
+                  <c:v>-1.7136818328981618</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>1.6541465898829877</c:v>
+                  <c:v>-1.7233900154516202</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>1.6642258451554426</c:v>
+                  <c:v>-1.733529893763619</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>1.6747892448942148</c:v>
+                  <c:v>-1.7441041249341871</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>1.6858325017146347</c:v>
+                  <c:v>-1.7551879809414861</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>1.6973521339859632</c:v>
+                  <c:v>-1.7666911636200933</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>1.7093489455747068</c:v>
+                  <c:v>-1.7709894968797713</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>1.7218275243293002</c:v>
+                  <c:v>-1.7897149040786542</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1062,256 +1059,256 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-0.11989295890919571</c:v>
+                  <c:v>9.1492751157495888E-4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-0.2564913650720313</c:v>
+                  <c:v>1.9380107544986203E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.40548218803949654</c:v>
+                  <c:v>3.0370170623905679E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-0.5625868560056535</c:v>
+                  <c:v>4.1803820710395456E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-0.72368591578868546</c:v>
+                  <c:v>5.3381698501331343E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-0.89397615754910342</c:v>
+                  <c:v>1.3157759753057441E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-1.0567432216490147</c:v>
+                  <c:v>2.1869550496589341E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-1.2174431340904013</c:v>
+                  <c:v>3.1205429864034073E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-1.3857419717199115</c:v>
+                  <c:v>4.0713713050877232E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-1.5525404083190808</c:v>
+                  <c:v>5.0225662190184206E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-1.6975277268560407</c:v>
+                  <c:v>3.4202433463459414E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-1.8352635592671529</c:v>
+                  <c:v>1.4793136806567908E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-1.9665730589535579</c:v>
+                  <c:v>-7.2514210232244025E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-2.0933483687798016</c:v>
+                  <c:v>-3.085749985403119E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-2.2165809291794014</c:v>
+                  <c:v>-5.5171737536308108E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-2.3070973213381696</c:v>
+                  <c:v>-0.11527060202289885</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-2.3896751137264083</c:v>
+                  <c:v>-0.18005917742343058</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-2.4660827682109754</c:v>
+                  <c:v>-0.24835479296698715</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-2.5383588193067186</c:v>
+                  <c:v>-0.31854407319406031</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-2.6081115523742371</c:v>
+                  <c:v>-0.38934787782083369</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-2.6511689414570383</c:v>
+                  <c:v>-0.48466297679704562</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-2.6894213690852653</c:v>
+                  <c:v>-0.58310328090575014</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-2.7241402903304679</c:v>
+                  <c:v>-0.68367940434092001</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-2.7567615498774622</c:v>
+                  <c:v>-0.78519266864072179</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-2.7883597387506676</c:v>
+                  <c:v>-0.88673461819119836</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-2.8089696518258989</c:v>
+                  <c:v>-0.99484702484020637</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-2.8278862818979622</c:v>
+                  <c:v>-1.1032786996437394</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-2.845736679362898</c:v>
+                  <c:v>-1.2116345953177454</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-2.863135454837773</c:v>
+                  <c:v>-1.3194987188833385</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-2.8804855301895693</c:v>
+                  <c:v>-1.4265799471028462</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-2.8905830206418348</c:v>
+                  <c:v>-1.537828170077804</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-2.8996181842041446</c:v>
+                  <c:v>-1.648887146879241</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-2.9079007847959693</c:v>
+                  <c:v>-1.7595417723946905</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-2.9158011348523805</c:v>
+                  <c:v>-1.86950345626683</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-2.9236390587223049</c:v>
+                  <c:v>-1.9784768298969579</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-2.9231993950436297</c:v>
+                  <c:v>-2.0855284564764931</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-2.9209666867608841</c:v>
+                  <c:v>-2.1914673157060083</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-2.9171231204214498</c:v>
+                  <c:v>-2.2963811629559849</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-2.911769206946091</c:v>
+                  <c:v>-2.4004268917252487</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-2.9049518599424506</c:v>
+                  <c:v>-2.5037356931093768</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-2.8940385324500828</c:v>
+                  <c:v>-2.6061166260749169</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-2.8814726221983555</c:v>
+                  <c:v>-2.7077912959215582</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-2.8675560755517027</c:v>
+                  <c:v>-2.8087819035527262</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-2.852573828002114</c:v>
+                  <c:v>-2.909098413265665</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-2.8367375662116778</c:v>
+                  <c:v>-3.0087429095384306</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-2.8184388359486112</c:v>
+                  <c:v>-3.1026399639058284</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-2.7992687429579166</c:v>
+                  <c:v>-3.1948333767250814</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-2.7794087331449391</c:v>
+                  <c:v>-3.2855143293944344</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-2.7590268287936426</c:v>
+                  <c:v>-3.3749499344847833</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-2.7382610472803992</c:v>
+                  <c:v>-3.4633544987890392</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-2.7204879688719319</c:v>
+                  <c:v>-3.5458701493699452</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-2.7056687985878014</c:v>
+                  <c:v>-3.6286311881190696</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-2.6905274014482505</c:v>
+                  <c:v>-3.7100210959082669</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-2.6751000655087287</c:v>
+                  <c:v>-3.7902081892557726</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>-2.6595309848436721</c:v>
+                  <c:v>-3.8693535099939775</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>-2.6426427140642361</c:v>
+                  <c:v>-3.9463127746038218</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>-2.6255265773697301</c:v>
+                  <c:v>-4.0221721575330438</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>-2.6082886651969006</c:v>
+                  <c:v>-4.0970219103658607</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>-2.5910266586371855</c:v>
+                  <c:v>-4.170955718841018</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>-2.5738164372193006</c:v>
+                  <c:v>-4.2440590458176164</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>-2.5564159346071147</c:v>
+                  <c:v>-4.314918856613903</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>-2.5391159005227371</c:v>
+                  <c:v>-4.3847466334413614</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>-2.5219623175955053</c:v>
+                  <c:v>-4.4536575845551596</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>-2.5049927014446194</c:v>
+                  <c:v>-4.5217748416950698</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>-2.4882326476251326</c:v>
+                  <c:v>-4.5891841340081063</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>-2.4711414631061412</c:v>
+                  <c:v>-4.6500669729501958</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>-2.4542179509998263</c:v>
+                  <c:v>-4.7091084258238824</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>-2.4374982348842056</c:v>
+                  <c:v>-4.766532007184221</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>-2.4210155162512792</c:v>
+                  <c:v>-4.822628127561801</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>-2.4047947478542997</c:v>
+                  <c:v>-4.8776257331803574</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>-2.3892334662780068</c:v>
+                  <c:v>-4.9292242743100285</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>-2.3740351065630216</c:v>
+                  <c:v>-4.9794617875934089</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>-2.3591939516777072</c:v>
+                  <c:v>-5.028529121718905</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>-2.344700190984228</c:v>
+                  <c:v>-5.0766333496403586</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>-2.3305456139527836</c:v>
+                  <c:v>-5.1239370559427844</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>-2.3167305493591472</c:v>
+                  <c:v>-5.1656385463514258</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>-2.303268027977734</c:v>
+                  <c:v>-5.2057448609437831</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>-2.2901533128280693</c:v>
+                  <c:v>-5.2445009570563741</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>-2.2773826674107212</c:v>
+                  <c:v>-5.2821935370182871</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>-2.264953178116369</c:v>
+                  <c:v>-5.3190444847133094</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>-2.2538427520225501</c:v>
+                  <c:v>-5.3544346165925845</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>-2.2432380041915723</c:v>
+                  <c:v>-5.3891368459431321</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>-2.2408179811543416</c:v>
+                  <c:v>-5.423664191250765</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>-2.2246311597601487</c:v>
+                  <c:v>-5.456897085822666</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1347,7 +1344,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Net Zero</c:v>
+                  <c:v>Current policies</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1638,256 +1635,256 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-0.11989295890919571</c:v>
+                  <c:v>9.1492751157495888E-4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-0.2564913650720313</c:v>
+                  <c:v>1.9380107544986203E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.40548218803949654</c:v>
+                  <c:v>3.0370170623905679E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-0.5625868560056535</c:v>
+                  <c:v>4.1803820710395456E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-0.72368591578868546</c:v>
+                  <c:v>5.3381698501331343E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-0.89397615754910342</c:v>
+                  <c:v>1.3157759753057441E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-1.2536848339774753</c:v>
+                  <c:v>0.21348505364844339</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-1.5465477388130644</c:v>
+                  <c:v>0.34910430938315251</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-1.4663796850371669</c:v>
+                  <c:v>0.10772874383697673</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-1.3499516421471625</c:v>
+                  <c:v>-0.16705601577994278</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-1.2432807826123216</c:v>
+                  <c:v>-0.43465890355091075</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-1.1740907821493396</c:v>
+                  <c:v>-0.66159570791660682</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-1.1293824838973121</c:v>
+                  <c:v>-0.86101032056353777</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-1.0904536525910724</c:v>
+                  <c:v>-1.0515687464137558</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-1.0594058486379065</c:v>
+                  <c:v>-1.2311097309259722</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.0183572616020098</c:v>
+                  <c:v>-1.4228025754553508</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-1.0154352355562501</c:v>
+                  <c:v>-1.5742008267198959</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-1.037065636868395</c:v>
+                  <c:v>-1.6992195584478065</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-1.0707668042763685</c:v>
+                  <c:v>-1.8105357584278448</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-1.1090001761417945</c:v>
+                  <c:v>-1.9158446646005745</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-1.1233479395032275</c:v>
+                  <c:v>-2.0422926708964284</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-1.1356564507584044</c:v>
+                  <c:v>-2.1692700651057328</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-1.147334199538641</c:v>
+                  <c:v>-2.2955382898167564</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-1.160195655963403</c:v>
+                  <c:v>-2.4194852035804293</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-1.1758545383770969</c:v>
+                  <c:v>-2.5396476528848577</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-1.1850823533255617</c:v>
+                  <c:v>-2.661324458444736</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-1.1986687041575239</c:v>
+                  <c:v>-2.7771446690231461</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-1.2155170209160682</c:v>
+                  <c:v>-2.8883528079100107</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-1.2337160576910144</c:v>
+                  <c:v>-2.9969917621188835</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-1.2518586150598643</c:v>
+                  <c:v>-3.1045562489061651</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-1.2614657210244462</c:v>
+                  <c:v>-3.2169190300692652</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-1.2691587127149351</c:v>
+                  <c:v>-3.3296402639445777</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-1.2732600629612678</c:v>
+                  <c:v>-3.4444508403099983</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-1.2703781735087571</c:v>
+                  <c:v>-3.5647533183807201</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-1.2540210547578035</c:v>
+                  <c:v>-3.6969161347232715</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-1.2342552264018036</c:v>
+                  <c:v>-3.8217313853343149</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-1.2131238461617344</c:v>
+                  <c:v>-3.9448919323131437</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-1.193489392035052</c:v>
+                  <c:v>-4.0639667698810111</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-1.1768444016053481</c:v>
+                  <c:v>-4.1779892250678348</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-1.1637977662731003</c:v>
+                  <c:v>-4.2867387241266375</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-1.1511488370674505</c:v>
+                  <c:v>-4.390502402670271</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-1.1416185393326339</c:v>
+                  <c:v>-4.4892722927368904</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-1.1346413446308934</c:v>
+                  <c:v>-4.5838049366044631</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-1.1294875920329184</c:v>
+                  <c:v>-4.6750075756943232</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-1.1253663585153451</c:v>
+                  <c:v>-4.7638116158136619</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-1.1192877374659904</c:v>
+                  <c:v>-4.846398105559679</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-1.1126615212282309</c:v>
+                  <c:v>-4.9270733084887386</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-1.1051623325475934</c:v>
+                  <c:v>-5.0064980472733112</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-1.0966302471387412</c:v>
+                  <c:v>-5.0852468488815639</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-1.0870101164449975</c:v>
+                  <c:v>-5.1637059738566133</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-1.0680057134171306</c:v>
+                  <c:v>-5.2500419439234447</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-1.060643959087848</c:v>
+                  <c:v>-5.3254923794368807</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-1.05568150858667</c:v>
+                  <c:v>-5.397441557757543</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-1.0508163034356865</c:v>
+                  <c:v>-5.468206895285399</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>-1.0449263794827357</c:v>
+                  <c:v>-5.538953308007299</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>-1.0350781535410358</c:v>
+                  <c:v>-5.6100666583201564</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>-1.0239183935763507</c:v>
+                  <c:v>-5.6811461839669679</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>-1.0116250753056444</c:v>
+                  <c:v>-5.7521787639958966</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>-0.99847212863372059</c:v>
+                  <c:v>-5.8230693764018344</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>-0.98467917066891175</c:v>
+                  <c:v>-5.8937551804897019</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>-0.97007667068378378</c:v>
+                  <c:v>-5.9627310400813149</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>-0.95496489217563596</c:v>
+                  <c:v>-6.0312211491092116</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>-0.93936110914166759</c:v>
+                  <c:v>-6.0993719673605673</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>-0.92326116455754281</c:v>
+                  <c:v>-6.1673530177726921</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>-0.90665351933153504</c:v>
+                  <c:v>-6.2352915712644119</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>-0.88775550044941642</c:v>
+                  <c:v>-6.2985615324749666</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>-0.86852547861959728</c:v>
+                  <c:v>-6.3604577669279738</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>-0.84888739793921308</c:v>
+                  <c:v>-6.4213119370468359</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>-0.82883728857620076</c:v>
+                  <c:v>-6.4814497093279027</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>-0.80839951654047004</c:v>
+                  <c:v>-6.5411000815981835</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>-0.78798787214297006</c:v>
+                  <c:v>-6.597973463650475</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>-0.7673256486760982</c:v>
+                  <c:v>-6.6540575869920682</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>-0.74642452707111007</c:v>
+                  <c:v>-6.7095267408472932</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>-0.72528794941011387</c:v>
+                  <c:v>-6.7645730315837538</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>-0.70391821298150248</c:v>
+                  <c:v>-6.8193461873122807</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>-0.68132849998288059</c:v>
+                  <c:v>-6.8700194906914147</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>-0.65872022851274359</c:v>
+                  <c:v>-6.9194266938419453</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>-0.63600672294508165</c:v>
+                  <c:v>-6.9678909725079947</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>-0.61315682225527857</c:v>
+                  <c:v>-7.0157234307819056</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>-0.59016393322215421</c:v>
+                  <c:v>-7.063148609647496</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>-0.56801025030791541</c:v>
+                  <c:v>-7.109622597534071</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>-0.54588587020560908</c:v>
+                  <c:v>-7.1558280095632254</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>-0.53146903557963476</c:v>
+                  <c:v>-7.1946536881305363</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>-0.50280363543084849</c:v>
+                  <c:v>-7.2466119899013197</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2028,6 +2025,16 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13363386341758349"/>
+          <c:y val="0.92513059948808829"/>
+          <c:w val="0.73273216562013122"/>
+          <c:h val="5.8117843903191829E-2"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2706,6 +2713,8 @@
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Données"/>
+      <sheetName val="Graphique1"/>
+      <sheetName val="Graphique1 (2)"/>
       <sheetName val="Gr Macro"/>
       <sheetName val="Gr inflation"/>
       <sheetName val="Gr émissions"/>
@@ -2758,270 +2767,244 @@
             <v>0</v>
           </cell>
           <cell r="J5">
-            <v>-0.19694161232846064</v>
+            <v>0.19161550315185405</v>
           </cell>
           <cell r="K5">
-            <v>-0.32910460472266312</v>
+            <v>0.31789887951911844</v>
           </cell>
           <cell r="L5">
-            <v>-8.0637713317255333E-2</v>
+            <v>6.7015030786099494E-2</v>
           </cell>
           <cell r="M5">
-            <v>0.20258876617191834</v>
+            <v>-0.21728167797012699</v>
           </cell>
           <cell r="N5">
-            <v>0.45424694424371914</v>
+            <v>-0.46886133701437016</v>
           </cell>
           <cell r="O5">
-            <v>0.6611727771178133</v>
+            <v>-0.67638884472317473</v>
           </cell>
           <cell r="P5">
-            <v>0.83719057505624583</v>
+            <v>-0.85375889954031337</v>
           </cell>
           <cell r="Q5">
-            <v>1.0028947161887292</v>
+            <v>-1.0207112465597246</v>
           </cell>
           <cell r="R5">
-            <v>1.1571750805414949</v>
+            <v>-1.1759379933896641</v>
           </cell>
           <cell r="S5">
-            <v>1.2887400597361598</v>
+            <v>-1.307531973432452</v>
           </cell>
           <cell r="T5">
-            <v>1.3742398781701581</v>
+            <v>-1.3941416492964653</v>
           </cell>
           <cell r="U5">
-            <v>1.4290171313425803</v>
+            <v>-1.4508647654808193</v>
           </cell>
           <cell r="V5">
-            <v>1.4675920150303501</v>
+            <v>-1.4919916852337844</v>
           </cell>
           <cell r="W5">
-            <v>1.4991113762324426</v>
+            <v>-1.5264967867797408</v>
           </cell>
           <cell r="X5">
-            <v>1.5278210019538108</v>
+            <v>-1.5576296940993828</v>
           </cell>
           <cell r="Y5">
-            <v>1.5537649183268609</v>
+            <v>-1.5861667841999827</v>
           </cell>
           <cell r="Z5">
-            <v>1.5768060907918269</v>
+            <v>-1.6118588854758364</v>
           </cell>
           <cell r="AA5">
-            <v>1.5965658939140592</v>
+            <v>-1.6342925349397075</v>
           </cell>
           <cell r="AB5">
-            <v>1.6125052003735707</v>
+            <v>-1.6529130346936594</v>
           </cell>
           <cell r="AC5">
-            <v>1.6238872985003372</v>
+            <v>-1.6664774336045296</v>
           </cell>
           <cell r="AD5">
-            <v>1.6292175777404383</v>
+            <v>-1.6738659693794067</v>
           </cell>
           <cell r="AE5">
-            <v>1.6302196584468298</v>
+            <v>-1.6767182125922653</v>
           </cell>
           <cell r="AF5">
-            <v>1.6294193971467585</v>
+            <v>-1.677493043235545</v>
           </cell>
           <cell r="AG5">
-            <v>1.628626915129705</v>
+            <v>-1.6779763018033189</v>
           </cell>
           <cell r="AH5">
-            <v>1.6291172996173886</v>
+            <v>-1.6790908599914611</v>
           </cell>
           <cell r="AI5">
-            <v>1.6304594714892096</v>
+            <v>-1.6807531170653367</v>
           </cell>
           <cell r="AJ5">
-            <v>1.6346407218347014</v>
+            <v>-1.6849090679153078</v>
           </cell>
           <cell r="AK5">
-            <v>1.6454229613436233</v>
+            <v>-1.6952498621138901</v>
           </cell>
           <cell r="AL5">
-            <v>1.6696180039645014</v>
+            <v>-1.7184393048263136</v>
           </cell>
           <cell r="AM5">
-            <v>1.6889441686418261</v>
+            <v>-1.7362029288578218</v>
           </cell>
           <cell r="AN5">
-            <v>1.7078428405991497</v>
+            <v>-1.7534246166071354</v>
           </cell>
           <cell r="AO5">
-            <v>1.7236337283863978</v>
+            <v>-1.7675856069250262</v>
           </cell>
           <cell r="AP5">
-            <v>1.7349248053407429</v>
+            <v>-1.7775623333425861</v>
           </cell>
           <cell r="AQ5">
-            <v>1.7411540936693504</v>
+            <v>-1.7830030310172607</v>
           </cell>
           <cell r="AR5">
-            <v>1.7428896953826323</v>
+            <v>-1.7843857765953541</v>
           </cell>
           <cell r="AS5">
-            <v>1.7398540828657216</v>
+            <v>-1.7814809968153322</v>
           </cell>
           <cell r="AT5">
-            <v>1.7329147309208093</v>
+            <v>-1.7750230330517369</v>
           </cell>
           <cell r="AU5">
-            <v>1.7230862359691956</v>
+            <v>-1.7659091624286583</v>
           </cell>
           <cell r="AV5">
-            <v>1.7113712076963328</v>
+            <v>-1.7550687062752313</v>
           </cell>
           <cell r="AW5">
-            <v>1.6991510984826208</v>
+            <v>-1.7437581416538506</v>
           </cell>
           <cell r="AX5">
-            <v>1.6866072217296857</v>
+            <v>-1.7322399317636572</v>
           </cell>
           <cell r="AY5">
-            <v>1.6742464005973456</v>
+            <v>-1.7209837178788767</v>
           </cell>
           <cell r="AZ5">
-            <v>1.6623965816549013</v>
+            <v>-1.7102969143967806</v>
           </cell>
           <cell r="BA5">
-            <v>1.6512509308354018</v>
+            <v>-1.7003514750675741</v>
           </cell>
           <cell r="BB5">
-            <v>1.6524822554548013</v>
+            <v>-1.7041717945534995</v>
           </cell>
           <cell r="BC5">
-            <v>1.6450248394999534</v>
+            <v>-1.6968611913178111</v>
           </cell>
           <cell r="BD5">
-            <v>1.6348458928615806</v>
+            <v>-1.6874204618492761</v>
           </cell>
           <cell r="BE5">
-            <v>1.6242837620730421</v>
+            <v>-1.6779987060296264</v>
           </cell>
           <cell r="BF5">
-            <v>1.6146046053609364</v>
+            <v>-1.6695997980133215</v>
           </cell>
           <cell r="BG5">
-            <v>1.6075645605232003</v>
+            <v>-1.6637538837163346</v>
           </cell>
           <cell r="BH5">
-            <v>1.6016081837933793</v>
+            <v>-1.6589740264339237</v>
           </cell>
           <cell r="BI5">
-            <v>1.5966635898912562</v>
+            <v>-1.6551568536300354</v>
           </cell>
           <cell r="BJ5">
-            <v>1.5925545300034649</v>
+            <v>-1.6521136575608164</v>
           </cell>
           <cell r="BK5">
-            <v>1.5891372665503889</v>
+            <v>-1.6496961346720851</v>
           </cell>
           <cell r="BL5">
-            <v>1.5863392639233309</v>
+            <v>-1.647812183467412</v>
           </cell>
           <cell r="BM5">
-            <v>1.5841510083471011</v>
+            <v>-1.6464745156678506</v>
           </cell>
           <cell r="BN5">
-            <v>1.5826012084538377</v>
+            <v>-1.6457143828054077</v>
           </cell>
           <cell r="BO5">
-            <v>1.5817315368870766</v>
+            <v>-1.6455781760776222</v>
           </cell>
           <cell r="BP5">
-            <v>1.5815791282935976</v>
+            <v>-1.6461074372563056</v>
           </cell>
           <cell r="BQ5">
-            <v>1.5833859626567248</v>
+            <v>-1.6484945595247713</v>
           </cell>
           <cell r="BR5">
-            <v>1.585692472380229</v>
+            <v>-1.6513493411040914</v>
           </cell>
           <cell r="BS5">
-            <v>1.5886108369449925</v>
+            <v>-1.6547799298626154</v>
           </cell>
           <cell r="BT5">
-            <v>1.5921782276750784</v>
+            <v>-1.6588215817661012</v>
           </cell>
           <cell r="BU5">
-            <v>1.5963952313138297</v>
+            <v>-1.663474348417826</v>
           </cell>
           <cell r="BV5">
-            <v>1.6012455941350368</v>
+            <v>-1.668749189340446</v>
           </cell>
           <cell r="BW5">
-            <v>1.6067094578869234</v>
+            <v>-1.6745957993986593</v>
           </cell>
           <cell r="BX5">
-            <v>1.6127694246065971</v>
+            <v>-1.6809976191283882</v>
           </cell>
           <cell r="BY5">
-            <v>1.6194122415741141</v>
+            <v>-1.6879396819433956</v>
           </cell>
           <cell r="BZ5">
-            <v>1.6266274009712811</v>
+            <v>-1.6954091313694963</v>
           </cell>
           <cell r="CA5">
-            <v>1.6354020493762667</v>
+            <v>-1.7043809443399893</v>
           </cell>
           <cell r="CB5">
-            <v>1.6445477994649904</v>
+            <v>-1.7136818328981618</v>
           </cell>
           <cell r="CC5">
-            <v>1.6541465898829877</v>
+            <v>-1.7233900154516202</v>
           </cell>
           <cell r="CD5">
-            <v>1.6642258451554426</v>
+            <v>-1.733529893763619</v>
           </cell>
           <cell r="CE5">
-            <v>1.6747892448942148</v>
+            <v>-1.7441041249341871</v>
           </cell>
           <cell r="CF5">
-            <v>1.6858325017146347</v>
+            <v>-1.7551879809414861</v>
           </cell>
           <cell r="CG5">
-            <v>1.6973521339859632</v>
+            <v>-1.7666911636200933</v>
           </cell>
           <cell r="CH5">
-            <v>1.7093489455747068</v>
+            <v>-1.7709894968797713</v>
           </cell>
           <cell r="CI5">
-            <v>1.7218275243293002</v>
+            <v>-1.7897149040786542</v>
           </cell>
           <cell r="CJ5">
-            <v>1.7347940252342653</v>
+            <v>-1.3563380790536539</v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24" refreshError="1"/>
-      <sheetData sheetId="25" refreshError="1"/>
-      <sheetData sheetId="26" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3331,259 +3314,259 @@
             <v>0</v>
           </cell>
           <cell r="D5">
-            <v>-0.11989295890919571</v>
+            <v>9.1492751157495888E-4</v>
           </cell>
           <cell r="E5">
-            <v>-0.2564913650720313</v>
+            <v>1.9380107544986203E-3</v>
           </cell>
           <cell r="F5">
-            <v>-0.40548218803949654</v>
+            <v>3.0370170623905679E-3</v>
           </cell>
           <cell r="G5">
-            <v>-0.5625868560056535</v>
+            <v>4.1803820710395456E-3</v>
           </cell>
           <cell r="H5">
-            <v>-0.72368591578868546</v>
+            <v>5.3381698501331343E-3</v>
           </cell>
           <cell r="I5">
-            <v>-0.89397615754910342</v>
+            <v>1.3157759753057441E-2</v>
           </cell>
           <cell r="J5">
-            <v>-1.2536848339774753</v>
+            <v>0.21348505364844339</v>
           </cell>
           <cell r="K5">
-            <v>-1.5465477388130644</v>
+            <v>0.34910430938315251</v>
           </cell>
           <cell r="L5">
-            <v>-1.4663796850371669</v>
+            <v>0.10772874383697673</v>
           </cell>
           <cell r="M5">
-            <v>-1.3499516421471625</v>
+            <v>-0.16705601577994278</v>
           </cell>
           <cell r="N5">
-            <v>-1.2432807826123216</v>
+            <v>-0.43465890355091075</v>
           </cell>
           <cell r="O5">
-            <v>-1.1740907821493396</v>
+            <v>-0.66159570791660682</v>
           </cell>
           <cell r="P5">
-            <v>-1.1293824838973121</v>
+            <v>-0.86101032056353777</v>
           </cell>
           <cell r="Q5">
-            <v>-1.0904536525910724</v>
+            <v>-1.0515687464137558</v>
           </cell>
           <cell r="R5">
-            <v>-1.0594058486379065</v>
+            <v>-1.2311097309259722</v>
           </cell>
           <cell r="S5">
-            <v>-1.0183572616020098</v>
+            <v>-1.4228025754553508</v>
           </cell>
           <cell r="T5">
-            <v>-1.0154352355562501</v>
+            <v>-1.5742008267198959</v>
           </cell>
           <cell r="U5">
-            <v>-1.037065636868395</v>
+            <v>-1.6992195584478065</v>
           </cell>
           <cell r="V5">
-            <v>-1.0707668042763685</v>
+            <v>-1.8105357584278448</v>
           </cell>
           <cell r="W5">
-            <v>-1.1090001761417945</v>
+            <v>-1.9158446646005745</v>
           </cell>
           <cell r="X5">
-            <v>-1.1233479395032275</v>
+            <v>-2.0422926708964284</v>
           </cell>
           <cell r="Y5">
-            <v>-1.1356564507584044</v>
+            <v>-2.1692700651057328</v>
           </cell>
           <cell r="Z5">
-            <v>-1.147334199538641</v>
+            <v>-2.2955382898167564</v>
           </cell>
           <cell r="AA5">
-            <v>-1.160195655963403</v>
+            <v>-2.4194852035804293</v>
           </cell>
           <cell r="AB5">
-            <v>-1.1758545383770969</v>
+            <v>-2.5396476528848577</v>
           </cell>
           <cell r="AC5">
-            <v>-1.1850823533255617</v>
+            <v>-2.661324458444736</v>
           </cell>
           <cell r="AD5">
-            <v>-1.1986687041575239</v>
+            <v>-2.7771446690231461</v>
           </cell>
           <cell r="AE5">
-            <v>-1.2155170209160682</v>
+            <v>-2.8883528079100107</v>
           </cell>
           <cell r="AF5">
-            <v>-1.2337160576910144</v>
+            <v>-2.9969917621188835</v>
           </cell>
           <cell r="AG5">
-            <v>-1.2518586150598643</v>
+            <v>-3.1045562489061651</v>
           </cell>
           <cell r="AH5">
-            <v>-1.2614657210244462</v>
+            <v>-3.2169190300692652</v>
           </cell>
           <cell r="AI5">
-            <v>-1.2691587127149351</v>
+            <v>-3.3296402639445777</v>
           </cell>
           <cell r="AJ5">
-            <v>-1.2732600629612678</v>
+            <v>-3.4444508403099983</v>
           </cell>
           <cell r="AK5">
-            <v>-1.2703781735087571</v>
+            <v>-3.5647533183807201</v>
           </cell>
           <cell r="AL5">
-            <v>-1.2540210547578035</v>
+            <v>-3.6969161347232715</v>
           </cell>
           <cell r="AM5">
-            <v>-1.2342552264018036</v>
+            <v>-3.8217313853343149</v>
           </cell>
           <cell r="AN5">
-            <v>-1.2131238461617344</v>
+            <v>-3.9448919323131437</v>
           </cell>
           <cell r="AO5">
-            <v>-1.193489392035052</v>
+            <v>-4.0639667698810111</v>
           </cell>
           <cell r="AP5">
-            <v>-1.1768444016053481</v>
+            <v>-4.1779892250678348</v>
           </cell>
           <cell r="AQ5">
-            <v>-1.1637977662731003</v>
+            <v>-4.2867387241266375</v>
           </cell>
           <cell r="AR5">
-            <v>-1.1511488370674505</v>
+            <v>-4.390502402670271</v>
           </cell>
           <cell r="AS5">
-            <v>-1.1416185393326339</v>
+            <v>-4.4892722927368904</v>
           </cell>
           <cell r="AT5">
-            <v>-1.1346413446308934</v>
+            <v>-4.5838049366044631</v>
           </cell>
           <cell r="AU5">
-            <v>-1.1294875920329184</v>
+            <v>-4.6750075756943232</v>
           </cell>
           <cell r="AV5">
-            <v>-1.1253663585153451</v>
+            <v>-4.7638116158136619</v>
           </cell>
           <cell r="AW5">
-            <v>-1.1192877374659904</v>
+            <v>-4.846398105559679</v>
           </cell>
           <cell r="AX5">
-            <v>-1.1126615212282309</v>
+            <v>-4.9270733084887386</v>
           </cell>
           <cell r="AY5">
-            <v>-1.1051623325475934</v>
+            <v>-5.0064980472733112</v>
           </cell>
           <cell r="AZ5">
-            <v>-1.0966302471387412</v>
+            <v>-5.0852468488815639</v>
           </cell>
           <cell r="BA5">
-            <v>-1.0870101164449975</v>
+            <v>-5.1637059738566133</v>
           </cell>
           <cell r="BB5">
-            <v>-1.0680057134171306</v>
+            <v>-5.2500419439234447</v>
           </cell>
           <cell r="BC5">
-            <v>-1.060643959087848</v>
+            <v>-5.3254923794368807</v>
           </cell>
           <cell r="BD5">
-            <v>-1.05568150858667</v>
+            <v>-5.397441557757543</v>
           </cell>
           <cell r="BE5">
-            <v>-1.0508163034356865</v>
+            <v>-5.468206895285399</v>
           </cell>
           <cell r="BF5">
-            <v>-1.0449263794827357</v>
+            <v>-5.538953308007299</v>
           </cell>
           <cell r="BG5">
-            <v>-1.0350781535410358</v>
+            <v>-5.6100666583201564</v>
           </cell>
           <cell r="BH5">
-            <v>-1.0239183935763507</v>
+            <v>-5.6811461839669679</v>
           </cell>
           <cell r="BI5">
-            <v>-1.0116250753056444</v>
+            <v>-5.7521787639958966</v>
           </cell>
           <cell r="BJ5">
-            <v>-0.99847212863372059</v>
+            <v>-5.8230693764018344</v>
           </cell>
           <cell r="BK5">
-            <v>-0.98467917066891175</v>
+            <v>-5.8937551804897019</v>
           </cell>
           <cell r="BL5">
-            <v>-0.97007667068378378</v>
+            <v>-5.9627310400813149</v>
           </cell>
           <cell r="BM5">
-            <v>-0.95496489217563596</v>
+            <v>-6.0312211491092116</v>
           </cell>
           <cell r="BN5">
-            <v>-0.93936110914166759</v>
+            <v>-6.0993719673605673</v>
           </cell>
           <cell r="BO5">
-            <v>-0.92326116455754281</v>
+            <v>-6.1673530177726921</v>
           </cell>
           <cell r="BP5">
-            <v>-0.90665351933153504</v>
+            <v>-6.2352915712644119</v>
           </cell>
           <cell r="BQ5">
-            <v>-0.88775550044941642</v>
+            <v>-6.2985615324749666</v>
           </cell>
           <cell r="BR5">
-            <v>-0.86852547861959728</v>
+            <v>-6.3604577669279738</v>
           </cell>
           <cell r="BS5">
-            <v>-0.84888739793921308</v>
+            <v>-6.4213119370468359</v>
           </cell>
           <cell r="BT5">
-            <v>-0.82883728857620076</v>
+            <v>-6.4814497093279027</v>
           </cell>
           <cell r="BU5">
-            <v>-0.80839951654047004</v>
+            <v>-6.5411000815981835</v>
           </cell>
           <cell r="BV5">
-            <v>-0.78798787214297006</v>
+            <v>-6.597973463650475</v>
           </cell>
           <cell r="BW5">
-            <v>-0.7673256486760982</v>
+            <v>-6.6540575869920682</v>
           </cell>
           <cell r="BX5">
-            <v>-0.74642452707111007</v>
+            <v>-6.7095267408472932</v>
           </cell>
           <cell r="BY5">
-            <v>-0.72528794941011387</v>
+            <v>-6.7645730315837538</v>
           </cell>
           <cell r="BZ5">
-            <v>-0.70391821298150248</v>
+            <v>-6.8193461873122807</v>
           </cell>
           <cell r="CA5">
-            <v>-0.68132849998288059</v>
+            <v>-6.8700194906914147</v>
           </cell>
           <cell r="CB5">
-            <v>-0.65872022851274359</v>
+            <v>-6.9194266938419453</v>
           </cell>
           <cell r="CC5">
-            <v>-0.63600672294508165</v>
+            <v>-6.9678909725079947</v>
           </cell>
           <cell r="CD5">
-            <v>-0.61315682225527857</v>
+            <v>-7.0157234307819056</v>
           </cell>
           <cell r="CE5">
-            <v>-0.59016393322215421</v>
+            <v>-7.063148609647496</v>
           </cell>
           <cell r="CF5">
-            <v>-0.56801025030791541</v>
+            <v>-7.109622597534071</v>
           </cell>
           <cell r="CG5">
-            <v>-0.54588587020560908</v>
+            <v>-7.1558280095632254</v>
           </cell>
           <cell r="CH5">
-            <v>-0.53146903557963476</v>
+            <v>-7.1946536881305363</v>
           </cell>
           <cell r="CI5">
-            <v>-0.50280363543084849</v>
+            <v>-7.2466119899013197</v>
           </cell>
           <cell r="CJ5">
-            <v>-0.9305997798967458</v>
+            <v>-6.8712948072433004</v>
           </cell>
         </row>
       </sheetData>
@@ -4300,319 +4283,319 @@
       </c>
       <c r="I2" s="2">
         <f>[1]Données!J5</f>
-        <v>-0.19694161232846064</v>
+        <v>0.19161550315185405</v>
       </c>
       <c r="J2" s="2">
         <f>[1]Données!K5</f>
-        <v>-0.32910460472266312</v>
+        <v>0.31789887951911844</v>
       </c>
       <c r="K2" s="2">
         <f>[1]Données!L5</f>
-        <v>-8.0637713317255333E-2</v>
+        <v>6.7015030786099494E-2</v>
       </c>
       <c r="L2" s="2">
         <f>[1]Données!M5</f>
-        <v>0.20258876617191834</v>
+        <v>-0.21728167797012699</v>
       </c>
       <c r="M2" s="2">
         <f>[1]Données!N5</f>
-        <v>0.45424694424371914</v>
+        <v>-0.46886133701437016</v>
       </c>
       <c r="N2" s="2">
         <f>[1]Données!O5</f>
-        <v>0.6611727771178133</v>
+        <v>-0.67638884472317473</v>
       </c>
       <c r="O2" s="2">
         <f>[1]Données!P5</f>
-        <v>0.83719057505624583</v>
+        <v>-0.85375889954031337</v>
       </c>
       <c r="P2" s="2">
         <f>[1]Données!Q5</f>
-        <v>1.0028947161887292</v>
+        <v>-1.0207112465597246</v>
       </c>
       <c r="Q2" s="2">
         <f>[1]Données!R5</f>
-        <v>1.1571750805414949</v>
+        <v>-1.1759379933896641</v>
       </c>
       <c r="R2" s="2">
         <f>[1]Données!S5</f>
-        <v>1.2887400597361598</v>
+        <v>-1.307531973432452</v>
       </c>
       <c r="S2" s="2">
         <f>[1]Données!T5</f>
-        <v>1.3742398781701581</v>
+        <v>-1.3941416492964653</v>
       </c>
       <c r="T2" s="2">
         <f>[1]Données!U5</f>
-        <v>1.4290171313425803</v>
+        <v>-1.4508647654808193</v>
       </c>
       <c r="U2" s="2">
         <f>[1]Données!V5</f>
-        <v>1.4675920150303501</v>
+        <v>-1.4919916852337844</v>
       </c>
       <c r="V2" s="2">
         <f>[1]Données!W5</f>
-        <v>1.4991113762324426</v>
+        <v>-1.5264967867797408</v>
       </c>
       <c r="W2" s="2">
         <f>[1]Données!X5</f>
-        <v>1.5278210019538108</v>
+        <v>-1.5576296940993828</v>
       </c>
       <c r="X2" s="2">
         <f>[1]Données!Y5</f>
-        <v>1.5537649183268609</v>
+        <v>-1.5861667841999827</v>
       </c>
       <c r="Y2" s="2">
         <f>[1]Données!Z5</f>
-        <v>1.5768060907918269</v>
+        <v>-1.6118588854758364</v>
       </c>
       <c r="Z2" s="2">
         <f>[1]Données!AA5</f>
-        <v>1.5965658939140592</v>
+        <v>-1.6342925349397075</v>
       </c>
       <c r="AA2" s="2">
         <f>[1]Données!AB5</f>
-        <v>1.6125052003735707</v>
+        <v>-1.6529130346936594</v>
       </c>
       <c r="AB2" s="2">
         <f>[1]Données!AC5</f>
-        <v>1.6238872985003372</v>
+        <v>-1.6664774336045296</v>
       </c>
       <c r="AC2" s="2">
         <f>[1]Données!AD5</f>
-        <v>1.6292175777404383</v>
+        <v>-1.6738659693794067</v>
       </c>
       <c r="AD2" s="2">
         <f>[1]Données!AE5</f>
-        <v>1.6302196584468298</v>
+        <v>-1.6767182125922653</v>
       </c>
       <c r="AE2" s="2">
         <f>[1]Données!AF5</f>
-        <v>1.6294193971467585</v>
+        <v>-1.677493043235545</v>
       </c>
       <c r="AF2" s="2">
         <f>[1]Données!AG5</f>
-        <v>1.628626915129705</v>
+        <v>-1.6779763018033189</v>
       </c>
       <c r="AG2" s="2">
         <f>[1]Données!AH5</f>
-        <v>1.6291172996173886</v>
+        <v>-1.6790908599914611</v>
       </c>
       <c r="AH2" s="2">
         <f>[1]Données!AI5</f>
-        <v>1.6304594714892096</v>
+        <v>-1.6807531170653367</v>
       </c>
       <c r="AI2" s="2">
         <f>[1]Données!AJ5</f>
-        <v>1.6346407218347014</v>
+        <v>-1.6849090679153078</v>
       </c>
       <c r="AJ2" s="2">
         <f>[1]Données!AK5</f>
-        <v>1.6454229613436233</v>
+        <v>-1.6952498621138901</v>
       </c>
       <c r="AK2" s="2">
         <f>[1]Données!AL5</f>
-        <v>1.6696180039645014</v>
+        <v>-1.7184393048263136</v>
       </c>
       <c r="AL2" s="2">
         <f>[1]Données!AM5</f>
-        <v>1.6889441686418261</v>
+        <v>-1.7362029288578218</v>
       </c>
       <c r="AM2" s="2">
         <f>[1]Données!AN5</f>
-        <v>1.7078428405991497</v>
+        <v>-1.7534246166071354</v>
       </c>
       <c r="AN2" s="2">
         <f>[1]Données!AO5</f>
-        <v>1.7236337283863978</v>
+        <v>-1.7675856069250262</v>
       </c>
       <c r="AO2" s="2">
         <f>[1]Données!AP5</f>
-        <v>1.7349248053407429</v>
+        <v>-1.7775623333425861</v>
       </c>
       <c r="AP2" s="2">
         <f>[1]Données!AQ5</f>
-        <v>1.7411540936693504</v>
+        <v>-1.7830030310172607</v>
       </c>
       <c r="AQ2" s="2">
         <f>[1]Données!AR5</f>
-        <v>1.7428896953826323</v>
+        <v>-1.7843857765953541</v>
       </c>
       <c r="AR2" s="2">
         <f>[1]Données!AS5</f>
-        <v>1.7398540828657216</v>
+        <v>-1.7814809968153322</v>
       </c>
       <c r="AS2" s="2">
         <f>[1]Données!AT5</f>
-        <v>1.7329147309208093</v>
+        <v>-1.7750230330517369</v>
       </c>
       <c r="AT2" s="2">
         <f>[1]Données!AU5</f>
-        <v>1.7230862359691956</v>
+        <v>-1.7659091624286583</v>
       </c>
       <c r="AU2" s="2">
         <f>[1]Données!AV5</f>
-        <v>1.7113712076963328</v>
+        <v>-1.7550687062752313</v>
       </c>
       <c r="AV2" s="2">
         <f>[1]Données!AW5</f>
-        <v>1.6991510984826208</v>
+        <v>-1.7437581416538506</v>
       </c>
       <c r="AW2" s="2">
         <f>[1]Données!AX5</f>
-        <v>1.6866072217296857</v>
+        <v>-1.7322399317636572</v>
       </c>
       <c r="AX2" s="2">
         <f>[1]Données!AY5</f>
-        <v>1.6742464005973456</v>
+        <v>-1.7209837178788767</v>
       </c>
       <c r="AY2" s="2">
         <f>[1]Données!AZ5</f>
-        <v>1.6623965816549013</v>
+        <v>-1.7102969143967806</v>
       </c>
       <c r="AZ2" s="2">
         <f>[1]Données!BA5</f>
-        <v>1.6512509308354018</v>
+        <v>-1.7003514750675741</v>
       </c>
       <c r="BA2" s="2">
         <f>[1]Données!BB5</f>
-        <v>1.6524822554548013</v>
+        <v>-1.7041717945534995</v>
       </c>
       <c r="BB2" s="2">
         <f>[1]Données!BC5</f>
-        <v>1.6450248394999534</v>
+        <v>-1.6968611913178111</v>
       </c>
       <c r="BC2" s="2">
         <f>[1]Données!BD5</f>
-        <v>1.6348458928615806</v>
+        <v>-1.6874204618492761</v>
       </c>
       <c r="BD2" s="2">
         <f>[1]Données!BE5</f>
-        <v>1.6242837620730421</v>
+        <v>-1.6779987060296264</v>
       </c>
       <c r="BE2" s="2">
         <f>[1]Données!BF5</f>
-        <v>1.6146046053609364</v>
+        <v>-1.6695997980133215</v>
       </c>
       <c r="BF2" s="2">
         <f>[1]Données!BG5</f>
-        <v>1.6075645605232003</v>
+        <v>-1.6637538837163346</v>
       </c>
       <c r="BG2" s="2">
         <f>[1]Données!BH5</f>
-        <v>1.6016081837933793</v>
+        <v>-1.6589740264339237</v>
       </c>
       <c r="BH2" s="2">
         <f>[1]Données!BI5</f>
-        <v>1.5966635898912562</v>
+        <v>-1.6551568536300354</v>
       </c>
       <c r="BI2" s="2">
         <f>[1]Données!BJ5</f>
-        <v>1.5925545300034649</v>
+        <v>-1.6521136575608164</v>
       </c>
       <c r="BJ2" s="2">
         <f>[1]Données!BK5</f>
-        <v>1.5891372665503889</v>
+        <v>-1.6496961346720851</v>
       </c>
       <c r="BK2" s="2">
         <f>[1]Données!BL5</f>
-        <v>1.5863392639233309</v>
+        <v>-1.647812183467412</v>
       </c>
       <c r="BL2" s="2">
         <f>[1]Données!BM5</f>
-        <v>1.5841510083471011</v>
+        <v>-1.6464745156678506</v>
       </c>
       <c r="BM2" s="2">
         <f>[1]Données!BN5</f>
-        <v>1.5826012084538377</v>
+        <v>-1.6457143828054077</v>
       </c>
       <c r="BN2" s="2">
         <f>[1]Données!BO5</f>
-        <v>1.5817315368870766</v>
+        <v>-1.6455781760776222</v>
       </c>
       <c r="BO2" s="2">
         <f>[1]Données!BP5</f>
-        <v>1.5815791282935976</v>
+        <v>-1.6461074372563056</v>
       </c>
       <c r="BP2" s="2">
         <f>[1]Données!BQ5</f>
-        <v>1.5833859626567248</v>
+        <v>-1.6484945595247713</v>
       </c>
       <c r="BQ2" s="2">
         <f>[1]Données!BR5</f>
-        <v>1.585692472380229</v>
+        <v>-1.6513493411040914</v>
       </c>
       <c r="BR2" s="2">
         <f>[1]Données!BS5</f>
-        <v>1.5886108369449925</v>
+        <v>-1.6547799298626154</v>
       </c>
       <c r="BS2" s="2">
         <f>[1]Données!BT5</f>
-        <v>1.5921782276750784</v>
+        <v>-1.6588215817661012</v>
       </c>
       <c r="BT2" s="2">
         <f>[1]Données!BU5</f>
-        <v>1.5963952313138297</v>
+        <v>-1.663474348417826</v>
       </c>
       <c r="BU2" s="2">
         <f>[1]Données!BV5</f>
-        <v>1.6012455941350368</v>
+        <v>-1.668749189340446</v>
       </c>
       <c r="BV2" s="2">
         <f>[1]Données!BW5</f>
-        <v>1.6067094578869234</v>
+        <v>-1.6745957993986593</v>
       </c>
       <c r="BW2" s="2">
         <f>[1]Données!BX5</f>
-        <v>1.6127694246065971</v>
+        <v>-1.6809976191283882</v>
       </c>
       <c r="BX2" s="2">
         <f>[1]Données!BY5</f>
-        <v>1.6194122415741141</v>
+        <v>-1.6879396819433956</v>
       </c>
       <c r="BY2" s="2">
         <f>[1]Données!BZ5</f>
-        <v>1.6266274009712811</v>
+        <v>-1.6954091313694963</v>
       </c>
       <c r="BZ2" s="2">
         <f>[1]Données!CA5</f>
-        <v>1.6354020493762667</v>
+        <v>-1.7043809443399893</v>
       </c>
       <c r="CA2" s="2">
         <f>[1]Données!CB5</f>
-        <v>1.6445477994649904</v>
+        <v>-1.7136818328981618</v>
       </c>
       <c r="CB2" s="2">
         <f>[1]Données!CC5</f>
-        <v>1.6541465898829877</v>
+        <v>-1.7233900154516202</v>
       </c>
       <c r="CC2" s="2">
         <f>[1]Données!CD5</f>
-        <v>1.6642258451554426</v>
+        <v>-1.733529893763619</v>
       </c>
       <c r="CD2" s="2">
         <f>[1]Données!CE5</f>
-        <v>1.6747892448942148</v>
+        <v>-1.7441041249341871</v>
       </c>
       <c r="CE2" s="2">
         <f>[1]Données!CF5</f>
-        <v>1.6858325017146347</v>
+        <v>-1.7551879809414861</v>
       </c>
       <c r="CF2" s="2">
         <f>[1]Données!CG5</f>
-        <v>1.6973521339859632</v>
+        <v>-1.7666911636200933</v>
       </c>
       <c r="CG2" s="2">
         <f>[1]Données!CH5</f>
-        <v>1.7093489455747068</v>
+        <v>-1.7709894968797713</v>
       </c>
       <c r="CH2" s="2">
         <f>[1]Données!CI5</f>
-        <v>1.7218275243293002</v>
+        <v>-1.7897149040786542</v>
       </c>
       <c r="CI2" s="2">
         <f>[1]Données!CJ5</f>
-        <v>1.7347940252342653</v>
+        <v>-1.3563380790536539</v>
       </c>
     </row>
     <row r="3" spans="1:87" x14ac:dyDescent="0.3">
@@ -4625,343 +4608,343 @@
       </c>
       <c r="C3" s="2">
         <f>[2]Données!D5</f>
-        <v>-0.11989295890919571</v>
+        <v>9.1492751157495888E-4</v>
       </c>
       <c r="D3" s="2">
         <f>[2]Données!E5</f>
-        <v>-0.2564913650720313</v>
+        <v>1.9380107544986203E-3</v>
       </c>
       <c r="E3" s="2">
         <f>[2]Données!F5</f>
-        <v>-0.40548218803949654</v>
+        <v>3.0370170623905679E-3</v>
       </c>
       <c r="F3" s="2">
         <f>[2]Données!G5</f>
-        <v>-0.5625868560056535</v>
+        <v>4.1803820710395456E-3</v>
       </c>
       <c r="G3" s="2">
         <f>[2]Données!H5</f>
-        <v>-0.72368591578868546</v>
+        <v>5.3381698501331343E-3</v>
       </c>
       <c r="H3" s="2">
         <f>[2]Données!I5</f>
-        <v>-0.89397615754910342</v>
+        <v>1.3157759753057441E-2</v>
       </c>
       <c r="I3" s="2">
         <f>[2]Données!J5</f>
-        <v>-1.2536848339774753</v>
+        <v>0.21348505364844339</v>
       </c>
       <c r="J3" s="2">
         <f>[2]Données!K5</f>
-        <v>-1.5465477388130644</v>
+        <v>0.34910430938315251</v>
       </c>
       <c r="K3" s="2">
         <f>[2]Données!L5</f>
-        <v>-1.4663796850371669</v>
+        <v>0.10772874383697673</v>
       </c>
       <c r="L3" s="2">
         <f>[2]Données!M5</f>
-        <v>-1.3499516421471625</v>
+        <v>-0.16705601577994278</v>
       </c>
       <c r="M3" s="2">
         <f>[2]Données!N5</f>
-        <v>-1.2432807826123216</v>
+        <v>-0.43465890355091075</v>
       </c>
       <c r="N3" s="2">
         <f>[2]Données!O5</f>
-        <v>-1.1740907821493396</v>
+        <v>-0.66159570791660682</v>
       </c>
       <c r="O3" s="2">
         <f>[2]Données!P5</f>
-        <v>-1.1293824838973121</v>
+        <v>-0.86101032056353777</v>
       </c>
       <c r="P3" s="2">
         <f>[2]Données!Q5</f>
-        <v>-1.0904536525910724</v>
+        <v>-1.0515687464137558</v>
       </c>
       <c r="Q3" s="2">
         <f>[2]Données!R5</f>
-        <v>-1.0594058486379065</v>
+        <v>-1.2311097309259722</v>
       </c>
       <c r="R3" s="2">
         <f>[2]Données!S5</f>
-        <v>-1.0183572616020098</v>
+        <v>-1.4228025754553508</v>
       </c>
       <c r="S3" s="2">
         <f>[2]Données!T5</f>
-        <v>-1.0154352355562501</v>
+        <v>-1.5742008267198959</v>
       </c>
       <c r="T3" s="2">
         <f>[2]Données!U5</f>
-        <v>-1.037065636868395</v>
+        <v>-1.6992195584478065</v>
       </c>
       <c r="U3" s="2">
         <f>[2]Données!V5</f>
-        <v>-1.0707668042763685</v>
+        <v>-1.8105357584278448</v>
       </c>
       <c r="V3" s="2">
         <f>[2]Données!W5</f>
-        <v>-1.1090001761417945</v>
+        <v>-1.9158446646005745</v>
       </c>
       <c r="W3" s="2">
         <f>[2]Données!X5</f>
-        <v>-1.1233479395032275</v>
+        <v>-2.0422926708964284</v>
       </c>
       <c r="X3" s="2">
         <f>[2]Données!Y5</f>
-        <v>-1.1356564507584044</v>
+        <v>-2.1692700651057328</v>
       </c>
       <c r="Y3" s="2">
         <f>[2]Données!Z5</f>
-        <v>-1.147334199538641</v>
+        <v>-2.2955382898167564</v>
       </c>
       <c r="Z3" s="2">
         <f>[2]Données!AA5</f>
-        <v>-1.160195655963403</v>
+        <v>-2.4194852035804293</v>
       </c>
       <c r="AA3" s="2">
         <f>[2]Données!AB5</f>
-        <v>-1.1758545383770969</v>
+        <v>-2.5396476528848577</v>
       </c>
       <c r="AB3" s="2">
         <f>[2]Données!AC5</f>
-        <v>-1.1850823533255617</v>
+        <v>-2.661324458444736</v>
       </c>
       <c r="AC3" s="2">
         <f>[2]Données!AD5</f>
-        <v>-1.1986687041575239</v>
+        <v>-2.7771446690231461</v>
       </c>
       <c r="AD3" s="2">
         <f>[2]Données!AE5</f>
-        <v>-1.2155170209160682</v>
+        <v>-2.8883528079100107</v>
       </c>
       <c r="AE3" s="2">
         <f>[2]Données!AF5</f>
-        <v>-1.2337160576910144</v>
+        <v>-2.9969917621188835</v>
       </c>
       <c r="AF3" s="2">
         <f>[2]Données!AG5</f>
-        <v>-1.2518586150598643</v>
+        <v>-3.1045562489061651</v>
       </c>
       <c r="AG3" s="2">
         <f>[2]Données!AH5</f>
-        <v>-1.2614657210244462</v>
+        <v>-3.2169190300692652</v>
       </c>
       <c r="AH3" s="2">
         <f>[2]Données!AI5</f>
-        <v>-1.2691587127149351</v>
+        <v>-3.3296402639445777</v>
       </c>
       <c r="AI3" s="2">
         <f>[2]Données!AJ5</f>
-        <v>-1.2732600629612678</v>
+        <v>-3.4444508403099983</v>
       </c>
       <c r="AJ3" s="2">
         <f>[2]Données!AK5</f>
-        <v>-1.2703781735087571</v>
+        <v>-3.5647533183807201</v>
       </c>
       <c r="AK3" s="2">
         <f>[2]Données!AL5</f>
-        <v>-1.2540210547578035</v>
+        <v>-3.6969161347232715</v>
       </c>
       <c r="AL3" s="2">
         <f>[2]Données!AM5</f>
-        <v>-1.2342552264018036</v>
+        <v>-3.8217313853343149</v>
       </c>
       <c r="AM3" s="2">
         <f>[2]Données!AN5</f>
-        <v>-1.2131238461617344</v>
+        <v>-3.9448919323131437</v>
       </c>
       <c r="AN3" s="2">
         <f>[2]Données!AO5</f>
-        <v>-1.193489392035052</v>
+        <v>-4.0639667698810111</v>
       </c>
       <c r="AO3" s="2">
         <f>[2]Données!AP5</f>
-        <v>-1.1768444016053481</v>
+        <v>-4.1779892250678348</v>
       </c>
       <c r="AP3" s="2">
         <f>[2]Données!AQ5</f>
-        <v>-1.1637977662731003</v>
+        <v>-4.2867387241266375</v>
       </c>
       <c r="AQ3" s="2">
         <f>[2]Données!AR5</f>
-        <v>-1.1511488370674505</v>
+        <v>-4.390502402670271</v>
       </c>
       <c r="AR3" s="2">
         <f>[2]Données!AS5</f>
-        <v>-1.1416185393326339</v>
+        <v>-4.4892722927368904</v>
       </c>
       <c r="AS3" s="2">
         <f>[2]Données!AT5</f>
-        <v>-1.1346413446308934</v>
+        <v>-4.5838049366044631</v>
       </c>
       <c r="AT3" s="2">
         <f>[2]Données!AU5</f>
-        <v>-1.1294875920329184</v>
+        <v>-4.6750075756943232</v>
       </c>
       <c r="AU3" s="2">
         <f>[2]Données!AV5</f>
-        <v>-1.1253663585153451</v>
+        <v>-4.7638116158136619</v>
       </c>
       <c r="AV3" s="2">
         <f>[2]Données!AW5</f>
-        <v>-1.1192877374659904</v>
+        <v>-4.846398105559679</v>
       </c>
       <c r="AW3" s="2">
         <f>[2]Données!AX5</f>
-        <v>-1.1126615212282309</v>
+        <v>-4.9270733084887386</v>
       </c>
       <c r="AX3" s="2">
         <f>[2]Données!AY5</f>
-        <v>-1.1051623325475934</v>
+        <v>-5.0064980472733112</v>
       </c>
       <c r="AY3" s="2">
         <f>[2]Données!AZ5</f>
-        <v>-1.0966302471387412</v>
+        <v>-5.0852468488815639</v>
       </c>
       <c r="AZ3" s="2">
         <f>[2]Données!BA5</f>
-        <v>-1.0870101164449975</v>
+        <v>-5.1637059738566133</v>
       </c>
       <c r="BA3" s="2">
         <f>[2]Données!BB5</f>
-        <v>-1.0680057134171306</v>
+        <v>-5.2500419439234447</v>
       </c>
       <c r="BB3" s="2">
         <f>[2]Données!BC5</f>
-        <v>-1.060643959087848</v>
+        <v>-5.3254923794368807</v>
       </c>
       <c r="BC3" s="2">
         <f>[2]Données!BD5</f>
-        <v>-1.05568150858667</v>
+        <v>-5.397441557757543</v>
       </c>
       <c r="BD3" s="2">
         <f>[2]Données!BE5</f>
-        <v>-1.0508163034356865</v>
+        <v>-5.468206895285399</v>
       </c>
       <c r="BE3" s="2">
         <f>[2]Données!BF5</f>
-        <v>-1.0449263794827357</v>
+        <v>-5.538953308007299</v>
       </c>
       <c r="BF3" s="2">
         <f>[2]Données!BG5</f>
-        <v>-1.0350781535410358</v>
+        <v>-5.6100666583201564</v>
       </c>
       <c r="BG3" s="2">
         <f>[2]Données!BH5</f>
-        <v>-1.0239183935763507</v>
+        <v>-5.6811461839669679</v>
       </c>
       <c r="BH3" s="2">
         <f>[2]Données!BI5</f>
-        <v>-1.0116250753056444</v>
+        <v>-5.7521787639958966</v>
       </c>
       <c r="BI3" s="2">
         <f>[2]Données!BJ5</f>
-        <v>-0.99847212863372059</v>
+        <v>-5.8230693764018344</v>
       </c>
       <c r="BJ3" s="2">
         <f>[2]Données!BK5</f>
-        <v>-0.98467917066891175</v>
+        <v>-5.8937551804897019</v>
       </c>
       <c r="BK3" s="2">
         <f>[2]Données!BL5</f>
-        <v>-0.97007667068378378</v>
+        <v>-5.9627310400813149</v>
       </c>
       <c r="BL3" s="2">
         <f>[2]Données!BM5</f>
-        <v>-0.95496489217563596</v>
+        <v>-6.0312211491092116</v>
       </c>
       <c r="BM3" s="2">
         <f>[2]Données!BN5</f>
-        <v>-0.93936110914166759</v>
+        <v>-6.0993719673605673</v>
       </c>
       <c r="BN3" s="2">
         <f>[2]Données!BO5</f>
-        <v>-0.92326116455754281</v>
+        <v>-6.1673530177726921</v>
       </c>
       <c r="BO3" s="2">
         <f>[2]Données!BP5</f>
-        <v>-0.90665351933153504</v>
+        <v>-6.2352915712644119</v>
       </c>
       <c r="BP3" s="2">
         <f>[2]Données!BQ5</f>
-        <v>-0.88775550044941642</v>
+        <v>-6.2985615324749666</v>
       </c>
       <c r="BQ3" s="2">
         <f>[2]Données!BR5</f>
-        <v>-0.86852547861959728</v>
+        <v>-6.3604577669279738</v>
       </c>
       <c r="BR3" s="2">
         <f>[2]Données!BS5</f>
-        <v>-0.84888739793921308</v>
+        <v>-6.4213119370468359</v>
       </c>
       <c r="BS3" s="2">
         <f>[2]Données!BT5</f>
-        <v>-0.82883728857620076</v>
+        <v>-6.4814497093279027</v>
       </c>
       <c r="BT3" s="2">
         <f>[2]Données!BU5</f>
-        <v>-0.80839951654047004</v>
+        <v>-6.5411000815981835</v>
       </c>
       <c r="BU3" s="2">
         <f>[2]Données!BV5</f>
-        <v>-0.78798787214297006</v>
+        <v>-6.597973463650475</v>
       </c>
       <c r="BV3" s="2">
         <f>[2]Données!BW5</f>
-        <v>-0.7673256486760982</v>
+        <v>-6.6540575869920682</v>
       </c>
       <c r="BW3" s="2">
         <f>[2]Données!BX5</f>
-        <v>-0.74642452707111007</v>
+        <v>-6.7095267408472932</v>
       </c>
       <c r="BX3" s="2">
         <f>[2]Données!BY5</f>
-        <v>-0.72528794941011387</v>
+        <v>-6.7645730315837538</v>
       </c>
       <c r="BY3" s="2">
         <f>[2]Données!BZ5</f>
-        <v>-0.70391821298150248</v>
+        <v>-6.8193461873122807</v>
       </c>
       <c r="BZ3" s="2">
         <f>[2]Données!CA5</f>
-        <v>-0.68132849998288059</v>
+        <v>-6.8700194906914147</v>
       </c>
       <c r="CA3" s="2">
         <f>[2]Données!CB5</f>
-        <v>-0.65872022851274359</v>
+        <v>-6.9194266938419453</v>
       </c>
       <c r="CB3" s="2">
         <f>[2]Données!CC5</f>
-        <v>-0.63600672294508165</v>
+        <v>-6.9678909725079947</v>
       </c>
       <c r="CC3" s="2">
         <f>[2]Données!CD5</f>
-        <v>-0.61315682225527857</v>
+        <v>-7.0157234307819056</v>
       </c>
       <c r="CD3" s="2">
         <f>[2]Données!CE5</f>
-        <v>-0.59016393322215421</v>
+        <v>-7.063148609647496</v>
       </c>
       <c r="CE3" s="2">
         <f>[2]Données!CF5</f>
-        <v>-0.56801025030791541</v>
+        <v>-7.109622597534071</v>
       </c>
       <c r="CF3" s="2">
         <f>[2]Données!CG5</f>
-        <v>-0.54588587020560908</v>
+        <v>-7.1558280095632254</v>
       </c>
       <c r="CG3" s="2">
         <f>[2]Données!CH5</f>
-        <v>-0.53146903557963476</v>
+        <v>-7.1946536881305363</v>
       </c>
       <c r="CH3" s="2">
         <f>[2]Données!CI5</f>
-        <v>-0.50280363543084849</v>
+        <v>-7.2466119899013197</v>
       </c>
       <c r="CI3" s="2">
         <f>[2]Données!CJ5</f>
-        <v>-0.9305997798967458</v>
+        <v>-6.8712948072433004</v>
       </c>
     </row>
     <row r="5" spans="1:87" x14ac:dyDescent="0.3">
@@ -5258,319 +5241,319 @@
       </c>
       <c r="I6" s="2">
         <f t="shared" si="0"/>
-        <v>-0.19694161232846064</v>
+        <v>0.19161550315185405</v>
       </c>
       <c r="J6" s="2">
         <f t="shared" si="0"/>
-        <v>-0.32910460472266312</v>
+        <v>0.31789887951911844</v>
       </c>
       <c r="K6" s="2">
         <f t="shared" si="0"/>
-        <v>-8.0637713317255333E-2</v>
+        <v>6.7015030786099494E-2</v>
       </c>
       <c r="L6" s="2">
         <f t="shared" si="0"/>
-        <v>0.20258876617191834</v>
+        <v>-0.21728167797012699</v>
       </c>
       <c r="M6" s="2">
         <f t="shared" si="0"/>
-        <v>0.45424694424371914</v>
+        <v>-0.46886133701437016</v>
       </c>
       <c r="N6" s="2">
         <f t="shared" si="0"/>
-        <v>0.6611727771178133</v>
+        <v>-0.67638884472317473</v>
       </c>
       <c r="O6" s="2">
         <f t="shared" si="0"/>
-        <v>0.83719057505624583</v>
+        <v>-0.85375889954031337</v>
       </c>
       <c r="P6" s="2">
         <f t="shared" si="0"/>
-        <v>1.0028947161887292</v>
+        <v>-1.0207112465597246</v>
       </c>
       <c r="Q6" s="2">
         <f t="shared" si="0"/>
-        <v>1.1571750805414949</v>
+        <v>-1.1759379933896641</v>
       </c>
       <c r="R6" s="2">
         <f t="shared" si="0"/>
-        <v>1.2887400597361598</v>
+        <v>-1.307531973432452</v>
       </c>
       <c r="S6" s="2">
         <f t="shared" si="0"/>
-        <v>1.3742398781701581</v>
+        <v>-1.3941416492964653</v>
       </c>
       <c r="T6" s="2">
         <f t="shared" si="0"/>
-        <v>1.4290171313425803</v>
+        <v>-1.4508647654808193</v>
       </c>
       <c r="U6" s="2">
         <f t="shared" si="0"/>
-        <v>1.4675920150303501</v>
+        <v>-1.4919916852337844</v>
       </c>
       <c r="V6" s="2">
         <f t="shared" si="0"/>
-        <v>1.4991113762324426</v>
+        <v>-1.5264967867797408</v>
       </c>
       <c r="W6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5278210019538108</v>
+        <v>-1.5576296940993828</v>
       </c>
       <c r="X6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5537649183268609</v>
+        <v>-1.5861667841999827</v>
       </c>
       <c r="Y6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5768060907918269</v>
+        <v>-1.6118588854758364</v>
       </c>
       <c r="Z6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5965658939140592</v>
+        <v>-1.6342925349397075</v>
       </c>
       <c r="AA6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6125052003735707</v>
+        <v>-1.6529130346936594</v>
       </c>
       <c r="AB6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6238872985003372</v>
+        <v>-1.6664774336045296</v>
       </c>
       <c r="AC6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6292175777404383</v>
+        <v>-1.6738659693794067</v>
       </c>
       <c r="AD6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6302196584468298</v>
+        <v>-1.6767182125922653</v>
       </c>
       <c r="AE6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6294193971467585</v>
+        <v>-1.677493043235545</v>
       </c>
       <c r="AF6" s="2">
         <f t="shared" si="0"/>
-        <v>1.628626915129705</v>
+        <v>-1.6779763018033189</v>
       </c>
       <c r="AG6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6291172996173886</v>
+        <v>-1.6790908599914611</v>
       </c>
       <c r="AH6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6304594714892096</v>
+        <v>-1.6807531170653367</v>
       </c>
       <c r="AI6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6346407218347014</v>
+        <v>-1.6849090679153078</v>
       </c>
       <c r="AJ6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6454229613436233</v>
+        <v>-1.6952498621138901</v>
       </c>
       <c r="AK6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6696180039645014</v>
+        <v>-1.7184393048263136</v>
       </c>
       <c r="AL6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6889441686418261</v>
+        <v>-1.7362029288578218</v>
       </c>
       <c r="AM6" s="2">
         <f t="shared" si="0"/>
-        <v>1.7078428405991497</v>
+        <v>-1.7534246166071354</v>
       </c>
       <c r="AN6" s="2">
         <f t="shared" si="0"/>
-        <v>1.7236337283863978</v>
+        <v>-1.7675856069250262</v>
       </c>
       <c r="AO6" s="2">
         <f t="shared" si="0"/>
-        <v>1.7349248053407429</v>
+        <v>-1.7775623333425861</v>
       </c>
       <c r="AP6" s="2">
         <f t="shared" si="0"/>
-        <v>1.7411540936693504</v>
+        <v>-1.7830030310172607</v>
       </c>
       <c r="AQ6" s="2">
         <f t="shared" si="0"/>
-        <v>1.7428896953826323</v>
+        <v>-1.7843857765953541</v>
       </c>
       <c r="AR6" s="2">
         <f t="shared" si="0"/>
-        <v>1.7398540828657216</v>
+        <v>-1.7814809968153322</v>
       </c>
       <c r="AS6" s="2">
         <f t="shared" si="0"/>
-        <v>1.7329147309208093</v>
+        <v>-1.7750230330517369</v>
       </c>
       <c r="AT6" s="2">
         <f t="shared" si="0"/>
-        <v>1.7230862359691956</v>
+        <v>-1.7659091624286583</v>
       </c>
       <c r="AU6" s="2">
         <f t="shared" si="0"/>
-        <v>1.7113712076963328</v>
+        <v>-1.7550687062752313</v>
       </c>
       <c r="AV6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6991510984826208</v>
+        <v>-1.7437581416538506</v>
       </c>
       <c r="AW6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6866072217296857</v>
+        <v>-1.7322399317636572</v>
       </c>
       <c r="AX6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6742464005973456</v>
+        <v>-1.7209837178788767</v>
       </c>
       <c r="AY6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6623965816549013</v>
+        <v>-1.7102969143967806</v>
       </c>
       <c r="AZ6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6512509308354018</v>
+        <v>-1.7003514750675741</v>
       </c>
       <c r="BA6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6524822554548013</v>
+        <v>-1.7041717945534995</v>
       </c>
       <c r="BB6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6450248394999534</v>
+        <v>-1.6968611913178111</v>
       </c>
       <c r="BC6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6348458928615806</v>
+        <v>-1.6874204618492761</v>
       </c>
       <c r="BD6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6242837620730421</v>
+        <v>-1.6779987060296264</v>
       </c>
       <c r="BE6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6146046053609364</v>
+        <v>-1.6695997980133215</v>
       </c>
       <c r="BF6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6075645605232003</v>
+        <v>-1.6637538837163346</v>
       </c>
       <c r="BG6" s="2">
         <f t="shared" si="0"/>
-        <v>1.6016081837933793</v>
+        <v>-1.6589740264339237</v>
       </c>
       <c r="BH6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5966635898912562</v>
+        <v>-1.6551568536300354</v>
       </c>
       <c r="BI6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5925545300034649</v>
+        <v>-1.6521136575608164</v>
       </c>
       <c r="BJ6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5891372665503889</v>
+        <v>-1.6496961346720851</v>
       </c>
       <c r="BK6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5863392639233309</v>
+        <v>-1.647812183467412</v>
       </c>
       <c r="BL6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5841510083471011</v>
+        <v>-1.6464745156678506</v>
       </c>
       <c r="BM6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5826012084538377</v>
+        <v>-1.6457143828054077</v>
       </c>
       <c r="BN6" s="2">
         <f t="shared" si="0"/>
-        <v>1.5817315368870766</v>
+        <v>-1.6455781760776222</v>
       </c>
       <c r="BO6" s="2">
         <f t="shared" ref="BO6:CI6" si="1">BO2</f>
-        <v>1.5815791282935976</v>
+        <v>-1.6461074372563056</v>
       </c>
       <c r="BP6" s="2">
         <f t="shared" si="1"/>
-        <v>1.5833859626567248</v>
+        <v>-1.6484945595247713</v>
       </c>
       <c r="BQ6" s="2">
         <f t="shared" si="1"/>
-        <v>1.585692472380229</v>
+        <v>-1.6513493411040914</v>
       </c>
       <c r="BR6" s="2">
         <f t="shared" si="1"/>
-        <v>1.5886108369449925</v>
+        <v>-1.6547799298626154</v>
       </c>
       <c r="BS6" s="2">
         <f t="shared" si="1"/>
-        <v>1.5921782276750784</v>
+        <v>-1.6588215817661012</v>
       </c>
       <c r="BT6" s="2">
         <f t="shared" si="1"/>
-        <v>1.5963952313138297</v>
+        <v>-1.663474348417826</v>
       </c>
       <c r="BU6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6012455941350368</v>
+        <v>-1.668749189340446</v>
       </c>
       <c r="BV6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6067094578869234</v>
+        <v>-1.6745957993986593</v>
       </c>
       <c r="BW6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6127694246065971</v>
+        <v>-1.6809976191283882</v>
       </c>
       <c r="BX6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6194122415741141</v>
+        <v>-1.6879396819433956</v>
       </c>
       <c r="BY6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6266274009712811</v>
+        <v>-1.6954091313694963</v>
       </c>
       <c r="BZ6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6354020493762667</v>
+        <v>-1.7043809443399893</v>
       </c>
       <c r="CA6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6445477994649904</v>
+        <v>-1.7136818328981618</v>
       </c>
       <c r="CB6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6541465898829877</v>
+        <v>-1.7233900154516202</v>
       </c>
       <c r="CC6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6642258451554426</v>
+        <v>-1.733529893763619</v>
       </c>
       <c r="CD6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6747892448942148</v>
+        <v>-1.7441041249341871</v>
       </c>
       <c r="CE6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6858325017146347</v>
+        <v>-1.7551879809414861</v>
       </c>
       <c r="CF6" s="2">
         <f t="shared" si="1"/>
-        <v>1.6973521339859632</v>
+        <v>-1.7666911636200933</v>
       </c>
       <c r="CG6" s="2">
         <f t="shared" si="1"/>
-        <v>1.7093489455747068</v>
+        <v>-1.7709894968797713</v>
       </c>
       <c r="CH6" s="2">
         <f t="shared" si="1"/>
-        <v>1.7218275243293002</v>
+        <v>-1.7897149040786542</v>
       </c>
       <c r="CI6" s="2">
         <f t="shared" si="1"/>
-        <v>1.7347940252342653</v>
+        <v>-1.3563380790536539</v>
       </c>
     </row>
     <row r="7" spans="1:87" x14ac:dyDescent="0.3">
@@ -5583,343 +5566,343 @@
       </c>
       <c r="C7" s="2">
         <f t="shared" ref="C7:BN7" si="2">C3-C2</f>
-        <v>-0.11989295890919571</v>
+        <v>9.1492751157495888E-4</v>
       </c>
       <c r="D7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.2564913650720313</v>
+        <v>1.9380107544986203E-3</v>
       </c>
       <c r="E7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.40548218803949654</v>
+        <v>3.0370170623905679E-3</v>
       </c>
       <c r="F7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.5625868560056535</v>
+        <v>4.1803820710395456E-3</v>
       </c>
       <c r="G7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.72368591578868546</v>
+        <v>5.3381698501331343E-3</v>
       </c>
       <c r="H7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.89397615754910342</v>
+        <v>1.3157759753057441E-2</v>
       </c>
       <c r="I7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.0567432216490147</v>
+        <v>2.1869550496589341E-2</v>
       </c>
       <c r="J7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.2174431340904013</v>
+        <v>3.1205429864034073E-2</v>
       </c>
       <c r="K7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.3857419717199115</v>
+        <v>4.0713713050877232E-2</v>
       </c>
       <c r="L7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.5525404083190808</v>
+        <v>5.0225662190184206E-2</v>
       </c>
       <c r="M7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.6975277268560407</v>
+        <v>3.4202433463459414E-2</v>
       </c>
       <c r="N7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.8352635592671529</v>
+        <v>1.4793136806567908E-2</v>
       </c>
       <c r="O7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.9665730589535579</v>
+        <v>-7.2514210232244025E-3</v>
       </c>
       <c r="P7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.0933483687798016</v>
+        <v>-3.085749985403119E-2</v>
       </c>
       <c r="Q7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.2165809291794014</v>
+        <v>-5.5171737536308108E-2</v>
       </c>
       <c r="R7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.3070973213381696</v>
+        <v>-0.11527060202289885</v>
       </c>
       <c r="S7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.3896751137264083</v>
+        <v>-0.18005917742343058</v>
       </c>
       <c r="T7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.4660827682109754</v>
+        <v>-0.24835479296698715</v>
       </c>
       <c r="U7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.5383588193067186</v>
+        <v>-0.31854407319406031</v>
       </c>
       <c r="V7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6081115523742371</v>
+        <v>-0.38934787782083369</v>
       </c>
       <c r="W7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6511689414570383</v>
+        <v>-0.48466297679704562</v>
       </c>
       <c r="X7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6894213690852653</v>
+        <v>-0.58310328090575014</v>
       </c>
       <c r="Y7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7241402903304679</v>
+        <v>-0.68367940434092001</v>
       </c>
       <c r="Z7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7567615498774622</v>
+        <v>-0.78519266864072179</v>
       </c>
       <c r="AA7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7883597387506676</v>
+        <v>-0.88673461819119836</v>
       </c>
       <c r="AB7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8089696518258989</v>
+        <v>-0.99484702484020637</v>
       </c>
       <c r="AC7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8278862818979622</v>
+        <v>-1.1032786996437394</v>
       </c>
       <c r="AD7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.845736679362898</v>
+        <v>-1.2116345953177454</v>
       </c>
       <c r="AE7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.863135454837773</v>
+        <v>-1.3194987188833385</v>
       </c>
       <c r="AF7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8804855301895693</v>
+        <v>-1.4265799471028462</v>
       </c>
       <c r="AG7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8905830206418348</v>
+        <v>-1.537828170077804</v>
       </c>
       <c r="AH7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8996181842041446</v>
+        <v>-1.648887146879241</v>
       </c>
       <c r="AI7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.9079007847959693</v>
+        <v>-1.7595417723946905</v>
       </c>
       <c r="AJ7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.9158011348523805</v>
+        <v>-1.86950345626683</v>
       </c>
       <c r="AK7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.9236390587223049</v>
+        <v>-1.9784768298969579</v>
       </c>
       <c r="AL7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.9231993950436297</v>
+        <v>-2.0855284564764931</v>
       </c>
       <c r="AM7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.9209666867608841</v>
+        <v>-2.1914673157060083</v>
       </c>
       <c r="AN7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.9171231204214498</v>
+        <v>-2.2963811629559849</v>
       </c>
       <c r="AO7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.911769206946091</v>
+        <v>-2.4004268917252487</v>
       </c>
       <c r="AP7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.9049518599424506</v>
+        <v>-2.5037356931093768</v>
       </c>
       <c r="AQ7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8940385324500828</v>
+        <v>-2.6061166260749169</v>
       </c>
       <c r="AR7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8814726221983555</v>
+        <v>-2.7077912959215582</v>
       </c>
       <c r="AS7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8675560755517027</v>
+        <v>-2.8087819035527262</v>
       </c>
       <c r="AT7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.852573828002114</v>
+        <v>-2.909098413265665</v>
       </c>
       <c r="AU7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8367375662116778</v>
+        <v>-3.0087429095384306</v>
       </c>
       <c r="AV7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8184388359486112</v>
+        <v>-3.1026399639058284</v>
       </c>
       <c r="AW7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7992687429579166</v>
+        <v>-3.1948333767250814</v>
       </c>
       <c r="AX7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7794087331449391</v>
+        <v>-3.2855143293944344</v>
       </c>
       <c r="AY7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7590268287936426</v>
+        <v>-3.3749499344847833</v>
       </c>
       <c r="AZ7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7382610472803992</v>
+        <v>-3.4633544987890392</v>
       </c>
       <c r="BA7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7204879688719319</v>
+        <v>-3.5458701493699452</v>
       </c>
       <c r="BB7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7056687985878014</v>
+        <v>-3.6286311881190696</v>
       </c>
       <c r="BC7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6905274014482505</v>
+        <v>-3.7100210959082669</v>
       </c>
       <c r="BD7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6751000655087287</v>
+        <v>-3.7902081892557726</v>
       </c>
       <c r="BE7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6595309848436721</v>
+        <v>-3.8693535099939775</v>
       </c>
       <c r="BF7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6426427140642361</v>
+        <v>-3.9463127746038218</v>
       </c>
       <c r="BG7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6255265773697301</v>
+        <v>-4.0221721575330438</v>
       </c>
       <c r="BH7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6082886651969006</v>
+        <v>-4.0970219103658607</v>
       </c>
       <c r="BI7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.5910266586371855</v>
+        <v>-4.170955718841018</v>
       </c>
       <c r="BJ7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.5738164372193006</v>
+        <v>-4.2440590458176164</v>
       </c>
       <c r="BK7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.5564159346071147</v>
+        <v>-4.314918856613903</v>
       </c>
       <c r="BL7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.5391159005227371</v>
+        <v>-4.3847466334413614</v>
       </c>
       <c r="BM7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.5219623175955053</v>
+        <v>-4.4536575845551596</v>
       </c>
       <c r="BN7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.5049927014446194</v>
+        <v>-4.5217748416950698</v>
       </c>
       <c r="BO7" s="2">
         <f t="shared" ref="BO7:CI7" si="3">BO3-BO2</f>
-        <v>-2.4882326476251326</v>
+        <v>-4.5891841340081063</v>
       </c>
       <c r="BP7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.4711414631061412</v>
+        <v>-4.6500669729501958</v>
       </c>
       <c r="BQ7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.4542179509998263</v>
+        <v>-4.7091084258238824</v>
       </c>
       <c r="BR7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.4374982348842056</v>
+        <v>-4.766532007184221</v>
       </c>
       <c r="BS7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.4210155162512792</v>
+        <v>-4.822628127561801</v>
       </c>
       <c r="BT7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.4047947478542997</v>
+        <v>-4.8776257331803574</v>
       </c>
       <c r="BU7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.3892334662780068</v>
+        <v>-4.9292242743100285</v>
       </c>
       <c r="BV7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.3740351065630216</v>
+        <v>-4.9794617875934089</v>
       </c>
       <c r="BW7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.3591939516777072</v>
+        <v>-5.028529121718905</v>
       </c>
       <c r="BX7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.344700190984228</v>
+        <v>-5.0766333496403586</v>
       </c>
       <c r="BY7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.3305456139527836</v>
+        <v>-5.1239370559427844</v>
       </c>
       <c r="BZ7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.3167305493591472</v>
+        <v>-5.1656385463514258</v>
       </c>
       <c r="CA7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.303268027977734</v>
+        <v>-5.2057448609437831</v>
       </c>
       <c r="CB7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.2901533128280693</v>
+        <v>-5.2445009570563741</v>
       </c>
       <c r="CC7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.2773826674107212</v>
+        <v>-5.2821935370182871</v>
       </c>
       <c r="CD7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.264953178116369</v>
+        <v>-5.3190444847133094</v>
       </c>
       <c r="CE7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.2538427520225501</v>
+        <v>-5.3544346165925845</v>
       </c>
       <c r="CF7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.2432380041915723</v>
+        <v>-5.3891368459431321</v>
       </c>
       <c r="CG7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.2408179811543416</v>
+        <v>-5.423664191250765</v>
       </c>
       <c r="CH7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.2246311597601487</v>
+        <v>-5.456897085822666</v>
       </c>
       <c r="CI7" s="2">
         <f t="shared" si="3"/>
-        <v>-2.6653938051310111</v>
+        <v>-5.514956728189647</v>
       </c>
     </row>
     <row r="8" spans="1:87" x14ac:dyDescent="0.3">
@@ -5932,343 +5915,343 @@
       </c>
       <c r="C8" s="2">
         <f t="shared" ref="C8:BN8" si="4">C3</f>
-        <v>-0.11989295890919571</v>
+        <v>9.1492751157495888E-4</v>
       </c>
       <c r="D8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.2564913650720313</v>
+        <v>1.9380107544986203E-3</v>
       </c>
       <c r="E8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.40548218803949654</v>
+        <v>3.0370170623905679E-3</v>
       </c>
       <c r="F8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.5625868560056535</v>
+        <v>4.1803820710395456E-3</v>
       </c>
       <c r="G8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.72368591578868546</v>
+        <v>5.3381698501331343E-3</v>
       </c>
       <c r="H8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.89397615754910342</v>
+        <v>1.3157759753057441E-2</v>
       </c>
       <c r="I8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2536848339774753</v>
+        <v>0.21348505364844339</v>
       </c>
       <c r="J8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.5465477388130644</v>
+        <v>0.34910430938315251</v>
       </c>
       <c r="K8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.4663796850371669</v>
+        <v>0.10772874383697673</v>
       </c>
       <c r="L8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.3499516421471625</v>
+        <v>-0.16705601577994278</v>
       </c>
       <c r="M8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2432807826123216</v>
+        <v>-0.43465890355091075</v>
       </c>
       <c r="N8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1740907821493396</v>
+        <v>-0.66159570791660682</v>
       </c>
       <c r="O8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1293824838973121</v>
+        <v>-0.86101032056353777</v>
       </c>
       <c r="P8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0904536525910724</v>
+        <v>-1.0515687464137558</v>
       </c>
       <c r="Q8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0594058486379065</v>
+        <v>-1.2311097309259722</v>
       </c>
       <c r="R8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0183572616020098</v>
+        <v>-1.4228025754553508</v>
       </c>
       <c r="S8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0154352355562501</v>
+        <v>-1.5742008267198959</v>
       </c>
       <c r="T8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.037065636868395</v>
+        <v>-1.6992195584478065</v>
       </c>
       <c r="U8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0707668042763685</v>
+        <v>-1.8105357584278448</v>
       </c>
       <c r="V8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1090001761417945</v>
+        <v>-1.9158446646005745</v>
       </c>
       <c r="W8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1233479395032275</v>
+        <v>-2.0422926708964284</v>
       </c>
       <c r="X8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1356564507584044</v>
+        <v>-2.1692700651057328</v>
       </c>
       <c r="Y8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.147334199538641</v>
+        <v>-2.2955382898167564</v>
       </c>
       <c r="Z8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.160195655963403</v>
+        <v>-2.4194852035804293</v>
       </c>
       <c r="AA8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1758545383770969</v>
+        <v>-2.5396476528848577</v>
       </c>
       <c r="AB8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1850823533255617</v>
+        <v>-2.661324458444736</v>
       </c>
       <c r="AC8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1986687041575239</v>
+        <v>-2.7771446690231461</v>
       </c>
       <c r="AD8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2155170209160682</v>
+        <v>-2.8883528079100107</v>
       </c>
       <c r="AE8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2337160576910144</v>
+        <v>-2.9969917621188835</v>
       </c>
       <c r="AF8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2518586150598643</v>
+        <v>-3.1045562489061651</v>
       </c>
       <c r="AG8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2614657210244462</v>
+        <v>-3.2169190300692652</v>
       </c>
       <c r="AH8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2691587127149351</v>
+        <v>-3.3296402639445777</v>
       </c>
       <c r="AI8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2732600629612678</v>
+        <v>-3.4444508403099983</v>
       </c>
       <c r="AJ8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2703781735087571</v>
+        <v>-3.5647533183807201</v>
       </c>
       <c r="AK8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2540210547578035</v>
+        <v>-3.6969161347232715</v>
       </c>
       <c r="AL8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2342552264018036</v>
+        <v>-3.8217313853343149</v>
       </c>
       <c r="AM8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2131238461617344</v>
+        <v>-3.9448919323131437</v>
       </c>
       <c r="AN8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.193489392035052</v>
+        <v>-4.0639667698810111</v>
       </c>
       <c r="AO8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1768444016053481</v>
+        <v>-4.1779892250678348</v>
       </c>
       <c r="AP8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1637977662731003</v>
+        <v>-4.2867387241266375</v>
       </c>
       <c r="AQ8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1511488370674505</v>
+        <v>-4.390502402670271</v>
       </c>
       <c r="AR8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1416185393326339</v>
+        <v>-4.4892722927368904</v>
       </c>
       <c r="AS8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1346413446308934</v>
+        <v>-4.5838049366044631</v>
       </c>
       <c r="AT8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1294875920329184</v>
+        <v>-4.6750075756943232</v>
       </c>
       <c r="AU8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1253663585153451</v>
+        <v>-4.7638116158136619</v>
       </c>
       <c r="AV8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1192877374659904</v>
+        <v>-4.846398105559679</v>
       </c>
       <c r="AW8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1126615212282309</v>
+        <v>-4.9270733084887386</v>
       </c>
       <c r="AX8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.1051623325475934</v>
+        <v>-5.0064980472733112</v>
       </c>
       <c r="AY8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0966302471387412</v>
+        <v>-5.0852468488815639</v>
       </c>
       <c r="AZ8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0870101164449975</v>
+        <v>-5.1637059738566133</v>
       </c>
       <c r="BA8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0680057134171306</v>
+        <v>-5.2500419439234447</v>
       </c>
       <c r="BB8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.060643959087848</v>
+        <v>-5.3254923794368807</v>
       </c>
       <c r="BC8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.05568150858667</v>
+        <v>-5.397441557757543</v>
       </c>
       <c r="BD8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0508163034356865</v>
+        <v>-5.468206895285399</v>
       </c>
       <c r="BE8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0449263794827357</v>
+        <v>-5.538953308007299</v>
       </c>
       <c r="BF8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0350781535410358</v>
+        <v>-5.6100666583201564</v>
       </c>
       <c r="BG8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0239183935763507</v>
+        <v>-5.6811461839669679</v>
       </c>
       <c r="BH8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0116250753056444</v>
+        <v>-5.7521787639958966</v>
       </c>
       <c r="BI8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.99847212863372059</v>
+        <v>-5.8230693764018344</v>
       </c>
       <c r="BJ8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.98467917066891175</v>
+        <v>-5.8937551804897019</v>
       </c>
       <c r="BK8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.97007667068378378</v>
+        <v>-5.9627310400813149</v>
       </c>
       <c r="BL8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.95496489217563596</v>
+        <v>-6.0312211491092116</v>
       </c>
       <c r="BM8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.93936110914166759</v>
+        <v>-6.0993719673605673</v>
       </c>
       <c r="BN8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.92326116455754281</v>
+        <v>-6.1673530177726921</v>
       </c>
       <c r="BO8" s="2">
         <f t="shared" ref="BO8:CI8" si="5">BO3</f>
-        <v>-0.90665351933153504</v>
+        <v>-6.2352915712644119</v>
       </c>
       <c r="BP8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.88775550044941642</v>
+        <v>-6.2985615324749666</v>
       </c>
       <c r="BQ8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.86852547861959728</v>
+        <v>-6.3604577669279738</v>
       </c>
       <c r="BR8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.84888739793921308</v>
+        <v>-6.4213119370468359</v>
       </c>
       <c r="BS8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.82883728857620076</v>
+        <v>-6.4814497093279027</v>
       </c>
       <c r="BT8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.80839951654047004</v>
+        <v>-6.5411000815981835</v>
       </c>
       <c r="BU8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.78798787214297006</v>
+        <v>-6.597973463650475</v>
       </c>
       <c r="BV8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.7673256486760982</v>
+        <v>-6.6540575869920682</v>
       </c>
       <c r="BW8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.74642452707111007</v>
+        <v>-6.7095267408472932</v>
       </c>
       <c r="BX8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.72528794941011387</v>
+        <v>-6.7645730315837538</v>
       </c>
       <c r="BY8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.70391821298150248</v>
+        <v>-6.8193461873122807</v>
       </c>
       <c r="BZ8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.68132849998288059</v>
+        <v>-6.8700194906914147</v>
       </c>
       <c r="CA8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.65872022851274359</v>
+        <v>-6.9194266938419453</v>
       </c>
       <c r="CB8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.63600672294508165</v>
+        <v>-6.9678909725079947</v>
       </c>
       <c r="CC8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.61315682225527857</v>
+        <v>-7.0157234307819056</v>
       </c>
       <c r="CD8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.59016393322215421</v>
+        <v>-7.063148609647496</v>
       </c>
       <c r="CE8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.56801025030791541</v>
+        <v>-7.109622597534071</v>
       </c>
       <c r="CF8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.54588587020560908</v>
+        <v>-7.1558280095632254</v>
       </c>
       <c r="CG8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.53146903557963476</v>
+        <v>-7.1946536881305363</v>
       </c>
       <c r="CH8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.50280363543084849</v>
+        <v>-7.2466119899013197</v>
       </c>
       <c r="CI8" s="2">
         <f t="shared" si="5"/>
-        <v>-0.9305997798967458</v>
+        <v>-6.8712948072433004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simule avec nouveau scénario mondial
</commit_message>
<xml_diff>
--- a/results/Décomposition CP.xlsx
+++ b/results/Décomposition CP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flori\Documents\Github\ThreeME_V3-ADEME\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10942160-48B6-4095-893D-0557620857BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866937E1-FED2-4E83-943F-2572853AC3A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{64203D87-38B7-4BDD-A33D-820F861F4EFC}"/>
   </bookViews>
@@ -519,238 +519,238 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.19161550315185405</c:v>
+                  <c:v>-8.2056637038441238E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.31789887951911844</c:v>
+                  <c:v>-0.21283364242431491</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>6.7015030786099494E-2</c:v>
+                  <c:v>-0.39025278208807412</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-0.21728167797012699</c:v>
+                  <c:v>-0.59628327178540275</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-0.46886133701437016</c:v>
+                  <c:v>-0.81562590353156939</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-0.67638884472317473</c:v>
+                  <c:v>-1.0216278909715992</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-0.85375889954031337</c:v>
+                  <c:v>-1.2032345153876411</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-1.0207112465597246</c:v>
+                  <c:v>-1.3504639790627215</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-1.1759379933896641</c:v>
+                  <c:v>-1.4585944232260228</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.307531973432452</c:v>
+                  <c:v>-1.5517555857743948</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-1.3941416492964653</c:v>
+                  <c:v>-1.5951026922136013</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-1.4508647654808193</c:v>
+                  <c:v>-1.6040668534222591</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-1.4919916852337844</c:v>
+                  <c:v>-1.5931250202945058</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-1.5264967867797408</c:v>
+                  <c:v>-1.5713350192618547</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-1.5576296940993828</c:v>
+                  <c:v>-1.5651218195565586</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-1.5861667841999827</c:v>
+                  <c:v>-1.554404043652069</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-1.6118588854758364</c:v>
+                  <c:v>-1.5381127661592275</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-1.6342925349397075</c:v>
+                  <c:v>-1.5150887663259005</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-1.6529130346936594</c:v>
+                  <c:v>-1.4843693729708951</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-1.6664774336045296</c:v>
+                  <c:v>-1.4670959735900491</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-1.6738659693794067</c:v>
+                  <c:v>-1.4415172238670282</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-1.6767182125922653</c:v>
+                  <c:v>-1.4083443590699352</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-1.677493043235545</c:v>
+                  <c:v>-1.369330271902458</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-1.6779763018033189</c:v>
+                  <c:v>-1.3259532326168944</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-1.6790908599914611</c:v>
+                  <c:v>-1.3024859273049971</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-1.6807531170653367</c:v>
+                  <c:v>-1.2777267899411027</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-1.6849090679153078</c:v>
+                  <c:v>-1.2527233993570031</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-1.6952498621138901</c:v>
+                  <c:v>-1.2304848598072127</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-1.7184393048263136</c:v>
+                  <c:v>-1.2174546113713047</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-1.7362029288578218</c:v>
+                  <c:v>-1.237908577251623</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-1.7534246166071354</c:v>
+                  <c:v>-1.2603538312162543</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-1.7675856069250262</c:v>
+                  <c:v>-1.280896991656888</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-1.7775623333425861</c:v>
+                  <c:v>-1.297188457191123</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-1.7830030310172607</c:v>
+                  <c:v>-1.3082209222382457</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-1.7843857765953541</c:v>
+                  <c:v>-1.3141866871164254</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-1.7814809968153322</c:v>
+                  <c:v>-1.3148074597939763</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-1.7750230330517369</c:v>
+                  <c:v>-1.3108556960684137</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-1.7659091624286583</c:v>
+                  <c:v>-1.303275763656131</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-1.7550687062752313</c:v>
+                  <c:v>-1.2930319435366266</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-1.7437581416538506</c:v>
+                  <c:v>-1.281342220396231</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-1.7322399317636572</c:v>
+                  <c:v>-1.2684877326585298</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-1.7209837178788767</c:v>
+                  <c:v>-1.2549757446242316</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-1.7102969143967806</c:v>
+                  <c:v>-1.2411581680791373</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-1.7003514750675741</c:v>
+                  <c:v>-1.2272642485102625</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-1.7041717945534995</c:v>
+                  <c:v>-1.2242065628020882</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-1.6968611913178111</c:v>
+                  <c:v>-1.212274094328003</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-1.6874204618492761</c:v>
+                  <c:v>-1.1969362266087136</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-1.6779987060296264</c:v>
+                  <c:v>-1.18070260801586</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>-1.6695997980133215</c:v>
+                  <c:v>-1.16492077109287</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>-1.6637538837163346</c:v>
+                  <c:v>-1.1511401161751533</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>-1.6589740264339237</c:v>
+                  <c:v>-1.1378958971931308</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>-1.6551568536300354</c:v>
+                  <c:v>-1.1250898290850242</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>-1.6521136575608164</c:v>
+                  <c:v>-1.1125532871455235</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>-1.6496961346720851</c:v>
+                  <c:v>-1.1001719824118905</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>-1.647812183467412</c:v>
+                  <c:v>-1.0878917622401674</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>-1.6464745156678506</c:v>
+                  <c:v>-1.0757687980817221</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>-1.6457143828054077</c:v>
+                  <c:v>-1.063870997528682</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>-1.6455781760776222</c:v>
+                  <c:v>-1.0522736454812165</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>-1.6461074372563056</c:v>
+                  <c:v>-1.0410385324777782</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>-1.6484945595247713</c:v>
+                  <c:v>-1.0312423250512404</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>-1.6513493411040914</c:v>
+                  <c:v>-1.0214957006012715</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>-1.6547799298626154</c:v>
+                  <c:v>-1.0118976129306012</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>-1.6588215817661012</c:v>
+                  <c:v>-1.0024819779150707</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>-1.663474348417826</c:v>
+                  <c:v>-0.99324739033723741</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>-1.668749189340446</c:v>
+                  <c:v>-0.98420512175648733</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>-1.6745957993986593</c:v>
+                  <c:v>-0.97529371947724375</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>-1.6809976191283882</c:v>
+                  <c:v>-0.96648595744011079</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>-1.6879396819433956</c:v>
+                  <c:v>-0.9577552203525963</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>-1.6954091313694963</c:v>
+                  <c:v>-0.94907697959949466</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>-1.7043809443399893</c:v>
+                  <c:v>-0.94129484741348746</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>-1.7136818328981618</c:v>
+                  <c:v>-0.93323535150678927</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>-1.7233900154516202</c:v>
+                  <c:v>-0.9249666077962293</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>-1.733529893763619</c:v>
+                  <c:v>-0.91651274199079369</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>-1.7441041249341871</c:v>
+                  <c:v>-0.90787715348179532</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>-1.7551879809414861</c:v>
+                  <c:v>-0.89914837199471798</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>-1.7666911636200933</c:v>
+                  <c:v>-0.8902214872785974</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>-1.7709894968797713</c:v>
+                  <c:v>-0.88109715314373949</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>-1.7897149040786542</c:v>
+                  <c:v>-0.87177687957782357</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1077,238 +1077,238 @@
                   <c:v>1.3157759753057441E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.1869550496589341E-2</c:v>
+                  <c:v>2.2292788023148269E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.1205429864034073E-2</c:v>
+                  <c:v>3.2139088170790586E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4.0713713050877232E-2</c:v>
+                  <c:v>4.2129485191733096E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>5.0225662190184206E-2</c:v>
+                  <c:v>5.1975242771151731E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.4202433463459414E-2</c:v>
+                  <c:v>3.6017857349646132E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.4793136806567908E-2</c:v>
+                  <c:v>1.6399497469810065E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-7.2514210232244025E-3</c:v>
+                  <c:v>-5.9892217015078408E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-3.085749985403119E-2</c:v>
+                  <c:v>-2.9968546411729413E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-5.5171737536308108E-2</c:v>
+                  <c:v>-5.4577153530033229E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-0.11527060202289885</c:v>
+                  <c:v>-0.11463976727003056</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-0.18005917742343058</c:v>
+                  <c:v>-0.17919008783575663</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-0.24835479296698715</c:v>
+                  <c:v>-0.24713328455195915</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-0.31854407319406031</c:v>
+                  <c:v>-0.31695567151074355</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-0.38934787782083369</c:v>
+                  <c:v>-0.38745994979798581</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-0.48466297679704562</c:v>
+                  <c:v>-0.48250703231480507</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-0.58310328090575014</c:v>
+                  <c:v>-0.58080471991275306</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-0.68367940434092001</c:v>
+                  <c:v>-0.68138580947760818</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-0.78519266864072179</c:v>
+                  <c:v>-0.78306998913987291</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-0.88673461819119836</c:v>
+                  <c:v>-0.88496209607368259</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-0.99484702484020637</c:v>
+                  <c:v>-0.99340996282157867</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-1.1032786996437394</c:v>
+                  <c:v>-1.1022916149202144</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-1.2116345953177454</c:v>
+                  <c:v>-1.2112272072063335</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-1.3194987188833385</c:v>
+                  <c:v>-1.3198210676801048</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-1.4265799471028462</c:v>
+                  <c:v>-1.4277976274376325</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-1.537828170077804</c:v>
+                  <c:v>-1.5397852860289496</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-1.648887146879241</c:v>
+                  <c:v>-1.6516752493175968</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-1.7595417723946905</c:v>
+                  <c:v>-1.7632678954715209</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-1.86950345626683</c:v>
+                  <c:v>-1.8742920847076738</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-1.9784768298969579</c:v>
+                  <c:v>-1.9844642318590289</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-2.0855284564764931</c:v>
+                  <c:v>-2.0919608909966803</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-2.1914673157060083</c:v>
+                  <c:v>-2.1982511042945796</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-2.2963811629559849</c:v>
+                  <c:v>-2.3034690719921258</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-2.4004268917252487</c:v>
+                  <c:v>-2.4078233531100168</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-2.5037356931093768</c:v>
+                  <c:v>-2.5114737457364145</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-2.6061166260749169</c:v>
+                  <c:v>-2.6142273067976896</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-2.7077912959215582</c:v>
+                  <c:v>-2.7162969204475695</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-2.8087819035527262</c:v>
+                  <c:v>-2.8177005006226441</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-2.909098413265665</c:v>
+                  <c:v>-2.9184480901740089</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-3.0087429095384306</c:v>
+                  <c:v>-3.0185437049097379</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-3.1026399639058284</c:v>
+                  <c:v>-3.1128941096520646</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-3.1948333767250814</c:v>
+                  <c:v>-3.2055617006753074</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-3.2855143293944344</c:v>
+                  <c:v>-3.2967397660182529</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-3.3749499344847833</c:v>
+                  <c:v>-3.3866969784453027</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-3.4633544987890392</c:v>
+                  <c:v>-3.4756487438021293</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-3.5458701493699452</c:v>
+                  <c:v>-3.5588213169056253</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-3.6286311881190696</c:v>
+                  <c:v>-3.6421334394924898</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-3.7100210959082669</c:v>
+                  <c:v>-3.7241246149772649</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-3.7902081892557726</c:v>
+                  <c:v>-3.8049512103243366</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>-3.8693535099939775</c:v>
+                  <c:v>-3.8847632236486902</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>-3.9463127746038218</c:v>
+                  <c:v>-3.9624153625143488</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>-4.0221721575330438</c:v>
+                  <c:v>-4.0389984244915134</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>-4.0970219103658607</c:v>
+                  <c:v>-4.1146046351699059</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>-4.170955718841018</c:v>
+                  <c:v>-4.1893280061036098</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>-4.2440590458176164</c:v>
+                  <c:v>-4.2632532113688342</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>-4.314918856613903</c:v>
+                  <c:v>-4.3349573485010335</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>-4.3847466334413614</c:v>
+                  <c:v>-4.4056564737814057</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>-4.4536575845551596</c:v>
+                  <c:v>-4.4754646684001642</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>-4.5217748416950698</c:v>
+                  <c:v>-4.5445046238458016</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>-4.5891841340081063</c:v>
+                  <c:v>-4.6128619288378747</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>-4.6500669729501958</c:v>
+                  <c:v>-4.6746905109283254</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>-4.7091084258238824</c:v>
+                  <c:v>-4.7347013171329611</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>-4.766532007184221</c:v>
+                  <c:v>-4.7931200537459144</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>-4.822628127561801</c:v>
+                  <c:v>-4.8502393825534114</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>-4.8776257331803574</c:v>
+                  <c:v>-4.9062901536244707</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>-4.9292242743100285</c:v>
+                  <c:v>-4.9589558561843994</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>-4.9794617875934089</c:v>
+                  <c:v>-5.0102887839834187</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>-5.028529121718905</c:v>
+                  <c:v>-5.0604815743773512</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>-5.0766333496403586</c:v>
+                  <c:v>-5.1097433773469092</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>-5.1239370559427844</c:v>
+                  <c:v>-5.1582385967361972</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>-5.1656385463514258</c:v>
+                  <c:v>-5.2011378789825091</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>-5.2057448609437831</c:v>
+                  <c:v>-5.2424753860368707</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>-5.2445009570563741</c:v>
+                  <c:v>-5.2824984944638285</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>-5.2821935370182871</c:v>
+                  <c:v>-5.3214961925659559</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>-5.3190444847133094</c:v>
+                  <c:v>-5.3596921868446117</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>-5.3544346165925845</c:v>
+                  <c:v>-5.3964613459674293</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>-5.3891368459431321</c:v>
+                  <c:v>-5.4325839433267742</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>-5.423664191250765</c:v>
+                  <c:v>-5.4681527339620732</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>-5.456897085822666</c:v>
+                  <c:v>-5.503241916564094</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1653,238 +1653,238 @@
                   <c:v>1.3157759753057441E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.21348505364844339</c:v>
+                  <c:v>-5.9763849015292969E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.34910430938315251</c:v>
+                  <c:v>-0.18069455425352432</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.10772874383697673</c:v>
+                  <c:v>-0.34812329689634103</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-0.16705601577994278</c:v>
+                  <c:v>-0.54430802901425102</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-0.43465890355091075</c:v>
+                  <c:v>-0.77960804618192325</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-0.66159570791660682</c:v>
+                  <c:v>-1.0052283935017892</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-0.86101032056353777</c:v>
+                  <c:v>-1.209223737089149</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-1.0515687464137558</c:v>
+                  <c:v>-1.3804325254744509</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-1.2311097309259722</c:v>
+                  <c:v>-1.5131715767560561</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.4228025754553508</c:v>
+                  <c:v>-1.6663953530444253</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-1.5742008267198959</c:v>
+                  <c:v>-1.774292780049358</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-1.6992195584478065</c:v>
+                  <c:v>-1.8512001379742182</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-1.8105357584278448</c:v>
+                  <c:v>-1.9100806918052493</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-1.9158446646005745</c:v>
+                  <c:v>-1.9587949690598405</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-2.0422926708964284</c:v>
+                  <c:v>-2.0476288518713637</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-2.1692700651057328</c:v>
+                  <c:v>-2.135208763564822</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-2.2955382898167564</c:v>
+                  <c:v>-2.2194985756368357</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-2.4194852035804293</c:v>
+                  <c:v>-2.2981587554657734</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-2.5396476528848577</c:v>
+                  <c:v>-2.3693314690445777</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-2.661324458444736</c:v>
+                  <c:v>-2.4605059364116277</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-2.7771446690231461</c:v>
+                  <c:v>-2.5438088387872426</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-2.8883528079100107</c:v>
+                  <c:v>-2.6195715662762686</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-2.9969917621188835</c:v>
+                  <c:v>-2.6891513395825628</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-3.1045562489061651</c:v>
+                  <c:v>-2.7537508600545269</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-3.2169190300692652</c:v>
+                  <c:v>-2.8422712133339467</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-3.3296402639445777</c:v>
+                  <c:v>-2.9294020392586995</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-3.4444508403099983</c:v>
+                  <c:v>-3.0159912948285239</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-3.5647533183807201</c:v>
+                  <c:v>-3.1047769445148865</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-3.6969161347232715</c:v>
+                  <c:v>-3.2019188432303336</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-3.8217313853343149</c:v>
+                  <c:v>-3.3298694682483032</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-3.9448919323131437</c:v>
+                  <c:v>-3.4586049355108339</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-4.0639667698810111</c:v>
+                  <c:v>-3.5843660636490138</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-4.1779892250678348</c:v>
+                  <c:v>-3.7050118103011398</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-4.2867387241266375</c:v>
+                  <c:v>-3.8196946679746602</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-4.390502402670271</c:v>
+                  <c:v>-3.9284139939141149</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-4.4892722927368904</c:v>
+                  <c:v>-4.0311043802415458</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-4.5838049366044631</c:v>
+                  <c:v>-4.1285561966910578</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-4.6750075756943232</c:v>
+                  <c:v>-4.2217238538301398</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-4.7638116158136619</c:v>
+                  <c:v>-4.3115756484463645</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-4.846398105559679</c:v>
+                  <c:v>-4.3942363300482956</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-4.9270733084887386</c:v>
+                  <c:v>-4.4740494333338372</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-5.0064980472733112</c:v>
+                  <c:v>-4.5517155106424845</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-5.0852468488815639</c:v>
+                  <c:v>-4.62785514652444</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-5.1637059738566133</c:v>
+                  <c:v>-4.7029129923123918</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-5.2500419439234447</c:v>
+                  <c:v>-4.7830278797077135</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-5.3254923794368807</c:v>
+                  <c:v>-4.8544075338204928</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-5.397441557757543</c:v>
+                  <c:v>-4.9210608415859785</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-5.468206895285399</c:v>
+                  <c:v>-4.9856538183401966</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>-5.538953308007299</c:v>
+                  <c:v>-5.0496839947415602</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>-5.6100666583201564</c:v>
+                  <c:v>-5.1135554786895021</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>-5.6811461839669679</c:v>
+                  <c:v>-5.1768943216846441</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>-5.7521787639958966</c:v>
+                  <c:v>-5.2396944642549297</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>-5.8230693764018344</c:v>
+                  <c:v>-5.3018812932491333</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>-5.8937551804897019</c:v>
+                  <c:v>-5.3634251937807242</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>-5.9627310400813149</c:v>
+                  <c:v>-5.4228491107412014</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>-6.0312211491092116</c:v>
+                  <c:v>-5.4814252718631273</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>-6.0993719673605673</c:v>
+                  <c:v>-5.5393356659288457</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>-6.1673530177726921</c:v>
+                  <c:v>-5.5967782693270181</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>-6.2352915712644119</c:v>
+                  <c:v>-5.6539004613156525</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>-6.2985615324749666</c:v>
+                  <c:v>-5.7059328359795654</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>-6.3604577669279738</c:v>
+                  <c:v>-5.7561970177342321</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>-6.4213119370468359</c:v>
+                  <c:v>-5.8050176666765152</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>-6.4814497093279027</c:v>
+                  <c:v>-5.8527213604684825</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>-6.5411000815981835</c:v>
+                  <c:v>-5.8995375439617082</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>-6.597973463650475</c:v>
+                  <c:v>-5.9431609779408863</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>-6.6540575869920682</c:v>
+                  <c:v>-5.9855825034606625</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>-6.7095267408472932</c:v>
+                  <c:v>-6.026967531817462</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>-6.7645730315837538</c:v>
+                  <c:v>-6.0674985976995055</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>-6.8193461873122807</c:v>
+                  <c:v>-6.1073155763356919</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>-6.8700194906914147</c:v>
+                  <c:v>-6.142432726395997</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>-6.9194266938419453</c:v>
+                  <c:v>-6.1757107375436604</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>-6.9678909725079947</c:v>
+                  <c:v>-6.2074651022600573</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>-7.0157234307819056</c:v>
+                  <c:v>-6.2380089345567491</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>-7.063148609647496</c:v>
+                  <c:v>-6.267569340326407</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>-7.109622597534071</c:v>
+                  <c:v>-6.2956097179621473</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>-7.1558280095632254</c:v>
+                  <c:v>-6.3228054306053716</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>-7.1946536881305363</c:v>
+                  <c:v>-6.3492498871058123</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>-7.2466119899013197</c:v>
+                  <c:v>-6.3750187961419176</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2676,7 +2676,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="9298459" cy="6065108"/>
+    <xdr:ext cx="9300308" cy="6076462"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Graphique 1">
@@ -2744,267 +2744,555 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0">
+        <row r="4">
+          <cell r="C4">
+            <v>42005</v>
+          </cell>
+          <cell r="D4">
+            <v>42370</v>
+          </cell>
+          <cell r="E4">
+            <v>42736</v>
+          </cell>
+          <cell r="F4">
+            <v>43101</v>
+          </cell>
+          <cell r="G4">
+            <v>43466</v>
+          </cell>
+          <cell r="H4">
+            <v>43831</v>
+          </cell>
+          <cell r="I4">
+            <v>44197</v>
+          </cell>
+          <cell r="J4">
+            <v>44562</v>
+          </cell>
+          <cell r="K4">
+            <v>44927</v>
+          </cell>
+          <cell r="L4">
+            <v>45292</v>
+          </cell>
+          <cell r="M4">
+            <v>45658</v>
+          </cell>
+          <cell r="N4">
+            <v>46023</v>
+          </cell>
+          <cell r="O4">
+            <v>46388</v>
+          </cell>
+          <cell r="P4">
+            <v>46753</v>
+          </cell>
+          <cell r="Q4">
+            <v>47119</v>
+          </cell>
+          <cell r="R4">
+            <v>47484</v>
+          </cell>
+          <cell r="S4">
+            <v>47849</v>
+          </cell>
+          <cell r="T4">
+            <v>48214</v>
+          </cell>
+          <cell r="U4">
+            <v>48580</v>
+          </cell>
+          <cell r="V4">
+            <v>48945</v>
+          </cell>
+          <cell r="W4">
+            <v>49310</v>
+          </cell>
+          <cell r="X4">
+            <v>49675</v>
+          </cell>
+          <cell r="Y4">
+            <v>50041</v>
+          </cell>
+          <cell r="Z4">
+            <v>50406</v>
+          </cell>
+          <cell r="AA4">
+            <v>50771</v>
+          </cell>
+          <cell r="AB4">
+            <v>51136</v>
+          </cell>
+          <cell r="AC4">
+            <v>51502</v>
+          </cell>
+          <cell r="AD4">
+            <v>51867</v>
+          </cell>
+          <cell r="AE4">
+            <v>52232</v>
+          </cell>
+          <cell r="AF4">
+            <v>52597</v>
+          </cell>
+          <cell r="AG4">
+            <v>52963</v>
+          </cell>
+          <cell r="AH4">
+            <v>53328</v>
+          </cell>
+          <cell r="AI4">
+            <v>53693</v>
+          </cell>
+          <cell r="AJ4">
+            <v>54058</v>
+          </cell>
+          <cell r="AK4">
+            <v>54424</v>
+          </cell>
+          <cell r="AL4">
+            <v>54789</v>
+          </cell>
+          <cell r="AM4">
+            <v>55154</v>
+          </cell>
+          <cell r="AN4">
+            <v>55519</v>
+          </cell>
+          <cell r="AO4">
+            <v>55885</v>
+          </cell>
+          <cell r="AP4">
+            <v>56250</v>
+          </cell>
+          <cell r="AQ4">
+            <v>56615</v>
+          </cell>
+          <cell r="AR4">
+            <v>56980</v>
+          </cell>
+          <cell r="AS4">
+            <v>57346</v>
+          </cell>
+          <cell r="AT4">
+            <v>57711</v>
+          </cell>
+          <cell r="AU4">
+            <v>58076</v>
+          </cell>
+          <cell r="AV4">
+            <v>58441</v>
+          </cell>
+          <cell r="AW4">
+            <v>58807</v>
+          </cell>
+          <cell r="AX4">
+            <v>59172</v>
+          </cell>
+          <cell r="AY4">
+            <v>59537</v>
+          </cell>
+          <cell r="AZ4">
+            <v>59902</v>
+          </cell>
+          <cell r="BA4">
+            <v>60268</v>
+          </cell>
+          <cell r="BB4">
+            <v>60633</v>
+          </cell>
+          <cell r="BC4">
+            <v>60998</v>
+          </cell>
+          <cell r="BD4">
+            <v>61363</v>
+          </cell>
+          <cell r="BE4">
+            <v>61729</v>
+          </cell>
+          <cell r="BF4">
+            <v>62094</v>
+          </cell>
+          <cell r="BG4">
+            <v>62459</v>
+          </cell>
+          <cell r="BH4">
+            <v>62824</v>
+          </cell>
+          <cell r="BI4">
+            <v>63190</v>
+          </cell>
+          <cell r="BJ4">
+            <v>63555</v>
+          </cell>
+          <cell r="BK4">
+            <v>63920</v>
+          </cell>
+          <cell r="BL4">
+            <v>64285</v>
+          </cell>
+          <cell r="BM4">
+            <v>64651</v>
+          </cell>
+          <cell r="BN4">
+            <v>65016</v>
+          </cell>
+          <cell r="BO4">
+            <v>65381</v>
+          </cell>
+          <cell r="BP4">
+            <v>65746</v>
+          </cell>
+          <cell r="BQ4">
+            <v>66112</v>
+          </cell>
+          <cell r="BR4">
+            <v>66477</v>
+          </cell>
+          <cell r="BS4">
+            <v>66842</v>
+          </cell>
+          <cell r="BT4">
+            <v>67207</v>
+          </cell>
+          <cell r="BU4">
+            <v>67573</v>
+          </cell>
+          <cell r="BV4">
+            <v>67938</v>
+          </cell>
+          <cell r="BW4">
+            <v>68303</v>
+          </cell>
+          <cell r="BX4">
+            <v>68668</v>
+          </cell>
+          <cell r="BY4">
+            <v>69034</v>
+          </cell>
+          <cell r="BZ4">
+            <v>69399</v>
+          </cell>
+          <cell r="CA4">
+            <v>69764</v>
+          </cell>
+          <cell r="CB4">
+            <v>70129</v>
+          </cell>
+          <cell r="CC4">
+            <v>70495</v>
+          </cell>
+          <cell r="CD4">
+            <v>70860</v>
+          </cell>
+          <cell r="CE4">
+            <v>71225</v>
+          </cell>
+          <cell r="CF4">
+            <v>71590</v>
+          </cell>
+          <cell r="CG4">
+            <v>71956</v>
+          </cell>
+          <cell r="CH4">
+            <v>72321</v>
+          </cell>
+          <cell r="CI4">
+            <v>72686</v>
+          </cell>
+          <cell r="CJ4">
+            <v>73051</v>
+          </cell>
+        </row>
         <row r="5">
           <cell r="C5">
             <v>0</v>
           </cell>
           <cell r="D5">
-            <v>0</v>
+            <v>9.1492751157495888E-4</v>
           </cell>
           <cell r="E5">
-            <v>0</v>
+            <v>1.9380107544986203E-3</v>
           </cell>
           <cell r="F5">
-            <v>0</v>
+            <v>3.0370170623905679E-3</v>
           </cell>
           <cell r="G5">
-            <v>0</v>
+            <v>4.1803820710395456E-3</v>
           </cell>
           <cell r="H5">
-            <v>0</v>
+            <v>5.3381698501331343E-3</v>
           </cell>
           <cell r="I5">
-            <v>0</v>
+            <v>1.3157759753057441E-2</v>
           </cell>
           <cell r="J5">
-            <v>0.19161550315185405</v>
+            <v>-5.9763849015292969E-2</v>
           </cell>
           <cell r="K5">
-            <v>0.31789887951911844</v>
+            <v>-0.18069455425352432</v>
           </cell>
           <cell r="L5">
-            <v>6.7015030786099494E-2</v>
+            <v>-0.34812329689634103</v>
           </cell>
           <cell r="M5">
-            <v>-0.21728167797012699</v>
+            <v>-0.54430802901425102</v>
           </cell>
           <cell r="N5">
-            <v>-0.46886133701437016</v>
+            <v>-0.77960804618192325</v>
           </cell>
           <cell r="O5">
-            <v>-0.67638884472317473</v>
+            <v>-1.0052283935017892</v>
           </cell>
           <cell r="P5">
-            <v>-0.85375889954031337</v>
+            <v>-1.209223737089149</v>
           </cell>
           <cell r="Q5">
-            <v>-1.0207112465597246</v>
+            <v>-1.3804325254744509</v>
           </cell>
           <cell r="R5">
-            <v>-1.1759379933896641</v>
+            <v>-1.5131715767560561</v>
           </cell>
           <cell r="S5">
-            <v>-1.307531973432452</v>
+            <v>-1.6663953530444253</v>
           </cell>
           <cell r="T5">
-            <v>-1.3941416492964653</v>
+            <v>-1.774292780049358</v>
           </cell>
           <cell r="U5">
-            <v>-1.4508647654808193</v>
+            <v>-1.8512001379742182</v>
           </cell>
           <cell r="V5">
-            <v>-1.4919916852337844</v>
+            <v>-1.9100806918052493</v>
           </cell>
           <cell r="W5">
-            <v>-1.5264967867797408</v>
+            <v>-1.9587949690598405</v>
           </cell>
           <cell r="X5">
-            <v>-1.5576296940993828</v>
+            <v>-2.0476288518713637</v>
           </cell>
           <cell r="Y5">
-            <v>-1.5861667841999827</v>
+            <v>-2.135208763564822</v>
           </cell>
           <cell r="Z5">
-            <v>-1.6118588854758364</v>
+            <v>-2.2194985756368357</v>
           </cell>
           <cell r="AA5">
-            <v>-1.6342925349397075</v>
+            <v>-2.2981587554657734</v>
           </cell>
           <cell r="AB5">
-            <v>-1.6529130346936594</v>
+            <v>-2.3693314690445777</v>
           </cell>
           <cell r="AC5">
-            <v>-1.6664774336045296</v>
+            <v>-2.4605059364116277</v>
           </cell>
           <cell r="AD5">
-            <v>-1.6738659693794067</v>
+            <v>-2.5438088387872426</v>
           </cell>
           <cell r="AE5">
-            <v>-1.6767182125922653</v>
+            <v>-2.6195715662762686</v>
           </cell>
           <cell r="AF5">
-            <v>-1.677493043235545</v>
+            <v>-2.6891513395825628</v>
           </cell>
           <cell r="AG5">
-            <v>-1.6779763018033189</v>
+            <v>-2.7537508600545269</v>
           </cell>
           <cell r="AH5">
-            <v>-1.6790908599914611</v>
+            <v>-2.8422712133339467</v>
           </cell>
           <cell r="AI5">
-            <v>-1.6807531170653367</v>
+            <v>-2.9294020392586995</v>
           </cell>
           <cell r="AJ5">
-            <v>-1.6849090679153078</v>
+            <v>-3.0159912948285239</v>
           </cell>
           <cell r="AK5">
-            <v>-1.6952498621138901</v>
+            <v>-3.1047769445148865</v>
           </cell>
           <cell r="AL5">
-            <v>-1.7184393048263136</v>
+            <v>-3.2019188432303336</v>
           </cell>
           <cell r="AM5">
-            <v>-1.7362029288578218</v>
+            <v>-3.3298694682483032</v>
           </cell>
           <cell r="AN5">
-            <v>-1.7534246166071354</v>
+            <v>-3.4586049355108339</v>
           </cell>
           <cell r="AO5">
-            <v>-1.7675856069250262</v>
+            <v>-3.5843660636490138</v>
           </cell>
           <cell r="AP5">
-            <v>-1.7775623333425861</v>
+            <v>-3.7050118103011398</v>
           </cell>
           <cell r="AQ5">
-            <v>-1.7830030310172607</v>
+            <v>-3.8196946679746602</v>
           </cell>
           <cell r="AR5">
-            <v>-1.7843857765953541</v>
+            <v>-3.9284139939141149</v>
           </cell>
           <cell r="AS5">
-            <v>-1.7814809968153322</v>
+            <v>-4.0311043802415458</v>
           </cell>
           <cell r="AT5">
-            <v>-1.7750230330517369</v>
+            <v>-4.1285561966910578</v>
           </cell>
           <cell r="AU5">
-            <v>-1.7659091624286583</v>
+            <v>-4.2217238538301398</v>
           </cell>
           <cell r="AV5">
-            <v>-1.7550687062752313</v>
+            <v>-4.3115756484463645</v>
           </cell>
           <cell r="AW5">
-            <v>-1.7437581416538506</v>
+            <v>-4.3942363300482956</v>
           </cell>
           <cell r="AX5">
-            <v>-1.7322399317636572</v>
+            <v>-4.4740494333338372</v>
           </cell>
           <cell r="AY5">
-            <v>-1.7209837178788767</v>
+            <v>-4.5517155106424845</v>
           </cell>
           <cell r="AZ5">
-            <v>-1.7102969143967806</v>
+            <v>-4.62785514652444</v>
           </cell>
           <cell r="BA5">
-            <v>-1.7003514750675741</v>
+            <v>-4.7029129923123918</v>
           </cell>
           <cell r="BB5">
-            <v>-1.7041717945534995</v>
+            <v>-4.7830278797077135</v>
           </cell>
           <cell r="BC5">
-            <v>-1.6968611913178111</v>
+            <v>-4.8544075338204928</v>
           </cell>
           <cell r="BD5">
-            <v>-1.6874204618492761</v>
+            <v>-4.9210608415859785</v>
           </cell>
           <cell r="BE5">
-            <v>-1.6779987060296264</v>
+            <v>-4.9856538183401966</v>
           </cell>
           <cell r="BF5">
-            <v>-1.6695997980133215</v>
+            <v>-5.0496839947415602</v>
           </cell>
           <cell r="BG5">
-            <v>-1.6637538837163346</v>
+            <v>-5.1135554786895021</v>
           </cell>
           <cell r="BH5">
-            <v>-1.6589740264339237</v>
+            <v>-5.1768943216846441</v>
           </cell>
           <cell r="BI5">
-            <v>-1.6551568536300354</v>
+            <v>-5.2396944642549297</v>
           </cell>
           <cell r="BJ5">
-            <v>-1.6521136575608164</v>
+            <v>-5.3018812932491333</v>
           </cell>
           <cell r="BK5">
-            <v>-1.6496961346720851</v>
+            <v>-5.3634251937807242</v>
           </cell>
           <cell r="BL5">
-            <v>-1.647812183467412</v>
+            <v>-5.4228491107412014</v>
           </cell>
           <cell r="BM5">
-            <v>-1.6464745156678506</v>
+            <v>-5.4814252718631273</v>
           </cell>
           <cell r="BN5">
-            <v>-1.6457143828054077</v>
+            <v>-5.5393356659288457</v>
           </cell>
           <cell r="BO5">
-            <v>-1.6455781760776222</v>
+            <v>-5.5967782693270181</v>
           </cell>
           <cell r="BP5">
-            <v>-1.6461074372563056</v>
+            <v>-5.6539004613156525</v>
           </cell>
           <cell r="BQ5">
-            <v>-1.6484945595247713</v>
+            <v>-5.7059328359795654</v>
           </cell>
           <cell r="BR5">
-            <v>-1.6513493411040914</v>
+            <v>-5.7561970177342321</v>
           </cell>
           <cell r="BS5">
-            <v>-1.6547799298626154</v>
+            <v>-5.8050176666765152</v>
           </cell>
           <cell r="BT5">
-            <v>-1.6588215817661012</v>
+            <v>-5.8527213604684825</v>
           </cell>
           <cell r="BU5">
-            <v>-1.663474348417826</v>
+            <v>-5.8995375439617082</v>
           </cell>
           <cell r="BV5">
-            <v>-1.668749189340446</v>
+            <v>-5.9431609779408863</v>
           </cell>
           <cell r="BW5">
-            <v>-1.6745957993986593</v>
+            <v>-5.9855825034606625</v>
           </cell>
           <cell r="BX5">
-            <v>-1.6809976191283882</v>
+            <v>-6.026967531817462</v>
           </cell>
           <cell r="BY5">
-            <v>-1.6879396819433956</v>
+            <v>-6.0674985976995055</v>
           </cell>
           <cell r="BZ5">
-            <v>-1.6954091313694963</v>
+            <v>-6.1073155763356919</v>
           </cell>
           <cell r="CA5">
-            <v>-1.7043809443399893</v>
+            <v>-6.142432726395997</v>
           </cell>
           <cell r="CB5">
-            <v>-1.7136818328981618</v>
+            <v>-6.1757107375436604</v>
           </cell>
           <cell r="CC5">
-            <v>-1.7233900154516202</v>
+            <v>-6.2074651022600573</v>
           </cell>
           <cell r="CD5">
-            <v>-1.733529893763619</v>
+            <v>-6.2380089345567491</v>
           </cell>
           <cell r="CE5">
-            <v>-1.7441041249341871</v>
+            <v>-6.267569340326407</v>
           </cell>
           <cell r="CF5">
-            <v>-1.7551879809414861</v>
+            <v>-6.2956097179621473</v>
           </cell>
           <cell r="CG5">
-            <v>-1.7666911636200933</v>
+            <v>-6.3228054306053716</v>
           </cell>
           <cell r="CH5">
-            <v>-1.7709894968797713</v>
+            <v>-6.3492498871058123</v>
           </cell>
           <cell r="CI5">
-            <v>-1.7897149040786542</v>
+            <v>-6.3750187961419176</v>
           </cell>
           <cell r="CJ5">
-            <v>-1.3563380790536539</v>
+            <v>-9.2488478004404406</v>
           </cell>
         </row>
       </sheetData>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="16" refreshError="1"/>
+      <sheetData sheetId="17" refreshError="1"/>
+      <sheetData sheetId="18" refreshError="1"/>
+      <sheetData sheetId="19" refreshError="1"/>
+      <sheetData sheetId="20" refreshError="1"/>
+      <sheetData sheetId="21" refreshError="1"/>
+      <sheetData sheetId="22" refreshError="1"/>
+      <sheetData sheetId="23" refreshError="1"/>
+      <sheetData sheetId="24" refreshError="1"/>
+      <sheetData sheetId="25" refreshError="1"/>
+      <sheetData sheetId="26" refreshError="1"/>
+      <sheetData sheetId="27" refreshError="1"/>
+      <sheetData sheetId="28" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3049,524 +3337,264 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0">
-        <row r="4">
-          <cell r="C4">
-            <v>42005</v>
-          </cell>
-          <cell r="D4">
-            <v>42370</v>
-          </cell>
-          <cell r="E4">
-            <v>42736</v>
-          </cell>
-          <cell r="F4">
-            <v>43101</v>
-          </cell>
-          <cell r="G4">
-            <v>43466</v>
-          </cell>
-          <cell r="H4">
-            <v>43831</v>
-          </cell>
-          <cell r="I4">
-            <v>44197</v>
-          </cell>
-          <cell r="J4">
-            <v>44562</v>
-          </cell>
-          <cell r="K4">
-            <v>44927</v>
-          </cell>
-          <cell r="L4">
-            <v>45292</v>
-          </cell>
-          <cell r="M4">
-            <v>45658</v>
-          </cell>
-          <cell r="N4">
-            <v>46023</v>
-          </cell>
-          <cell r="O4">
-            <v>46388</v>
-          </cell>
-          <cell r="P4">
-            <v>46753</v>
-          </cell>
-          <cell r="Q4">
-            <v>47119</v>
-          </cell>
-          <cell r="R4">
-            <v>47484</v>
-          </cell>
-          <cell r="S4">
-            <v>47849</v>
-          </cell>
-          <cell r="T4">
-            <v>48214</v>
-          </cell>
-          <cell r="U4">
-            <v>48580</v>
-          </cell>
-          <cell r="V4">
-            <v>48945</v>
-          </cell>
-          <cell r="W4">
-            <v>49310</v>
-          </cell>
-          <cell r="X4">
-            <v>49675</v>
-          </cell>
-          <cell r="Y4">
-            <v>50041</v>
-          </cell>
-          <cell r="Z4">
-            <v>50406</v>
-          </cell>
-          <cell r="AA4">
-            <v>50771</v>
-          </cell>
-          <cell r="AB4">
-            <v>51136</v>
-          </cell>
-          <cell r="AC4">
-            <v>51502</v>
-          </cell>
-          <cell r="AD4">
-            <v>51867</v>
-          </cell>
-          <cell r="AE4">
-            <v>52232</v>
-          </cell>
-          <cell r="AF4">
-            <v>52597</v>
-          </cell>
-          <cell r="AG4">
-            <v>52963</v>
-          </cell>
-          <cell r="AH4">
-            <v>53328</v>
-          </cell>
-          <cell r="AI4">
-            <v>53693</v>
-          </cell>
-          <cell r="AJ4">
-            <v>54058</v>
-          </cell>
-          <cell r="AK4">
-            <v>54424</v>
-          </cell>
-          <cell r="AL4">
-            <v>54789</v>
-          </cell>
-          <cell r="AM4">
-            <v>55154</v>
-          </cell>
-          <cell r="AN4">
-            <v>55519</v>
-          </cell>
-          <cell r="AO4">
-            <v>55885</v>
-          </cell>
-          <cell r="AP4">
-            <v>56250</v>
-          </cell>
-          <cell r="AQ4">
-            <v>56615</v>
-          </cell>
-          <cell r="AR4">
-            <v>56980</v>
-          </cell>
-          <cell r="AS4">
-            <v>57346</v>
-          </cell>
-          <cell r="AT4">
-            <v>57711</v>
-          </cell>
-          <cell r="AU4">
-            <v>58076</v>
-          </cell>
-          <cell r="AV4">
-            <v>58441</v>
-          </cell>
-          <cell r="AW4">
-            <v>58807</v>
-          </cell>
-          <cell r="AX4">
-            <v>59172</v>
-          </cell>
-          <cell r="AY4">
-            <v>59537</v>
-          </cell>
-          <cell r="AZ4">
-            <v>59902</v>
-          </cell>
-          <cell r="BA4">
-            <v>60268</v>
-          </cell>
-          <cell r="BB4">
-            <v>60633</v>
-          </cell>
-          <cell r="BC4">
-            <v>60998</v>
-          </cell>
-          <cell r="BD4">
-            <v>61363</v>
-          </cell>
-          <cell r="BE4">
-            <v>61729</v>
-          </cell>
-          <cell r="BF4">
-            <v>62094</v>
-          </cell>
-          <cell r="BG4">
-            <v>62459</v>
-          </cell>
-          <cell r="BH4">
-            <v>62824</v>
-          </cell>
-          <cell r="BI4">
-            <v>63190</v>
-          </cell>
-          <cell r="BJ4">
-            <v>63555</v>
-          </cell>
-          <cell r="BK4">
-            <v>63920</v>
-          </cell>
-          <cell r="BL4">
-            <v>64285</v>
-          </cell>
-          <cell r="BM4">
-            <v>64651</v>
-          </cell>
-          <cell r="BN4">
-            <v>65016</v>
-          </cell>
-          <cell r="BO4">
-            <v>65381</v>
-          </cell>
-          <cell r="BP4">
-            <v>65746</v>
-          </cell>
-          <cell r="BQ4">
-            <v>66112</v>
-          </cell>
-          <cell r="BR4">
-            <v>66477</v>
-          </cell>
-          <cell r="BS4">
-            <v>66842</v>
-          </cell>
-          <cell r="BT4">
-            <v>67207</v>
-          </cell>
-          <cell r="BU4">
-            <v>67573</v>
-          </cell>
-          <cell r="BV4">
-            <v>67938</v>
-          </cell>
-          <cell r="BW4">
-            <v>68303</v>
-          </cell>
-          <cell r="BX4">
-            <v>68668</v>
-          </cell>
-          <cell r="BY4">
-            <v>69034</v>
-          </cell>
-          <cell r="BZ4">
-            <v>69399</v>
-          </cell>
-          <cell r="CA4">
-            <v>69764</v>
-          </cell>
-          <cell r="CB4">
-            <v>70129</v>
-          </cell>
-          <cell r="CC4">
-            <v>70495</v>
-          </cell>
-          <cell r="CD4">
-            <v>70860</v>
-          </cell>
-          <cell r="CE4">
-            <v>71225</v>
-          </cell>
-          <cell r="CF4">
-            <v>71590</v>
-          </cell>
-          <cell r="CG4">
-            <v>71956</v>
-          </cell>
-          <cell r="CH4">
-            <v>72321</v>
-          </cell>
-          <cell r="CI4">
-            <v>72686</v>
-          </cell>
-          <cell r="CJ4">
-            <v>73051</v>
-          </cell>
-        </row>
         <row r="5">
           <cell r="C5">
             <v>0</v>
           </cell>
           <cell r="D5">
-            <v>9.1492751157495888E-4</v>
+            <v>0</v>
           </cell>
           <cell r="E5">
-            <v>1.9380107544986203E-3</v>
+            <v>0</v>
           </cell>
           <cell r="F5">
-            <v>3.0370170623905679E-3</v>
+            <v>0</v>
           </cell>
           <cell r="G5">
-            <v>4.1803820710395456E-3</v>
+            <v>0</v>
           </cell>
           <cell r="H5">
-            <v>5.3381698501331343E-3</v>
+            <v>0</v>
           </cell>
           <cell r="I5">
-            <v>1.3157759753057441E-2</v>
+            <v>0</v>
           </cell>
           <cell r="J5">
-            <v>0.21348505364844339</v>
+            <v>-8.2056637038441238E-2</v>
           </cell>
           <cell r="K5">
-            <v>0.34910430938315251</v>
+            <v>-0.21283364242431491</v>
           </cell>
           <cell r="L5">
-            <v>0.10772874383697673</v>
+            <v>-0.39025278208807412</v>
           </cell>
           <cell r="M5">
-            <v>-0.16705601577994278</v>
+            <v>-0.59628327178540275</v>
           </cell>
           <cell r="N5">
-            <v>-0.43465890355091075</v>
+            <v>-0.81562590353156939</v>
           </cell>
           <cell r="O5">
-            <v>-0.66159570791660682</v>
+            <v>-1.0216278909715992</v>
           </cell>
           <cell r="P5">
-            <v>-0.86101032056353777</v>
+            <v>-1.2032345153876411</v>
           </cell>
           <cell r="Q5">
-            <v>-1.0515687464137558</v>
+            <v>-1.3504639790627215</v>
           </cell>
           <cell r="R5">
-            <v>-1.2311097309259722</v>
+            <v>-1.4585944232260228</v>
           </cell>
           <cell r="S5">
-            <v>-1.4228025754553508</v>
+            <v>-1.5517555857743948</v>
           </cell>
           <cell r="T5">
-            <v>-1.5742008267198959</v>
+            <v>-1.5951026922136013</v>
           </cell>
           <cell r="U5">
-            <v>-1.6992195584478065</v>
+            <v>-1.6040668534222591</v>
           </cell>
           <cell r="V5">
-            <v>-1.8105357584278448</v>
+            <v>-1.5931250202945058</v>
           </cell>
           <cell r="W5">
-            <v>-1.9158446646005745</v>
+            <v>-1.5713350192618547</v>
           </cell>
           <cell r="X5">
-            <v>-2.0422926708964284</v>
+            <v>-1.5651218195565586</v>
           </cell>
           <cell r="Y5">
-            <v>-2.1692700651057328</v>
+            <v>-1.554404043652069</v>
           </cell>
           <cell r="Z5">
-            <v>-2.2955382898167564</v>
+            <v>-1.5381127661592275</v>
           </cell>
           <cell r="AA5">
-            <v>-2.4194852035804293</v>
+            <v>-1.5150887663259005</v>
           </cell>
           <cell r="AB5">
-            <v>-2.5396476528848577</v>
+            <v>-1.4843693729708951</v>
           </cell>
           <cell r="AC5">
-            <v>-2.661324458444736</v>
+            <v>-1.4670959735900491</v>
           </cell>
           <cell r="AD5">
-            <v>-2.7771446690231461</v>
+            <v>-1.4415172238670282</v>
           </cell>
           <cell r="AE5">
-            <v>-2.8883528079100107</v>
+            <v>-1.4083443590699352</v>
           </cell>
           <cell r="AF5">
-            <v>-2.9969917621188835</v>
+            <v>-1.369330271902458</v>
           </cell>
           <cell r="AG5">
-            <v>-3.1045562489061651</v>
+            <v>-1.3259532326168944</v>
           </cell>
           <cell r="AH5">
-            <v>-3.2169190300692652</v>
+            <v>-1.3024859273049971</v>
           </cell>
           <cell r="AI5">
-            <v>-3.3296402639445777</v>
+            <v>-1.2777267899411027</v>
           </cell>
           <cell r="AJ5">
-            <v>-3.4444508403099983</v>
+            <v>-1.2527233993570031</v>
           </cell>
           <cell r="AK5">
-            <v>-3.5647533183807201</v>
+            <v>-1.2304848598072127</v>
           </cell>
           <cell r="AL5">
-            <v>-3.6969161347232715</v>
+            <v>-1.2174546113713047</v>
           </cell>
           <cell r="AM5">
-            <v>-3.8217313853343149</v>
+            <v>-1.237908577251623</v>
           </cell>
           <cell r="AN5">
-            <v>-3.9448919323131437</v>
+            <v>-1.2603538312162543</v>
           </cell>
           <cell r="AO5">
-            <v>-4.0639667698810111</v>
+            <v>-1.280896991656888</v>
           </cell>
           <cell r="AP5">
-            <v>-4.1779892250678348</v>
+            <v>-1.297188457191123</v>
           </cell>
           <cell r="AQ5">
-            <v>-4.2867387241266375</v>
+            <v>-1.3082209222382457</v>
           </cell>
           <cell r="AR5">
-            <v>-4.390502402670271</v>
+            <v>-1.3141866871164254</v>
           </cell>
           <cell r="AS5">
-            <v>-4.4892722927368904</v>
+            <v>-1.3148074597939763</v>
           </cell>
           <cell r="AT5">
-            <v>-4.5838049366044631</v>
+            <v>-1.3108556960684137</v>
           </cell>
           <cell r="AU5">
-            <v>-4.6750075756943232</v>
+            <v>-1.303275763656131</v>
           </cell>
           <cell r="AV5">
-            <v>-4.7638116158136619</v>
+            <v>-1.2930319435366266</v>
           </cell>
           <cell r="AW5">
-            <v>-4.846398105559679</v>
+            <v>-1.281342220396231</v>
           </cell>
           <cell r="AX5">
-            <v>-4.9270733084887386</v>
+            <v>-1.2684877326585298</v>
           </cell>
           <cell r="AY5">
-            <v>-5.0064980472733112</v>
+            <v>-1.2549757446242316</v>
           </cell>
           <cell r="AZ5">
-            <v>-5.0852468488815639</v>
+            <v>-1.2411581680791373</v>
           </cell>
           <cell r="BA5">
-            <v>-5.1637059738566133</v>
+            <v>-1.2272642485102625</v>
           </cell>
           <cell r="BB5">
-            <v>-5.2500419439234447</v>
+            <v>-1.2242065628020882</v>
           </cell>
           <cell r="BC5">
-            <v>-5.3254923794368807</v>
+            <v>-1.212274094328003</v>
           </cell>
           <cell r="BD5">
-            <v>-5.397441557757543</v>
+            <v>-1.1969362266087136</v>
           </cell>
           <cell r="BE5">
-            <v>-5.468206895285399</v>
+            <v>-1.18070260801586</v>
           </cell>
           <cell r="BF5">
-            <v>-5.538953308007299</v>
+            <v>-1.16492077109287</v>
           </cell>
           <cell r="BG5">
-            <v>-5.6100666583201564</v>
+            <v>-1.1511401161751533</v>
           </cell>
           <cell r="BH5">
-            <v>-5.6811461839669679</v>
+            <v>-1.1378958971931308</v>
           </cell>
           <cell r="BI5">
-            <v>-5.7521787639958966</v>
+            <v>-1.1250898290850242</v>
           </cell>
           <cell r="BJ5">
-            <v>-5.8230693764018344</v>
+            <v>-1.1125532871455235</v>
           </cell>
           <cell r="BK5">
-            <v>-5.8937551804897019</v>
+            <v>-1.1001719824118905</v>
           </cell>
           <cell r="BL5">
-            <v>-5.9627310400813149</v>
+            <v>-1.0878917622401674</v>
           </cell>
           <cell r="BM5">
-            <v>-6.0312211491092116</v>
+            <v>-1.0757687980817221</v>
           </cell>
           <cell r="BN5">
-            <v>-6.0993719673605673</v>
+            <v>-1.063870997528682</v>
           </cell>
           <cell r="BO5">
-            <v>-6.1673530177726921</v>
+            <v>-1.0522736454812165</v>
           </cell>
           <cell r="BP5">
-            <v>-6.2352915712644119</v>
+            <v>-1.0410385324777782</v>
           </cell>
           <cell r="BQ5">
-            <v>-6.2985615324749666</v>
+            <v>-1.0312423250512404</v>
           </cell>
           <cell r="BR5">
-            <v>-6.3604577669279738</v>
+            <v>-1.0214957006012715</v>
           </cell>
           <cell r="BS5">
-            <v>-6.4213119370468359</v>
+            <v>-1.0118976129306012</v>
           </cell>
           <cell r="BT5">
-            <v>-6.4814497093279027</v>
+            <v>-1.0024819779150707</v>
           </cell>
           <cell r="BU5">
-            <v>-6.5411000815981835</v>
+            <v>-0.99324739033723741</v>
           </cell>
           <cell r="BV5">
-            <v>-6.597973463650475</v>
+            <v>-0.98420512175648733</v>
           </cell>
           <cell r="BW5">
-            <v>-6.6540575869920682</v>
+            <v>-0.97529371947724375</v>
           </cell>
           <cell r="BX5">
-            <v>-6.7095267408472932</v>
+            <v>-0.96648595744011079</v>
           </cell>
           <cell r="BY5">
-            <v>-6.7645730315837538</v>
+            <v>-0.9577552203525963</v>
           </cell>
           <cell r="BZ5">
-            <v>-6.8193461873122807</v>
+            <v>-0.94907697959949466</v>
           </cell>
           <cell r="CA5">
-            <v>-6.8700194906914147</v>
+            <v>-0.94129484741348746</v>
           </cell>
           <cell r="CB5">
-            <v>-6.9194266938419453</v>
+            <v>-0.93323535150678927</v>
           </cell>
           <cell r="CC5">
-            <v>-6.9678909725079947</v>
+            <v>-0.9249666077962293</v>
           </cell>
           <cell r="CD5">
-            <v>-7.0157234307819056</v>
+            <v>-0.91651274199079369</v>
           </cell>
           <cell r="CE5">
-            <v>-7.063148609647496</v>
+            <v>-0.90787715348179532</v>
           </cell>
           <cell r="CF5">
-            <v>-7.109622597534071</v>
+            <v>-0.89914837199471798</v>
           </cell>
           <cell r="CG5">
-            <v>-7.1558280095632254</v>
+            <v>-0.8902214872785974</v>
           </cell>
           <cell r="CH5">
-            <v>-7.1946536881305363</v>
+            <v>-0.88109715314373949</v>
           </cell>
           <cell r="CI5">
-            <v>-7.2466119899013197</v>
+            <v>-0.87177687957782357</v>
           </cell>
           <cell r="CJ5">
-            <v>-6.8712948072433004</v>
+            <v>-9.2488478004404406</v>
           </cell>
         </row>
       </sheetData>
@@ -3905,347 +3933,347 @@
   <sheetData>
     <row r="1" spans="1:87" x14ac:dyDescent="0.3">
       <c r="B1" s="1">
-        <f>[2]Données!C4</f>
+        <f>[1]Données!C4</f>
         <v>42005</v>
       </c>
       <c r="C1" s="1">
-        <f>[2]Données!D4</f>
+        <f>[1]Données!D4</f>
         <v>42370</v>
       </c>
       <c r="D1" s="1">
-        <f>[2]Données!E4</f>
+        <f>[1]Données!E4</f>
         <v>42736</v>
       </c>
       <c r="E1" s="1">
-        <f>[2]Données!F4</f>
+        <f>[1]Données!F4</f>
         <v>43101</v>
       </c>
       <c r="F1" s="1">
-        <f>[2]Données!G4</f>
+        <f>[1]Données!G4</f>
         <v>43466</v>
       </c>
       <c r="G1" s="1">
-        <f>[2]Données!H4</f>
+        <f>[1]Données!H4</f>
         <v>43831</v>
       </c>
       <c r="H1" s="1">
-        <f>[2]Données!I4</f>
+        <f>[1]Données!I4</f>
         <v>44197</v>
       </c>
       <c r="I1" s="1">
-        <f>[2]Données!J4</f>
+        <f>[1]Données!J4</f>
         <v>44562</v>
       </c>
       <c r="J1" s="1">
-        <f>[2]Données!K4</f>
+        <f>[1]Données!K4</f>
         <v>44927</v>
       </c>
       <c r="K1" s="1">
-        <f>[2]Données!L4</f>
+        <f>[1]Données!L4</f>
         <v>45292</v>
       </c>
       <c r="L1" s="1">
-        <f>[2]Données!M4</f>
+        <f>[1]Données!M4</f>
         <v>45658</v>
       </c>
       <c r="M1" s="1">
-        <f>[2]Données!N4</f>
+        <f>[1]Données!N4</f>
         <v>46023</v>
       </c>
       <c r="N1" s="1">
-        <f>[2]Données!O4</f>
+        <f>[1]Données!O4</f>
         <v>46388</v>
       </c>
       <c r="O1" s="1">
-        <f>[2]Données!P4</f>
+        <f>[1]Données!P4</f>
         <v>46753</v>
       </c>
       <c r="P1" s="1">
-        <f>[2]Données!Q4</f>
+        <f>[1]Données!Q4</f>
         <v>47119</v>
       </c>
       <c r="Q1" s="1">
-        <f>[2]Données!R4</f>
+        <f>[1]Données!R4</f>
         <v>47484</v>
       </c>
       <c r="R1" s="1">
-        <f>[2]Données!S4</f>
+        <f>[1]Données!S4</f>
         <v>47849</v>
       </c>
       <c r="S1" s="1">
-        <f>[2]Données!T4</f>
+        <f>[1]Données!T4</f>
         <v>48214</v>
       </c>
       <c r="T1" s="1">
-        <f>[2]Données!U4</f>
+        <f>[1]Données!U4</f>
         <v>48580</v>
       </c>
       <c r="U1" s="1">
-        <f>[2]Données!V4</f>
+        <f>[1]Données!V4</f>
         <v>48945</v>
       </c>
       <c r="V1" s="1">
-        <f>[2]Données!W4</f>
+        <f>[1]Données!W4</f>
         <v>49310</v>
       </c>
       <c r="W1" s="1">
-        <f>[2]Données!X4</f>
+        <f>[1]Données!X4</f>
         <v>49675</v>
       </c>
       <c r="X1" s="1">
-        <f>[2]Données!Y4</f>
+        <f>[1]Données!Y4</f>
         <v>50041</v>
       </c>
       <c r="Y1" s="1">
-        <f>[2]Données!Z4</f>
+        <f>[1]Données!Z4</f>
         <v>50406</v>
       </c>
       <c r="Z1" s="1">
-        <f>[2]Données!AA4</f>
+        <f>[1]Données!AA4</f>
         <v>50771</v>
       </c>
       <c r="AA1" s="1">
-        <f>[2]Données!AB4</f>
+        <f>[1]Données!AB4</f>
         <v>51136</v>
       </c>
       <c r="AB1" s="1">
-        <f>[2]Données!AC4</f>
+        <f>[1]Données!AC4</f>
         <v>51502</v>
       </c>
       <c r="AC1" s="1">
-        <f>[2]Données!AD4</f>
+        <f>[1]Données!AD4</f>
         <v>51867</v>
       </c>
       <c r="AD1" s="1">
-        <f>[2]Données!AE4</f>
+        <f>[1]Données!AE4</f>
         <v>52232</v>
       </c>
       <c r="AE1" s="1">
-        <f>[2]Données!AF4</f>
+        <f>[1]Données!AF4</f>
         <v>52597</v>
       </c>
       <c r="AF1" s="1">
-        <f>[2]Données!AG4</f>
+        <f>[1]Données!AG4</f>
         <v>52963</v>
       </c>
       <c r="AG1" s="1">
-        <f>[2]Données!AH4</f>
+        <f>[1]Données!AH4</f>
         <v>53328</v>
       </c>
       <c r="AH1" s="1">
-        <f>[2]Données!AI4</f>
+        <f>[1]Données!AI4</f>
         <v>53693</v>
       </c>
       <c r="AI1" s="1">
-        <f>[2]Données!AJ4</f>
+        <f>[1]Données!AJ4</f>
         <v>54058</v>
       </c>
       <c r="AJ1" s="1">
-        <f>[2]Données!AK4</f>
+        <f>[1]Données!AK4</f>
         <v>54424</v>
       </c>
       <c r="AK1" s="1">
-        <f>[2]Données!AL4</f>
+        <f>[1]Données!AL4</f>
         <v>54789</v>
       </c>
       <c r="AL1" s="1">
-        <f>[2]Données!AM4</f>
+        <f>[1]Données!AM4</f>
         <v>55154</v>
       </c>
       <c r="AM1" s="1">
-        <f>[2]Données!AN4</f>
+        <f>[1]Données!AN4</f>
         <v>55519</v>
       </c>
       <c r="AN1" s="1">
-        <f>[2]Données!AO4</f>
+        <f>[1]Données!AO4</f>
         <v>55885</v>
       </c>
       <c r="AO1" s="1">
-        <f>[2]Données!AP4</f>
+        <f>[1]Données!AP4</f>
         <v>56250</v>
       </c>
       <c r="AP1" s="1">
-        <f>[2]Données!AQ4</f>
+        <f>[1]Données!AQ4</f>
         <v>56615</v>
       </c>
       <c r="AQ1" s="1">
-        <f>[2]Données!AR4</f>
+        <f>[1]Données!AR4</f>
         <v>56980</v>
       </c>
       <c r="AR1" s="1">
-        <f>[2]Données!AS4</f>
+        <f>[1]Données!AS4</f>
         <v>57346</v>
       </c>
       <c r="AS1" s="1">
-        <f>[2]Données!AT4</f>
+        <f>[1]Données!AT4</f>
         <v>57711</v>
       </c>
       <c r="AT1" s="1">
-        <f>[2]Données!AU4</f>
+        <f>[1]Données!AU4</f>
         <v>58076</v>
       </c>
       <c r="AU1" s="1">
-        <f>[2]Données!AV4</f>
+        <f>[1]Données!AV4</f>
         <v>58441</v>
       </c>
       <c r="AV1" s="1">
-        <f>[2]Données!AW4</f>
+        <f>[1]Données!AW4</f>
         <v>58807</v>
       </c>
       <c r="AW1" s="1">
-        <f>[2]Données!AX4</f>
+        <f>[1]Données!AX4</f>
         <v>59172</v>
       </c>
       <c r="AX1" s="1">
-        <f>[2]Données!AY4</f>
+        <f>[1]Données!AY4</f>
         <v>59537</v>
       </c>
       <c r="AY1" s="1">
-        <f>[2]Données!AZ4</f>
+        <f>[1]Données!AZ4</f>
         <v>59902</v>
       </c>
       <c r="AZ1" s="1">
-        <f>[2]Données!BA4</f>
+        <f>[1]Données!BA4</f>
         <v>60268</v>
       </c>
       <c r="BA1" s="1">
-        <f>[2]Données!BB4</f>
+        <f>[1]Données!BB4</f>
         <v>60633</v>
       </c>
       <c r="BB1" s="1">
-        <f>[2]Données!BC4</f>
+        <f>[1]Données!BC4</f>
         <v>60998</v>
       </c>
       <c r="BC1" s="1">
-        <f>[2]Données!BD4</f>
+        <f>[1]Données!BD4</f>
         <v>61363</v>
       </c>
       <c r="BD1" s="1">
-        <f>[2]Données!BE4</f>
+        <f>[1]Données!BE4</f>
         <v>61729</v>
       </c>
       <c r="BE1" s="1">
-        <f>[2]Données!BF4</f>
+        <f>[1]Données!BF4</f>
         <v>62094</v>
       </c>
       <c r="BF1" s="1">
-        <f>[2]Données!BG4</f>
+        <f>[1]Données!BG4</f>
         <v>62459</v>
       </c>
       <c r="BG1" s="1">
-        <f>[2]Données!BH4</f>
+        <f>[1]Données!BH4</f>
         <v>62824</v>
       </c>
       <c r="BH1" s="1">
-        <f>[2]Données!BI4</f>
+        <f>[1]Données!BI4</f>
         <v>63190</v>
       </c>
       <c r="BI1" s="1">
-        <f>[2]Données!BJ4</f>
+        <f>[1]Données!BJ4</f>
         <v>63555</v>
       </c>
       <c r="BJ1" s="1">
-        <f>[2]Données!BK4</f>
+        <f>[1]Données!BK4</f>
         <v>63920</v>
       </c>
       <c r="BK1" s="1">
-        <f>[2]Données!BL4</f>
+        <f>[1]Données!BL4</f>
         <v>64285</v>
       </c>
       <c r="BL1" s="1">
-        <f>[2]Données!BM4</f>
+        <f>[1]Données!BM4</f>
         <v>64651</v>
       </c>
       <c r="BM1" s="1">
-        <f>[2]Données!BN4</f>
+        <f>[1]Données!BN4</f>
         <v>65016</v>
       </c>
       <c r="BN1" s="1">
-        <f>[2]Données!BO4</f>
+        <f>[1]Données!BO4</f>
         <v>65381</v>
       </c>
       <c r="BO1" s="1">
-        <f>[2]Données!BP4</f>
+        <f>[1]Données!BP4</f>
         <v>65746</v>
       </c>
       <c r="BP1" s="1">
-        <f>[2]Données!BQ4</f>
+        <f>[1]Données!BQ4</f>
         <v>66112</v>
       </c>
       <c r="BQ1" s="1">
-        <f>[2]Données!BR4</f>
+        <f>[1]Données!BR4</f>
         <v>66477</v>
       </c>
       <c r="BR1" s="1">
-        <f>[2]Données!BS4</f>
+        <f>[1]Données!BS4</f>
         <v>66842</v>
       </c>
       <c r="BS1" s="1">
-        <f>[2]Données!BT4</f>
+        <f>[1]Données!BT4</f>
         <v>67207</v>
       </c>
       <c r="BT1" s="1">
-        <f>[2]Données!BU4</f>
+        <f>[1]Données!BU4</f>
         <v>67573</v>
       </c>
       <c r="BU1" s="1">
-        <f>[2]Données!BV4</f>
+        <f>[1]Données!BV4</f>
         <v>67938</v>
       </c>
       <c r="BV1" s="1">
-        <f>[2]Données!BW4</f>
+        <f>[1]Données!BW4</f>
         <v>68303</v>
       </c>
       <c r="BW1" s="1">
-        <f>[2]Données!BX4</f>
+        <f>[1]Données!BX4</f>
         <v>68668</v>
       </c>
       <c r="BX1" s="1">
-        <f>[2]Données!BY4</f>
+        <f>[1]Données!BY4</f>
         <v>69034</v>
       </c>
       <c r="BY1" s="1">
-        <f>[2]Données!BZ4</f>
+        <f>[1]Données!BZ4</f>
         <v>69399</v>
       </c>
       <c r="BZ1" s="1">
-        <f>[2]Données!CA4</f>
+        <f>[1]Données!CA4</f>
         <v>69764</v>
       </c>
       <c r="CA1" s="1">
-        <f>[2]Données!CB4</f>
+        <f>[1]Données!CB4</f>
         <v>70129</v>
       </c>
       <c r="CB1" s="1">
-        <f>[2]Données!CC4</f>
+        <f>[1]Données!CC4</f>
         <v>70495</v>
       </c>
       <c r="CC1" s="1">
-        <f>[2]Données!CD4</f>
+        <f>[1]Données!CD4</f>
         <v>70860</v>
       </c>
       <c r="CD1" s="1">
-        <f>[2]Données!CE4</f>
+        <f>[1]Données!CE4</f>
         <v>71225</v>
       </c>
       <c r="CE1" s="1">
-        <f>[2]Données!CF4</f>
+        <f>[1]Données!CF4</f>
         <v>71590</v>
       </c>
       <c r="CF1" s="1">
-        <f>[2]Données!CG4</f>
+        <f>[1]Données!CG4</f>
         <v>71956</v>
       </c>
       <c r="CG1" s="1">
-        <f>[2]Données!CH4</f>
+        <f>[1]Données!CH4</f>
         <v>72321</v>
       </c>
       <c r="CH1" s="1">
-        <f>[2]Données!CI4</f>
+        <f>[1]Données!CI4</f>
         <v>72686</v>
       </c>
       <c r="CI1" s="1">
-        <f>[2]Données!CJ4</f>
+        <f>[1]Données!CJ4</f>
         <v>73051</v>
       </c>
     </row>
@@ -4254,348 +4282,348 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <f>[1]Données!C5</f>
+        <f>[2]Données!C5</f>
         <v>0</v>
       </c>
       <c r="C2" s="2">
-        <f>[1]Données!D5</f>
+        <f>[2]Données!D5</f>
         <v>0</v>
       </c>
       <c r="D2" s="2">
-        <f>[1]Données!E5</f>
+        <f>[2]Données!E5</f>
         <v>0</v>
       </c>
       <c r="E2" s="2">
-        <f>[1]Données!F5</f>
+        <f>[2]Données!F5</f>
         <v>0</v>
       </c>
       <c r="F2" s="2">
-        <f>[1]Données!G5</f>
+        <f>[2]Données!G5</f>
         <v>0</v>
       </c>
       <c r="G2" s="2">
-        <f>[1]Données!H5</f>
+        <f>[2]Données!H5</f>
         <v>0</v>
       </c>
       <c r="H2" s="2">
-        <f>[1]Données!I5</f>
+        <f>[2]Données!I5</f>
         <v>0</v>
       </c>
       <c r="I2" s="2">
-        <f>[1]Données!J5</f>
-        <v>0.19161550315185405</v>
+        <f>[2]Données!J5</f>
+        <v>-8.2056637038441238E-2</v>
       </c>
       <c r="J2" s="2">
-        <f>[1]Données!K5</f>
-        <v>0.31789887951911844</v>
+        <f>[2]Données!K5</f>
+        <v>-0.21283364242431491</v>
       </c>
       <c r="K2" s="2">
-        <f>[1]Données!L5</f>
-        <v>6.7015030786099494E-2</v>
+        <f>[2]Données!L5</f>
+        <v>-0.39025278208807412</v>
       </c>
       <c r="L2" s="2">
-        <f>[1]Données!M5</f>
-        <v>-0.21728167797012699</v>
+        <f>[2]Données!M5</f>
+        <v>-0.59628327178540275</v>
       </c>
       <c r="M2" s="2">
-        <f>[1]Données!N5</f>
-        <v>-0.46886133701437016</v>
+        <f>[2]Données!N5</f>
+        <v>-0.81562590353156939</v>
       </c>
       <c r="N2" s="2">
-        <f>[1]Données!O5</f>
-        <v>-0.67638884472317473</v>
+        <f>[2]Données!O5</f>
+        <v>-1.0216278909715992</v>
       </c>
       <c r="O2" s="2">
-        <f>[1]Données!P5</f>
-        <v>-0.85375889954031337</v>
+        <f>[2]Données!P5</f>
+        <v>-1.2032345153876411</v>
       </c>
       <c r="P2" s="2">
-        <f>[1]Données!Q5</f>
-        <v>-1.0207112465597246</v>
+        <f>[2]Données!Q5</f>
+        <v>-1.3504639790627215</v>
       </c>
       <c r="Q2" s="2">
-        <f>[1]Données!R5</f>
-        <v>-1.1759379933896641</v>
+        <f>[2]Données!R5</f>
+        <v>-1.4585944232260228</v>
       </c>
       <c r="R2" s="2">
-        <f>[1]Données!S5</f>
-        <v>-1.307531973432452</v>
+        <f>[2]Données!S5</f>
+        <v>-1.5517555857743948</v>
       </c>
       <c r="S2" s="2">
-        <f>[1]Données!T5</f>
-        <v>-1.3941416492964653</v>
+        <f>[2]Données!T5</f>
+        <v>-1.5951026922136013</v>
       </c>
       <c r="T2" s="2">
-        <f>[1]Données!U5</f>
-        <v>-1.4508647654808193</v>
+        <f>[2]Données!U5</f>
+        <v>-1.6040668534222591</v>
       </c>
       <c r="U2" s="2">
-        <f>[1]Données!V5</f>
-        <v>-1.4919916852337844</v>
+        <f>[2]Données!V5</f>
+        <v>-1.5931250202945058</v>
       </c>
       <c r="V2" s="2">
-        <f>[1]Données!W5</f>
-        <v>-1.5264967867797408</v>
+        <f>[2]Données!W5</f>
+        <v>-1.5713350192618547</v>
       </c>
       <c r="W2" s="2">
-        <f>[1]Données!X5</f>
-        <v>-1.5576296940993828</v>
+        <f>[2]Données!X5</f>
+        <v>-1.5651218195565586</v>
       </c>
       <c r="X2" s="2">
-        <f>[1]Données!Y5</f>
-        <v>-1.5861667841999827</v>
+        <f>[2]Données!Y5</f>
+        <v>-1.554404043652069</v>
       </c>
       <c r="Y2" s="2">
-        <f>[1]Données!Z5</f>
-        <v>-1.6118588854758364</v>
+        <f>[2]Données!Z5</f>
+        <v>-1.5381127661592275</v>
       </c>
       <c r="Z2" s="2">
-        <f>[1]Données!AA5</f>
-        <v>-1.6342925349397075</v>
+        <f>[2]Données!AA5</f>
+        <v>-1.5150887663259005</v>
       </c>
       <c r="AA2" s="2">
-        <f>[1]Données!AB5</f>
-        <v>-1.6529130346936594</v>
+        <f>[2]Données!AB5</f>
+        <v>-1.4843693729708951</v>
       </c>
       <c r="AB2" s="2">
-        <f>[1]Données!AC5</f>
-        <v>-1.6664774336045296</v>
+        <f>[2]Données!AC5</f>
+        <v>-1.4670959735900491</v>
       </c>
       <c r="AC2" s="2">
-        <f>[1]Données!AD5</f>
-        <v>-1.6738659693794067</v>
+        <f>[2]Données!AD5</f>
+        <v>-1.4415172238670282</v>
       </c>
       <c r="AD2" s="2">
-        <f>[1]Données!AE5</f>
-        <v>-1.6767182125922653</v>
+        <f>[2]Données!AE5</f>
+        <v>-1.4083443590699352</v>
       </c>
       <c r="AE2" s="2">
-        <f>[1]Données!AF5</f>
-        <v>-1.677493043235545</v>
+        <f>[2]Données!AF5</f>
+        <v>-1.369330271902458</v>
       </c>
       <c r="AF2" s="2">
-        <f>[1]Données!AG5</f>
-        <v>-1.6779763018033189</v>
+        <f>[2]Données!AG5</f>
+        <v>-1.3259532326168944</v>
       </c>
       <c r="AG2" s="2">
-        <f>[1]Données!AH5</f>
-        <v>-1.6790908599914611</v>
+        <f>[2]Données!AH5</f>
+        <v>-1.3024859273049971</v>
       </c>
       <c r="AH2" s="2">
-        <f>[1]Données!AI5</f>
-        <v>-1.6807531170653367</v>
+        <f>[2]Données!AI5</f>
+        <v>-1.2777267899411027</v>
       </c>
       <c r="AI2" s="2">
-        <f>[1]Données!AJ5</f>
-        <v>-1.6849090679153078</v>
+        <f>[2]Données!AJ5</f>
+        <v>-1.2527233993570031</v>
       </c>
       <c r="AJ2" s="2">
-        <f>[1]Données!AK5</f>
-        <v>-1.6952498621138901</v>
+        <f>[2]Données!AK5</f>
+        <v>-1.2304848598072127</v>
       </c>
       <c r="AK2" s="2">
-        <f>[1]Données!AL5</f>
-        <v>-1.7184393048263136</v>
+        <f>[2]Données!AL5</f>
+        <v>-1.2174546113713047</v>
       </c>
       <c r="AL2" s="2">
-        <f>[1]Données!AM5</f>
-        <v>-1.7362029288578218</v>
+        <f>[2]Données!AM5</f>
+        <v>-1.237908577251623</v>
       </c>
       <c r="AM2" s="2">
-        <f>[1]Données!AN5</f>
-        <v>-1.7534246166071354</v>
+        <f>[2]Données!AN5</f>
+        <v>-1.2603538312162543</v>
       </c>
       <c r="AN2" s="2">
-        <f>[1]Données!AO5</f>
-        <v>-1.7675856069250262</v>
+        <f>[2]Données!AO5</f>
+        <v>-1.280896991656888</v>
       </c>
       <c r="AO2" s="2">
-        <f>[1]Données!AP5</f>
-        <v>-1.7775623333425861</v>
+        <f>[2]Données!AP5</f>
+        <v>-1.297188457191123</v>
       </c>
       <c r="AP2" s="2">
-        <f>[1]Données!AQ5</f>
-        <v>-1.7830030310172607</v>
+        <f>[2]Données!AQ5</f>
+        <v>-1.3082209222382457</v>
       </c>
       <c r="AQ2" s="2">
-        <f>[1]Données!AR5</f>
-        <v>-1.7843857765953541</v>
+        <f>[2]Données!AR5</f>
+        <v>-1.3141866871164254</v>
       </c>
       <c r="AR2" s="2">
-        <f>[1]Données!AS5</f>
-        <v>-1.7814809968153322</v>
+        <f>[2]Données!AS5</f>
+        <v>-1.3148074597939763</v>
       </c>
       <c r="AS2" s="2">
-        <f>[1]Données!AT5</f>
-        <v>-1.7750230330517369</v>
+        <f>[2]Données!AT5</f>
+        <v>-1.3108556960684137</v>
       </c>
       <c r="AT2" s="2">
-        <f>[1]Données!AU5</f>
-        <v>-1.7659091624286583</v>
+        <f>[2]Données!AU5</f>
+        <v>-1.303275763656131</v>
       </c>
       <c r="AU2" s="2">
-        <f>[1]Données!AV5</f>
-        <v>-1.7550687062752313</v>
+        <f>[2]Données!AV5</f>
+        <v>-1.2930319435366266</v>
       </c>
       <c r="AV2" s="2">
-        <f>[1]Données!AW5</f>
-        <v>-1.7437581416538506</v>
+        <f>[2]Données!AW5</f>
+        <v>-1.281342220396231</v>
       </c>
       <c r="AW2" s="2">
-        <f>[1]Données!AX5</f>
-        <v>-1.7322399317636572</v>
+        <f>[2]Données!AX5</f>
+        <v>-1.2684877326585298</v>
       </c>
       <c r="AX2" s="2">
-        <f>[1]Données!AY5</f>
-        <v>-1.7209837178788767</v>
+        <f>[2]Données!AY5</f>
+        <v>-1.2549757446242316</v>
       </c>
       <c r="AY2" s="2">
-        <f>[1]Données!AZ5</f>
-        <v>-1.7102969143967806</v>
+        <f>[2]Données!AZ5</f>
+        <v>-1.2411581680791373</v>
       </c>
       <c r="AZ2" s="2">
-        <f>[1]Données!BA5</f>
-        <v>-1.7003514750675741</v>
+        <f>[2]Données!BA5</f>
+        <v>-1.2272642485102625</v>
       </c>
       <c r="BA2" s="2">
-        <f>[1]Données!BB5</f>
-        <v>-1.7041717945534995</v>
+        <f>[2]Données!BB5</f>
+        <v>-1.2242065628020882</v>
       </c>
       <c r="BB2" s="2">
-        <f>[1]Données!BC5</f>
-        <v>-1.6968611913178111</v>
+        <f>[2]Données!BC5</f>
+        <v>-1.212274094328003</v>
       </c>
       <c r="BC2" s="2">
-        <f>[1]Données!BD5</f>
-        <v>-1.6874204618492761</v>
+        <f>[2]Données!BD5</f>
+        <v>-1.1969362266087136</v>
       </c>
       <c r="BD2" s="2">
-        <f>[1]Données!BE5</f>
-        <v>-1.6779987060296264</v>
+        <f>[2]Données!BE5</f>
+        <v>-1.18070260801586</v>
       </c>
       <c r="BE2" s="2">
-        <f>[1]Données!BF5</f>
-        <v>-1.6695997980133215</v>
+        <f>[2]Données!BF5</f>
+        <v>-1.16492077109287</v>
       </c>
       <c r="BF2" s="2">
-        <f>[1]Données!BG5</f>
-        <v>-1.6637538837163346</v>
+        <f>[2]Données!BG5</f>
+        <v>-1.1511401161751533</v>
       </c>
       <c r="BG2" s="2">
-        <f>[1]Données!BH5</f>
-        <v>-1.6589740264339237</v>
+        <f>[2]Données!BH5</f>
+        <v>-1.1378958971931308</v>
       </c>
       <c r="BH2" s="2">
-        <f>[1]Données!BI5</f>
-        <v>-1.6551568536300354</v>
+        <f>[2]Données!BI5</f>
+        <v>-1.1250898290850242</v>
       </c>
       <c r="BI2" s="2">
-        <f>[1]Données!BJ5</f>
-        <v>-1.6521136575608164</v>
+        <f>[2]Données!BJ5</f>
+        <v>-1.1125532871455235</v>
       </c>
       <c r="BJ2" s="2">
-        <f>[1]Données!BK5</f>
-        <v>-1.6496961346720851</v>
+        <f>[2]Données!BK5</f>
+        <v>-1.1001719824118905</v>
       </c>
       <c r="BK2" s="2">
-        <f>[1]Données!BL5</f>
-        <v>-1.647812183467412</v>
+        <f>[2]Données!BL5</f>
+        <v>-1.0878917622401674</v>
       </c>
       <c r="BL2" s="2">
-        <f>[1]Données!BM5</f>
-        <v>-1.6464745156678506</v>
+        <f>[2]Données!BM5</f>
+        <v>-1.0757687980817221</v>
       </c>
       <c r="BM2" s="2">
-        <f>[1]Données!BN5</f>
-        <v>-1.6457143828054077</v>
+        <f>[2]Données!BN5</f>
+        <v>-1.063870997528682</v>
       </c>
       <c r="BN2" s="2">
-        <f>[1]Données!BO5</f>
-        <v>-1.6455781760776222</v>
+        <f>[2]Données!BO5</f>
+        <v>-1.0522736454812165</v>
       </c>
       <c r="BO2" s="2">
-        <f>[1]Données!BP5</f>
-        <v>-1.6461074372563056</v>
+        <f>[2]Données!BP5</f>
+        <v>-1.0410385324777782</v>
       </c>
       <c r="BP2" s="2">
-        <f>[1]Données!BQ5</f>
-        <v>-1.6484945595247713</v>
+        <f>[2]Données!BQ5</f>
+        <v>-1.0312423250512404</v>
       </c>
       <c r="BQ2" s="2">
-        <f>[1]Données!BR5</f>
-        <v>-1.6513493411040914</v>
+        <f>[2]Données!BR5</f>
+        <v>-1.0214957006012715</v>
       </c>
       <c r="BR2" s="2">
-        <f>[1]Données!BS5</f>
-        <v>-1.6547799298626154</v>
+        <f>[2]Données!BS5</f>
+        <v>-1.0118976129306012</v>
       </c>
       <c r="BS2" s="2">
-        <f>[1]Données!BT5</f>
-        <v>-1.6588215817661012</v>
+        <f>[2]Données!BT5</f>
+        <v>-1.0024819779150707</v>
       </c>
       <c r="BT2" s="2">
-        <f>[1]Données!BU5</f>
-        <v>-1.663474348417826</v>
+        <f>[2]Données!BU5</f>
+        <v>-0.99324739033723741</v>
       </c>
       <c r="BU2" s="2">
-        <f>[1]Données!BV5</f>
-        <v>-1.668749189340446</v>
+        <f>[2]Données!BV5</f>
+        <v>-0.98420512175648733</v>
       </c>
       <c r="BV2" s="2">
-        <f>[1]Données!BW5</f>
-        <v>-1.6745957993986593</v>
+        <f>[2]Données!BW5</f>
+        <v>-0.97529371947724375</v>
       </c>
       <c r="BW2" s="2">
-        <f>[1]Données!BX5</f>
-        <v>-1.6809976191283882</v>
+        <f>[2]Données!BX5</f>
+        <v>-0.96648595744011079</v>
       </c>
       <c r="BX2" s="2">
-        <f>[1]Données!BY5</f>
-        <v>-1.6879396819433956</v>
+        <f>[2]Données!BY5</f>
+        <v>-0.9577552203525963</v>
       </c>
       <c r="BY2" s="2">
-        <f>[1]Données!BZ5</f>
-        <v>-1.6954091313694963</v>
+        <f>[2]Données!BZ5</f>
+        <v>-0.94907697959949466</v>
       </c>
       <c r="BZ2" s="2">
-        <f>[1]Données!CA5</f>
-        <v>-1.7043809443399893</v>
+        <f>[2]Données!CA5</f>
+        <v>-0.94129484741348746</v>
       </c>
       <c r="CA2" s="2">
-        <f>[1]Données!CB5</f>
-        <v>-1.7136818328981618</v>
+        <f>[2]Données!CB5</f>
+        <v>-0.93323535150678927</v>
       </c>
       <c r="CB2" s="2">
-        <f>[1]Données!CC5</f>
-        <v>-1.7233900154516202</v>
+        <f>[2]Données!CC5</f>
+        <v>-0.9249666077962293</v>
       </c>
       <c r="CC2" s="2">
-        <f>[1]Données!CD5</f>
-        <v>-1.733529893763619</v>
+        <f>[2]Données!CD5</f>
+        <v>-0.91651274199079369</v>
       </c>
       <c r="CD2" s="2">
-        <f>[1]Données!CE5</f>
-        <v>-1.7441041249341871</v>
+        <f>[2]Données!CE5</f>
+        <v>-0.90787715348179532</v>
       </c>
       <c r="CE2" s="2">
-        <f>[1]Données!CF5</f>
-        <v>-1.7551879809414861</v>
+        <f>[2]Données!CF5</f>
+        <v>-0.89914837199471798</v>
       </c>
       <c r="CF2" s="2">
-        <f>[1]Données!CG5</f>
-        <v>-1.7666911636200933</v>
+        <f>[2]Données!CG5</f>
+        <v>-0.8902214872785974</v>
       </c>
       <c r="CG2" s="2">
-        <f>[1]Données!CH5</f>
-        <v>-1.7709894968797713</v>
+        <f>[2]Données!CH5</f>
+        <v>-0.88109715314373949</v>
       </c>
       <c r="CH2" s="2">
-        <f>[1]Données!CI5</f>
-        <v>-1.7897149040786542</v>
+        <f>[2]Données!CI5</f>
+        <v>-0.87177687957782357</v>
       </c>
       <c r="CI2" s="2">
-        <f>[1]Données!CJ5</f>
-        <v>-1.3563380790536539</v>
+        <f>[2]Données!CJ5</f>
+        <v>-9.2488478004404406</v>
       </c>
     </row>
     <row r="3" spans="1:87" x14ac:dyDescent="0.3">
@@ -4603,348 +4631,348 @@
         <v>3</v>
       </c>
       <c r="B3" s="2">
-        <f>[2]Données!C5</f>
+        <f>[1]Données!C5</f>
         <v>0</v>
       </c>
       <c r="C3" s="2">
-        <f>[2]Données!D5</f>
+        <f>[1]Données!D5</f>
         <v>9.1492751157495888E-4</v>
       </c>
       <c r="D3" s="2">
-        <f>[2]Données!E5</f>
+        <f>[1]Données!E5</f>
         <v>1.9380107544986203E-3</v>
       </c>
       <c r="E3" s="2">
-        <f>[2]Données!F5</f>
+        <f>[1]Données!F5</f>
         <v>3.0370170623905679E-3</v>
       </c>
       <c r="F3" s="2">
-        <f>[2]Données!G5</f>
+        <f>[1]Données!G5</f>
         <v>4.1803820710395456E-3</v>
       </c>
       <c r="G3" s="2">
-        <f>[2]Données!H5</f>
+        <f>[1]Données!H5</f>
         <v>5.3381698501331343E-3</v>
       </c>
       <c r="H3" s="2">
-        <f>[2]Données!I5</f>
+        <f>[1]Données!I5</f>
         <v>1.3157759753057441E-2</v>
       </c>
       <c r="I3" s="2">
-        <f>[2]Données!J5</f>
-        <v>0.21348505364844339</v>
+        <f>[1]Données!J5</f>
+        <v>-5.9763849015292969E-2</v>
       </c>
       <c r="J3" s="2">
-        <f>[2]Données!K5</f>
-        <v>0.34910430938315251</v>
+        <f>[1]Données!K5</f>
+        <v>-0.18069455425352432</v>
       </c>
       <c r="K3" s="2">
-        <f>[2]Données!L5</f>
-        <v>0.10772874383697673</v>
+        <f>[1]Données!L5</f>
+        <v>-0.34812329689634103</v>
       </c>
       <c r="L3" s="2">
-        <f>[2]Données!M5</f>
-        <v>-0.16705601577994278</v>
+        <f>[1]Données!M5</f>
+        <v>-0.54430802901425102</v>
       </c>
       <c r="M3" s="2">
-        <f>[2]Données!N5</f>
-        <v>-0.43465890355091075</v>
+        <f>[1]Données!N5</f>
+        <v>-0.77960804618192325</v>
       </c>
       <c r="N3" s="2">
-        <f>[2]Données!O5</f>
-        <v>-0.66159570791660682</v>
+        <f>[1]Données!O5</f>
+        <v>-1.0052283935017892</v>
       </c>
       <c r="O3" s="2">
-        <f>[2]Données!P5</f>
-        <v>-0.86101032056353777</v>
+        <f>[1]Données!P5</f>
+        <v>-1.209223737089149</v>
       </c>
       <c r="P3" s="2">
-        <f>[2]Données!Q5</f>
-        <v>-1.0515687464137558</v>
+        <f>[1]Données!Q5</f>
+        <v>-1.3804325254744509</v>
       </c>
       <c r="Q3" s="2">
-        <f>[2]Données!R5</f>
-        <v>-1.2311097309259722</v>
+        <f>[1]Données!R5</f>
+        <v>-1.5131715767560561</v>
       </c>
       <c r="R3" s="2">
-        <f>[2]Données!S5</f>
-        <v>-1.4228025754553508</v>
+        <f>[1]Données!S5</f>
+        <v>-1.6663953530444253</v>
       </c>
       <c r="S3" s="2">
-        <f>[2]Données!T5</f>
-        <v>-1.5742008267198959</v>
+        <f>[1]Données!T5</f>
+        <v>-1.774292780049358</v>
       </c>
       <c r="T3" s="2">
-        <f>[2]Données!U5</f>
-        <v>-1.6992195584478065</v>
+        <f>[1]Données!U5</f>
+        <v>-1.8512001379742182</v>
       </c>
       <c r="U3" s="2">
-        <f>[2]Données!V5</f>
-        <v>-1.8105357584278448</v>
+        <f>[1]Données!V5</f>
+        <v>-1.9100806918052493</v>
       </c>
       <c r="V3" s="2">
-        <f>[2]Données!W5</f>
-        <v>-1.9158446646005745</v>
+        <f>[1]Données!W5</f>
+        <v>-1.9587949690598405</v>
       </c>
       <c r="W3" s="2">
-        <f>[2]Données!X5</f>
-        <v>-2.0422926708964284</v>
+        <f>[1]Données!X5</f>
+        <v>-2.0476288518713637</v>
       </c>
       <c r="X3" s="2">
-        <f>[2]Données!Y5</f>
-        <v>-2.1692700651057328</v>
+        <f>[1]Données!Y5</f>
+        <v>-2.135208763564822</v>
       </c>
       <c r="Y3" s="2">
-        <f>[2]Données!Z5</f>
-        <v>-2.2955382898167564</v>
+        <f>[1]Données!Z5</f>
+        <v>-2.2194985756368357</v>
       </c>
       <c r="Z3" s="2">
-        <f>[2]Données!AA5</f>
-        <v>-2.4194852035804293</v>
+        <f>[1]Données!AA5</f>
+        <v>-2.2981587554657734</v>
       </c>
       <c r="AA3" s="2">
-        <f>[2]Données!AB5</f>
-        <v>-2.5396476528848577</v>
+        <f>[1]Données!AB5</f>
+        <v>-2.3693314690445777</v>
       </c>
       <c r="AB3" s="2">
-        <f>[2]Données!AC5</f>
-        <v>-2.661324458444736</v>
+        <f>[1]Données!AC5</f>
+        <v>-2.4605059364116277</v>
       </c>
       <c r="AC3" s="2">
-        <f>[2]Données!AD5</f>
-        <v>-2.7771446690231461</v>
+        <f>[1]Données!AD5</f>
+        <v>-2.5438088387872426</v>
       </c>
       <c r="AD3" s="2">
-        <f>[2]Données!AE5</f>
-        <v>-2.8883528079100107</v>
+        <f>[1]Données!AE5</f>
+        <v>-2.6195715662762686</v>
       </c>
       <c r="AE3" s="2">
-        <f>[2]Données!AF5</f>
-        <v>-2.9969917621188835</v>
+        <f>[1]Données!AF5</f>
+        <v>-2.6891513395825628</v>
       </c>
       <c r="AF3" s="2">
-        <f>[2]Données!AG5</f>
-        <v>-3.1045562489061651</v>
+        <f>[1]Données!AG5</f>
+        <v>-2.7537508600545269</v>
       </c>
       <c r="AG3" s="2">
-        <f>[2]Données!AH5</f>
-        <v>-3.2169190300692652</v>
+        <f>[1]Données!AH5</f>
+        <v>-2.8422712133339467</v>
       </c>
       <c r="AH3" s="2">
-        <f>[2]Données!AI5</f>
-        <v>-3.3296402639445777</v>
+        <f>[1]Données!AI5</f>
+        <v>-2.9294020392586995</v>
       </c>
       <c r="AI3" s="2">
-        <f>[2]Données!AJ5</f>
-        <v>-3.4444508403099983</v>
+        <f>[1]Données!AJ5</f>
+        <v>-3.0159912948285239</v>
       </c>
       <c r="AJ3" s="2">
-        <f>[2]Données!AK5</f>
-        <v>-3.5647533183807201</v>
+        <f>[1]Données!AK5</f>
+        <v>-3.1047769445148865</v>
       </c>
       <c r="AK3" s="2">
-        <f>[2]Données!AL5</f>
-        <v>-3.6969161347232715</v>
+        <f>[1]Données!AL5</f>
+        <v>-3.2019188432303336</v>
       </c>
       <c r="AL3" s="2">
-        <f>[2]Données!AM5</f>
-        <v>-3.8217313853343149</v>
+        <f>[1]Données!AM5</f>
+        <v>-3.3298694682483032</v>
       </c>
       <c r="AM3" s="2">
-        <f>[2]Données!AN5</f>
-        <v>-3.9448919323131437</v>
+        <f>[1]Données!AN5</f>
+        <v>-3.4586049355108339</v>
       </c>
       <c r="AN3" s="2">
-        <f>[2]Données!AO5</f>
-        <v>-4.0639667698810111</v>
+        <f>[1]Données!AO5</f>
+        <v>-3.5843660636490138</v>
       </c>
       <c r="AO3" s="2">
-        <f>[2]Données!AP5</f>
-        <v>-4.1779892250678348</v>
+        <f>[1]Données!AP5</f>
+        <v>-3.7050118103011398</v>
       </c>
       <c r="AP3" s="2">
-        <f>[2]Données!AQ5</f>
-        <v>-4.2867387241266375</v>
+        <f>[1]Données!AQ5</f>
+        <v>-3.8196946679746602</v>
       </c>
       <c r="AQ3" s="2">
-        <f>[2]Données!AR5</f>
-        <v>-4.390502402670271</v>
+        <f>[1]Données!AR5</f>
+        <v>-3.9284139939141149</v>
       </c>
       <c r="AR3" s="2">
-        <f>[2]Données!AS5</f>
-        <v>-4.4892722927368904</v>
+        <f>[1]Données!AS5</f>
+        <v>-4.0311043802415458</v>
       </c>
       <c r="AS3" s="2">
-        <f>[2]Données!AT5</f>
-        <v>-4.5838049366044631</v>
+        <f>[1]Données!AT5</f>
+        <v>-4.1285561966910578</v>
       </c>
       <c r="AT3" s="2">
-        <f>[2]Données!AU5</f>
-        <v>-4.6750075756943232</v>
+        <f>[1]Données!AU5</f>
+        <v>-4.2217238538301398</v>
       </c>
       <c r="AU3" s="2">
-        <f>[2]Données!AV5</f>
-        <v>-4.7638116158136619</v>
+        <f>[1]Données!AV5</f>
+        <v>-4.3115756484463645</v>
       </c>
       <c r="AV3" s="2">
-        <f>[2]Données!AW5</f>
-        <v>-4.846398105559679</v>
+        <f>[1]Données!AW5</f>
+        <v>-4.3942363300482956</v>
       </c>
       <c r="AW3" s="2">
-        <f>[2]Données!AX5</f>
-        <v>-4.9270733084887386</v>
+        <f>[1]Données!AX5</f>
+        <v>-4.4740494333338372</v>
       </c>
       <c r="AX3" s="2">
-        <f>[2]Données!AY5</f>
-        <v>-5.0064980472733112</v>
+        <f>[1]Données!AY5</f>
+        <v>-4.5517155106424845</v>
       </c>
       <c r="AY3" s="2">
-        <f>[2]Données!AZ5</f>
-        <v>-5.0852468488815639</v>
+        <f>[1]Données!AZ5</f>
+        <v>-4.62785514652444</v>
       </c>
       <c r="AZ3" s="2">
-        <f>[2]Données!BA5</f>
-        <v>-5.1637059738566133</v>
+        <f>[1]Données!BA5</f>
+        <v>-4.7029129923123918</v>
       </c>
       <c r="BA3" s="2">
-        <f>[2]Données!BB5</f>
-        <v>-5.2500419439234447</v>
+        <f>[1]Données!BB5</f>
+        <v>-4.7830278797077135</v>
       </c>
       <c r="BB3" s="2">
-        <f>[2]Données!BC5</f>
-        <v>-5.3254923794368807</v>
+        <f>[1]Données!BC5</f>
+        <v>-4.8544075338204928</v>
       </c>
       <c r="BC3" s="2">
-        <f>[2]Données!BD5</f>
-        <v>-5.397441557757543</v>
+        <f>[1]Données!BD5</f>
+        <v>-4.9210608415859785</v>
       </c>
       <c r="BD3" s="2">
-        <f>[2]Données!BE5</f>
-        <v>-5.468206895285399</v>
+        <f>[1]Données!BE5</f>
+        <v>-4.9856538183401966</v>
       </c>
       <c r="BE3" s="2">
-        <f>[2]Données!BF5</f>
-        <v>-5.538953308007299</v>
+        <f>[1]Données!BF5</f>
+        <v>-5.0496839947415602</v>
       </c>
       <c r="BF3" s="2">
-        <f>[2]Données!BG5</f>
-        <v>-5.6100666583201564</v>
+        <f>[1]Données!BG5</f>
+        <v>-5.1135554786895021</v>
       </c>
       <c r="BG3" s="2">
-        <f>[2]Données!BH5</f>
-        <v>-5.6811461839669679</v>
+        <f>[1]Données!BH5</f>
+        <v>-5.1768943216846441</v>
       </c>
       <c r="BH3" s="2">
-        <f>[2]Données!BI5</f>
-        <v>-5.7521787639958966</v>
+        <f>[1]Données!BI5</f>
+        <v>-5.2396944642549297</v>
       </c>
       <c r="BI3" s="2">
-        <f>[2]Données!BJ5</f>
-        <v>-5.8230693764018344</v>
+        <f>[1]Données!BJ5</f>
+        <v>-5.3018812932491333</v>
       </c>
       <c r="BJ3" s="2">
-        <f>[2]Données!BK5</f>
-        <v>-5.8937551804897019</v>
+        <f>[1]Données!BK5</f>
+        <v>-5.3634251937807242</v>
       </c>
       <c r="BK3" s="2">
-        <f>[2]Données!BL5</f>
-        <v>-5.9627310400813149</v>
+        <f>[1]Données!BL5</f>
+        <v>-5.4228491107412014</v>
       </c>
       <c r="BL3" s="2">
-        <f>[2]Données!BM5</f>
-        <v>-6.0312211491092116</v>
+        <f>[1]Données!BM5</f>
+        <v>-5.4814252718631273</v>
       </c>
       <c r="BM3" s="2">
-        <f>[2]Données!BN5</f>
-        <v>-6.0993719673605673</v>
+        <f>[1]Données!BN5</f>
+        <v>-5.5393356659288457</v>
       </c>
       <c r="BN3" s="2">
-        <f>[2]Données!BO5</f>
-        <v>-6.1673530177726921</v>
+        <f>[1]Données!BO5</f>
+        <v>-5.5967782693270181</v>
       </c>
       <c r="BO3" s="2">
-        <f>[2]Données!BP5</f>
-        <v>-6.2352915712644119</v>
+        <f>[1]Données!BP5</f>
+        <v>-5.6539004613156525</v>
       </c>
       <c r="BP3" s="2">
-        <f>[2]Données!BQ5</f>
-        <v>-6.2985615324749666</v>
+        <f>[1]Données!BQ5</f>
+        <v>-5.7059328359795654</v>
       </c>
       <c r="BQ3" s="2">
-        <f>[2]Données!BR5</f>
-        <v>-6.3604577669279738</v>
+        <f>[1]Données!BR5</f>
+        <v>-5.7561970177342321</v>
       </c>
       <c r="BR3" s="2">
-        <f>[2]Données!BS5</f>
-        <v>-6.4213119370468359</v>
+        <f>[1]Données!BS5</f>
+        <v>-5.8050176666765152</v>
       </c>
       <c r="BS3" s="2">
-        <f>[2]Données!BT5</f>
-        <v>-6.4814497093279027</v>
+        <f>[1]Données!BT5</f>
+        <v>-5.8527213604684825</v>
       </c>
       <c r="BT3" s="2">
-        <f>[2]Données!BU5</f>
-        <v>-6.5411000815981835</v>
+        <f>[1]Données!BU5</f>
+        <v>-5.8995375439617082</v>
       </c>
       <c r="BU3" s="2">
-        <f>[2]Données!BV5</f>
-        <v>-6.597973463650475</v>
+        <f>[1]Données!BV5</f>
+        <v>-5.9431609779408863</v>
       </c>
       <c r="BV3" s="2">
-        <f>[2]Données!BW5</f>
-        <v>-6.6540575869920682</v>
+        <f>[1]Données!BW5</f>
+        <v>-5.9855825034606625</v>
       </c>
       <c r="BW3" s="2">
-        <f>[2]Données!BX5</f>
-        <v>-6.7095267408472932</v>
+        <f>[1]Données!BX5</f>
+        <v>-6.026967531817462</v>
       </c>
       <c r="BX3" s="2">
-        <f>[2]Données!BY5</f>
-        <v>-6.7645730315837538</v>
+        <f>[1]Données!BY5</f>
+        <v>-6.0674985976995055</v>
       </c>
       <c r="BY3" s="2">
-        <f>[2]Données!BZ5</f>
-        <v>-6.8193461873122807</v>
+        <f>[1]Données!BZ5</f>
+        <v>-6.1073155763356919</v>
       </c>
       <c r="BZ3" s="2">
-        <f>[2]Données!CA5</f>
-        <v>-6.8700194906914147</v>
+        <f>[1]Données!CA5</f>
+        <v>-6.142432726395997</v>
       </c>
       <c r="CA3" s="2">
-        <f>[2]Données!CB5</f>
-        <v>-6.9194266938419453</v>
+        <f>[1]Données!CB5</f>
+        <v>-6.1757107375436604</v>
       </c>
       <c r="CB3" s="2">
-        <f>[2]Données!CC5</f>
-        <v>-6.9678909725079947</v>
+        <f>[1]Données!CC5</f>
+        <v>-6.2074651022600573</v>
       </c>
       <c r="CC3" s="2">
-        <f>[2]Données!CD5</f>
-        <v>-7.0157234307819056</v>
+        <f>[1]Données!CD5</f>
+        <v>-6.2380089345567491</v>
       </c>
       <c r="CD3" s="2">
-        <f>[2]Données!CE5</f>
-        <v>-7.063148609647496</v>
+        <f>[1]Données!CE5</f>
+        <v>-6.267569340326407</v>
       </c>
       <c r="CE3" s="2">
-        <f>[2]Données!CF5</f>
-        <v>-7.109622597534071</v>
+        <f>[1]Données!CF5</f>
+        <v>-6.2956097179621473</v>
       </c>
       <c r="CF3" s="2">
-        <f>[2]Données!CG5</f>
-        <v>-7.1558280095632254</v>
+        <f>[1]Données!CG5</f>
+        <v>-6.3228054306053716</v>
       </c>
       <c r="CG3" s="2">
-        <f>[2]Données!CH5</f>
-        <v>-7.1946536881305363</v>
+        <f>[1]Données!CH5</f>
+        <v>-6.3492498871058123</v>
       </c>
       <c r="CH3" s="2">
-        <f>[2]Données!CI5</f>
-        <v>-7.2466119899013197</v>
+        <f>[1]Données!CI5</f>
+        <v>-6.3750187961419176</v>
       </c>
       <c r="CI3" s="2">
-        <f>[2]Données!CJ5</f>
-        <v>-6.8712948072433004</v>
+        <f>[1]Données!CJ5</f>
+        <v>-9.2488478004404406</v>
       </c>
     </row>
     <row r="5" spans="1:87" x14ac:dyDescent="0.3">
@@ -5241,319 +5269,319 @@
       </c>
       <c r="I6" s="2">
         <f t="shared" si="0"/>
-        <v>0.19161550315185405</v>
+        <v>-8.2056637038441238E-2</v>
       </c>
       <c r="J6" s="2">
         <f t="shared" si="0"/>
-        <v>0.31789887951911844</v>
+        <v>-0.21283364242431491</v>
       </c>
       <c r="K6" s="2">
         <f t="shared" si="0"/>
-        <v>6.7015030786099494E-2</v>
+        <v>-0.39025278208807412</v>
       </c>
       <c r="L6" s="2">
         <f t="shared" si="0"/>
-        <v>-0.21728167797012699</v>
+        <v>-0.59628327178540275</v>
       </c>
       <c r="M6" s="2">
         <f t="shared" si="0"/>
-        <v>-0.46886133701437016</v>
+        <v>-0.81562590353156939</v>
       </c>
       <c r="N6" s="2">
         <f t="shared" si="0"/>
-        <v>-0.67638884472317473</v>
+        <v>-1.0216278909715992</v>
       </c>
       <c r="O6" s="2">
         <f t="shared" si="0"/>
-        <v>-0.85375889954031337</v>
+        <v>-1.2032345153876411</v>
       </c>
       <c r="P6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.0207112465597246</v>
+        <v>-1.3504639790627215</v>
       </c>
       <c r="Q6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.1759379933896641</v>
+        <v>-1.4585944232260228</v>
       </c>
       <c r="R6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.307531973432452</v>
+        <v>-1.5517555857743948</v>
       </c>
       <c r="S6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.3941416492964653</v>
+        <v>-1.5951026922136013</v>
       </c>
       <c r="T6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.4508647654808193</v>
+        <v>-1.6040668534222591</v>
       </c>
       <c r="U6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.4919916852337844</v>
+        <v>-1.5931250202945058</v>
       </c>
       <c r="V6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.5264967867797408</v>
+        <v>-1.5713350192618547</v>
       </c>
       <c r="W6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.5576296940993828</v>
+        <v>-1.5651218195565586</v>
       </c>
       <c r="X6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.5861667841999827</v>
+        <v>-1.554404043652069</v>
       </c>
       <c r="Y6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6118588854758364</v>
+        <v>-1.5381127661592275</v>
       </c>
       <c r="Z6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6342925349397075</v>
+        <v>-1.5150887663259005</v>
       </c>
       <c r="AA6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6529130346936594</v>
+        <v>-1.4843693729708951</v>
       </c>
       <c r="AB6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6664774336045296</v>
+        <v>-1.4670959735900491</v>
       </c>
       <c r="AC6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6738659693794067</v>
+        <v>-1.4415172238670282</v>
       </c>
       <c r="AD6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6767182125922653</v>
+        <v>-1.4083443590699352</v>
       </c>
       <c r="AE6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.677493043235545</v>
+        <v>-1.369330271902458</v>
       </c>
       <c r="AF6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6779763018033189</v>
+        <v>-1.3259532326168944</v>
       </c>
       <c r="AG6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6790908599914611</v>
+        <v>-1.3024859273049971</v>
       </c>
       <c r="AH6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6807531170653367</v>
+        <v>-1.2777267899411027</v>
       </c>
       <c r="AI6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6849090679153078</v>
+        <v>-1.2527233993570031</v>
       </c>
       <c r="AJ6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6952498621138901</v>
+        <v>-1.2304848598072127</v>
       </c>
       <c r="AK6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7184393048263136</v>
+        <v>-1.2174546113713047</v>
       </c>
       <c r="AL6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7362029288578218</v>
+        <v>-1.237908577251623</v>
       </c>
       <c r="AM6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7534246166071354</v>
+        <v>-1.2603538312162543</v>
       </c>
       <c r="AN6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7675856069250262</v>
+        <v>-1.280896991656888</v>
       </c>
       <c r="AO6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7775623333425861</v>
+        <v>-1.297188457191123</v>
       </c>
       <c r="AP6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7830030310172607</v>
+        <v>-1.3082209222382457</v>
       </c>
       <c r="AQ6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7843857765953541</v>
+        <v>-1.3141866871164254</v>
       </c>
       <c r="AR6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7814809968153322</v>
+        <v>-1.3148074597939763</v>
       </c>
       <c r="AS6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7750230330517369</v>
+        <v>-1.3108556960684137</v>
       </c>
       <c r="AT6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7659091624286583</v>
+        <v>-1.303275763656131</v>
       </c>
       <c r="AU6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7550687062752313</v>
+        <v>-1.2930319435366266</v>
       </c>
       <c r="AV6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7437581416538506</v>
+        <v>-1.281342220396231</v>
       </c>
       <c r="AW6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7322399317636572</v>
+        <v>-1.2684877326585298</v>
       </c>
       <c r="AX6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7209837178788767</v>
+        <v>-1.2549757446242316</v>
       </c>
       <c r="AY6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7102969143967806</v>
+        <v>-1.2411581680791373</v>
       </c>
       <c r="AZ6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7003514750675741</v>
+        <v>-1.2272642485102625</v>
       </c>
       <c r="BA6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.7041717945534995</v>
+        <v>-1.2242065628020882</v>
       </c>
       <c r="BB6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6968611913178111</v>
+        <v>-1.212274094328003</v>
       </c>
       <c r="BC6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6874204618492761</v>
+        <v>-1.1969362266087136</v>
       </c>
       <c r="BD6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6779987060296264</v>
+        <v>-1.18070260801586</v>
       </c>
       <c r="BE6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6695997980133215</v>
+        <v>-1.16492077109287</v>
       </c>
       <c r="BF6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6637538837163346</v>
+        <v>-1.1511401161751533</v>
       </c>
       <c r="BG6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6589740264339237</v>
+        <v>-1.1378958971931308</v>
       </c>
       <c r="BH6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6551568536300354</v>
+        <v>-1.1250898290850242</v>
       </c>
       <c r="BI6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6521136575608164</v>
+        <v>-1.1125532871455235</v>
       </c>
       <c r="BJ6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6496961346720851</v>
+        <v>-1.1001719824118905</v>
       </c>
       <c r="BK6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.647812183467412</v>
+        <v>-1.0878917622401674</v>
       </c>
       <c r="BL6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6464745156678506</v>
+        <v>-1.0757687980817221</v>
       </c>
       <c r="BM6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6457143828054077</v>
+        <v>-1.063870997528682</v>
       </c>
       <c r="BN6" s="2">
         <f t="shared" si="0"/>
-        <v>-1.6455781760776222</v>
+        <v>-1.0522736454812165</v>
       </c>
       <c r="BO6" s="2">
         <f t="shared" ref="BO6:CI6" si="1">BO2</f>
-        <v>-1.6461074372563056</v>
+        <v>-1.0410385324777782</v>
       </c>
       <c r="BP6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.6484945595247713</v>
+        <v>-1.0312423250512404</v>
       </c>
       <c r="BQ6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.6513493411040914</v>
+        <v>-1.0214957006012715</v>
       </c>
       <c r="BR6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.6547799298626154</v>
+        <v>-1.0118976129306012</v>
       </c>
       <c r="BS6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.6588215817661012</v>
+        <v>-1.0024819779150707</v>
       </c>
       <c r="BT6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.663474348417826</v>
+        <v>-0.99324739033723741</v>
       </c>
       <c r="BU6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.668749189340446</v>
+        <v>-0.98420512175648733</v>
       </c>
       <c r="BV6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.6745957993986593</v>
+        <v>-0.97529371947724375</v>
       </c>
       <c r="BW6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.6809976191283882</v>
+        <v>-0.96648595744011079</v>
       </c>
       <c r="BX6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.6879396819433956</v>
+        <v>-0.9577552203525963</v>
       </c>
       <c r="BY6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.6954091313694963</v>
+        <v>-0.94907697959949466</v>
       </c>
       <c r="BZ6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.7043809443399893</v>
+        <v>-0.94129484741348746</v>
       </c>
       <c r="CA6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.7136818328981618</v>
+        <v>-0.93323535150678927</v>
       </c>
       <c r="CB6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.7233900154516202</v>
+        <v>-0.9249666077962293</v>
       </c>
       <c r="CC6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.733529893763619</v>
+        <v>-0.91651274199079369</v>
       </c>
       <c r="CD6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.7441041249341871</v>
+        <v>-0.90787715348179532</v>
       </c>
       <c r="CE6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.7551879809414861</v>
+        <v>-0.89914837199471798</v>
       </c>
       <c r="CF6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.7666911636200933</v>
+        <v>-0.8902214872785974</v>
       </c>
       <c r="CG6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.7709894968797713</v>
+        <v>-0.88109715314373949</v>
       </c>
       <c r="CH6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.7897149040786542</v>
+        <v>-0.87177687957782357</v>
       </c>
       <c r="CI6" s="2">
         <f t="shared" si="1"/>
-        <v>-1.3563380790536539</v>
+        <v>-9.2488478004404406</v>
       </c>
     </row>
     <row r="7" spans="1:87" x14ac:dyDescent="0.3">
@@ -5590,319 +5618,319 @@
       </c>
       <c r="I7" s="2">
         <f t="shared" si="2"/>
-        <v>2.1869550496589341E-2</v>
+        <v>2.2292788023148269E-2</v>
       </c>
       <c r="J7" s="2">
         <f t="shared" si="2"/>
-        <v>3.1205429864034073E-2</v>
+        <v>3.2139088170790586E-2</v>
       </c>
       <c r="K7" s="2">
         <f t="shared" si="2"/>
-        <v>4.0713713050877232E-2</v>
+        <v>4.2129485191733096E-2</v>
       </c>
       <c r="L7" s="2">
         <f t="shared" si="2"/>
-        <v>5.0225662190184206E-2</v>
+        <v>5.1975242771151731E-2</v>
       </c>
       <c r="M7" s="2">
         <f t="shared" si="2"/>
-        <v>3.4202433463459414E-2</v>
+        <v>3.6017857349646132E-2</v>
       </c>
       <c r="N7" s="2">
         <f t="shared" si="2"/>
-        <v>1.4793136806567908E-2</v>
+        <v>1.6399497469810065E-2</v>
       </c>
       <c r="O7" s="2">
         <f t="shared" si="2"/>
-        <v>-7.2514210232244025E-3</v>
+        <v>-5.9892217015078408E-3</v>
       </c>
       <c r="P7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.085749985403119E-2</v>
+        <v>-2.9968546411729413E-2</v>
       </c>
       <c r="Q7" s="2">
         <f t="shared" si="2"/>
-        <v>-5.5171737536308108E-2</v>
+        <v>-5.4577153530033229E-2</v>
       </c>
       <c r="R7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.11527060202289885</v>
+        <v>-0.11463976727003056</v>
       </c>
       <c r="S7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.18005917742343058</v>
+        <v>-0.17919008783575663</v>
       </c>
       <c r="T7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.24835479296698715</v>
+        <v>-0.24713328455195915</v>
       </c>
       <c r="U7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.31854407319406031</v>
+        <v>-0.31695567151074355</v>
       </c>
       <c r="V7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.38934787782083369</v>
+        <v>-0.38745994979798581</v>
       </c>
       <c r="W7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.48466297679704562</v>
+        <v>-0.48250703231480507</v>
       </c>
       <c r="X7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.58310328090575014</v>
+        <v>-0.58080471991275306</v>
       </c>
       <c r="Y7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.68367940434092001</v>
+        <v>-0.68138580947760818</v>
       </c>
       <c r="Z7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.78519266864072179</v>
+        <v>-0.78306998913987291</v>
       </c>
       <c r="AA7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.88673461819119836</v>
+        <v>-0.88496209607368259</v>
       </c>
       <c r="AB7" s="2">
         <f t="shared" si="2"/>
-        <v>-0.99484702484020637</v>
+        <v>-0.99340996282157867</v>
       </c>
       <c r="AC7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.1032786996437394</v>
+        <v>-1.1022916149202144</v>
       </c>
       <c r="AD7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.2116345953177454</v>
+        <v>-1.2112272072063335</v>
       </c>
       <c r="AE7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.3194987188833385</v>
+        <v>-1.3198210676801048</v>
       </c>
       <c r="AF7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.4265799471028462</v>
+        <v>-1.4277976274376325</v>
       </c>
       <c r="AG7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.537828170077804</v>
+        <v>-1.5397852860289496</v>
       </c>
       <c r="AH7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.648887146879241</v>
+        <v>-1.6516752493175968</v>
       </c>
       <c r="AI7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.7595417723946905</v>
+        <v>-1.7632678954715209</v>
       </c>
       <c r="AJ7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.86950345626683</v>
+        <v>-1.8742920847076738</v>
       </c>
       <c r="AK7" s="2">
         <f t="shared" si="2"/>
-        <v>-1.9784768298969579</v>
+        <v>-1.9844642318590289</v>
       </c>
       <c r="AL7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.0855284564764931</v>
+        <v>-2.0919608909966803</v>
       </c>
       <c r="AM7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.1914673157060083</v>
+        <v>-2.1982511042945796</v>
       </c>
       <c r="AN7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.2963811629559849</v>
+        <v>-2.3034690719921258</v>
       </c>
       <c r="AO7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.4004268917252487</v>
+        <v>-2.4078233531100168</v>
       </c>
       <c r="AP7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.5037356931093768</v>
+        <v>-2.5114737457364145</v>
       </c>
       <c r="AQ7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.6061166260749169</v>
+        <v>-2.6142273067976896</v>
       </c>
       <c r="AR7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.7077912959215582</v>
+        <v>-2.7162969204475695</v>
       </c>
       <c r="AS7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.8087819035527262</v>
+        <v>-2.8177005006226441</v>
       </c>
       <c r="AT7" s="2">
         <f t="shared" si="2"/>
-        <v>-2.909098413265665</v>
+        <v>-2.9184480901740089</v>
       </c>
       <c r="AU7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.0087429095384306</v>
+        <v>-3.0185437049097379</v>
       </c>
       <c r="AV7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.1026399639058284</v>
+        <v>-3.1128941096520646</v>
       </c>
       <c r="AW7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.1948333767250814</v>
+        <v>-3.2055617006753074</v>
       </c>
       <c r="AX7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.2855143293944344</v>
+        <v>-3.2967397660182529</v>
       </c>
       <c r="AY7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.3749499344847833</v>
+        <v>-3.3866969784453027</v>
       </c>
       <c r="AZ7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.4633544987890392</v>
+        <v>-3.4756487438021293</v>
       </c>
       <c r="BA7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.5458701493699452</v>
+        <v>-3.5588213169056253</v>
       </c>
       <c r="BB7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.6286311881190696</v>
+        <v>-3.6421334394924898</v>
       </c>
       <c r="BC7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.7100210959082669</v>
+        <v>-3.7241246149772649</v>
       </c>
       <c r="BD7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.7902081892557726</v>
+        <v>-3.8049512103243366</v>
       </c>
       <c r="BE7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.8693535099939775</v>
+        <v>-3.8847632236486902</v>
       </c>
       <c r="BF7" s="2">
         <f t="shared" si="2"/>
-        <v>-3.9463127746038218</v>
+        <v>-3.9624153625143488</v>
       </c>
       <c r="BG7" s="2">
         <f t="shared" si="2"/>
-        <v>-4.0221721575330438</v>
+        <v>-4.0389984244915134</v>
       </c>
       <c r="BH7" s="2">
         <f t="shared" si="2"/>
-        <v>-4.0970219103658607</v>
+        <v>-4.1146046351699059</v>
       </c>
       <c r="BI7" s="2">
         <f t="shared" si="2"/>
-        <v>-4.170955718841018</v>
+        <v>-4.1893280061036098</v>
       </c>
       <c r="BJ7" s="2">
         <f t="shared" si="2"/>
-        <v>-4.2440590458176164</v>
+        <v>-4.2632532113688342</v>
       </c>
       <c r="BK7" s="2">
         <f t="shared" si="2"/>
-        <v>-4.314918856613903</v>
+        <v>-4.3349573485010335</v>
       </c>
       <c r="BL7" s="2">
         <f t="shared" si="2"/>
-        <v>-4.3847466334413614</v>
+        <v>-4.4056564737814057</v>
       </c>
       <c r="BM7" s="2">
         <f t="shared" si="2"/>
-        <v>-4.4536575845551596</v>
+        <v>-4.4754646684001642</v>
       </c>
       <c r="BN7" s="2">
         <f t="shared" si="2"/>
-        <v>-4.5217748416950698</v>
+        <v>-4.5445046238458016</v>
       </c>
       <c r="BO7" s="2">
         <f t="shared" ref="BO7:CI7" si="3">BO3-BO2</f>
-        <v>-4.5891841340081063</v>
+        <v>-4.6128619288378747</v>
       </c>
       <c r="BP7" s="2">
         <f t="shared" si="3"/>
-        <v>-4.6500669729501958</v>
+        <v>-4.6746905109283254</v>
       </c>
       <c r="BQ7" s="2">
         <f t="shared" si="3"/>
-        <v>-4.7091084258238824</v>
+        <v>-4.7347013171329611</v>
       </c>
       <c r="BR7" s="2">
         <f t="shared" si="3"/>
-        <v>-4.766532007184221</v>
+        <v>-4.7931200537459144</v>
       </c>
       <c r="BS7" s="2">
         <f t="shared" si="3"/>
-        <v>-4.822628127561801</v>
+        <v>-4.8502393825534114</v>
       </c>
       <c r="BT7" s="2">
         <f t="shared" si="3"/>
-        <v>-4.8776257331803574</v>
+        <v>-4.9062901536244707</v>
       </c>
       <c r="BU7" s="2">
         <f t="shared" si="3"/>
-        <v>-4.9292242743100285</v>
+        <v>-4.9589558561843994</v>
       </c>
       <c r="BV7" s="2">
         <f t="shared" si="3"/>
-        <v>-4.9794617875934089</v>
+        <v>-5.0102887839834187</v>
       </c>
       <c r="BW7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.028529121718905</v>
+        <v>-5.0604815743773512</v>
       </c>
       <c r="BX7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.0766333496403586</v>
+        <v>-5.1097433773469092</v>
       </c>
       <c r="BY7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.1239370559427844</v>
+        <v>-5.1582385967361972</v>
       </c>
       <c r="BZ7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.1656385463514258</v>
+        <v>-5.2011378789825091</v>
       </c>
       <c r="CA7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.2057448609437831</v>
+        <v>-5.2424753860368707</v>
       </c>
       <c r="CB7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.2445009570563741</v>
+        <v>-5.2824984944638285</v>
       </c>
       <c r="CC7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.2821935370182871</v>
+        <v>-5.3214961925659559</v>
       </c>
       <c r="CD7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.3190444847133094</v>
+        <v>-5.3596921868446117</v>
       </c>
       <c r="CE7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.3544346165925845</v>
+        <v>-5.3964613459674293</v>
       </c>
       <c r="CF7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.3891368459431321</v>
+        <v>-5.4325839433267742</v>
       </c>
       <c r="CG7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.423664191250765</v>
+        <v>-5.4681527339620732</v>
       </c>
       <c r="CH7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.456897085822666</v>
+        <v>-5.503241916564094</v>
       </c>
       <c r="CI7" s="2">
         <f t="shared" si="3"/>
-        <v>-5.514956728189647</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:87" x14ac:dyDescent="0.3">
@@ -5939,319 +5967,319 @@
       </c>
       <c r="I8" s="2">
         <f t="shared" si="4"/>
-        <v>0.21348505364844339</v>
+        <v>-5.9763849015292969E-2</v>
       </c>
       <c r="J8" s="2">
         <f t="shared" si="4"/>
-        <v>0.34910430938315251</v>
+        <v>-0.18069455425352432</v>
       </c>
       <c r="K8" s="2">
         <f t="shared" si="4"/>
-        <v>0.10772874383697673</v>
+        <v>-0.34812329689634103</v>
       </c>
       <c r="L8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.16705601577994278</v>
+        <v>-0.54430802901425102</v>
       </c>
       <c r="M8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.43465890355091075</v>
+        <v>-0.77960804618192325</v>
       </c>
       <c r="N8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.66159570791660682</v>
+        <v>-1.0052283935017892</v>
       </c>
       <c r="O8" s="2">
         <f t="shared" si="4"/>
-        <v>-0.86101032056353777</v>
+        <v>-1.209223737089149</v>
       </c>
       <c r="P8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.0515687464137558</v>
+        <v>-1.3804325254744509</v>
       </c>
       <c r="Q8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.2311097309259722</v>
+        <v>-1.5131715767560561</v>
       </c>
       <c r="R8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.4228025754553508</v>
+        <v>-1.6663953530444253</v>
       </c>
       <c r="S8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.5742008267198959</v>
+        <v>-1.774292780049358</v>
       </c>
       <c r="T8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.6992195584478065</v>
+        <v>-1.8512001379742182</v>
       </c>
       <c r="U8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.8105357584278448</v>
+        <v>-1.9100806918052493</v>
       </c>
       <c r="V8" s="2">
         <f t="shared" si="4"/>
-        <v>-1.9158446646005745</v>
+        <v>-1.9587949690598405</v>
       </c>
       <c r="W8" s="2">
         <f t="shared" si="4"/>
-        <v>-2.0422926708964284</v>
+        <v>-2.0476288518713637</v>
       </c>
       <c r="X8" s="2">
         <f t="shared" si="4"/>
-        <v>-2.1692700651057328</v>
+        <v>-2.135208763564822</v>
       </c>
       <c r="Y8" s="2">
         <f t="shared" si="4"/>
-        <v>-2.2955382898167564</v>
+        <v>-2.2194985756368357</v>
       </c>
       <c r="Z8" s="2">
         <f t="shared" si="4"/>
-        <v>-2.4194852035804293</v>
+        <v>-2.2981587554657734</v>
       </c>
       <c r="AA8" s="2">
         <f t="shared" si="4"/>
-        <v>-2.5396476528848577</v>
+        <v>-2.3693314690445777</v>
       </c>
       <c r="AB8" s="2">
         <f t="shared" si="4"/>
-        <v>-2.661324458444736</v>
+        <v>-2.4605059364116277</v>
       </c>
       <c r="AC8" s="2">
         <f t="shared" si="4"/>
-        <v>-2.7771446690231461</v>
+        <v>-2.5438088387872426</v>
       </c>
       <c r="AD8" s="2">
         <f t="shared" si="4"/>
-        <v>-2.8883528079100107</v>
+        <v>-2.6195715662762686</v>
       </c>
       <c r="AE8" s="2">
         <f t="shared" si="4"/>
-        <v>-2.9969917621188835</v>
+        <v>-2.6891513395825628</v>
       </c>
       <c r="AF8" s="2">
         <f t="shared" si="4"/>
-        <v>-3.1045562489061651</v>
+        <v>-2.7537508600545269</v>
       </c>
       <c r="AG8" s="2">
         <f t="shared" si="4"/>
-        <v>-3.2169190300692652</v>
+        <v>-2.8422712133339467</v>
       </c>
       <c r="AH8" s="2">
         <f t="shared" si="4"/>
-        <v>-3.3296402639445777</v>
+        <v>-2.9294020392586995</v>
       </c>
       <c r="AI8" s="2">
         <f t="shared" si="4"/>
-        <v>-3.4444508403099983</v>
+        <v>-3.0159912948285239</v>
       </c>
       <c r="AJ8" s="2">
         <f t="shared" si="4"/>
-        <v>-3.5647533183807201</v>
+        <v>-3.1047769445148865</v>
       </c>
       <c r="AK8" s="2">
         <f t="shared" si="4"/>
-        <v>-3.6969161347232715</v>
+        <v>-3.2019188432303336</v>
       </c>
       <c r="AL8" s="2">
         <f t="shared" si="4"/>
-        <v>-3.8217313853343149</v>
+        <v>-3.3298694682483032</v>
       </c>
       <c r="AM8" s="2">
         <f t="shared" si="4"/>
-        <v>-3.9448919323131437</v>
+        <v>-3.4586049355108339</v>
       </c>
       <c r="AN8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.0639667698810111</v>
+        <v>-3.5843660636490138</v>
       </c>
       <c r="AO8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.1779892250678348</v>
+        <v>-3.7050118103011398</v>
       </c>
       <c r="AP8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.2867387241266375</v>
+        <v>-3.8196946679746602</v>
       </c>
       <c r="AQ8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.390502402670271</v>
+        <v>-3.9284139939141149</v>
       </c>
       <c r="AR8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.4892722927368904</v>
+        <v>-4.0311043802415458</v>
       </c>
       <c r="AS8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.5838049366044631</v>
+        <v>-4.1285561966910578</v>
       </c>
       <c r="AT8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.6750075756943232</v>
+        <v>-4.2217238538301398</v>
       </c>
       <c r="AU8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.7638116158136619</v>
+        <v>-4.3115756484463645</v>
       </c>
       <c r="AV8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.846398105559679</v>
+        <v>-4.3942363300482956</v>
       </c>
       <c r="AW8" s="2">
         <f t="shared" si="4"/>
-        <v>-4.9270733084887386</v>
+        <v>-4.4740494333338372</v>
       </c>
       <c r="AX8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.0064980472733112</v>
+        <v>-4.5517155106424845</v>
       </c>
       <c r="AY8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.0852468488815639</v>
+        <v>-4.62785514652444</v>
       </c>
       <c r="AZ8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.1637059738566133</v>
+        <v>-4.7029129923123918</v>
       </c>
       <c r="BA8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.2500419439234447</v>
+        <v>-4.7830278797077135</v>
       </c>
       <c r="BB8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.3254923794368807</v>
+        <v>-4.8544075338204928</v>
       </c>
       <c r="BC8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.397441557757543</v>
+        <v>-4.9210608415859785</v>
       </c>
       <c r="BD8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.468206895285399</v>
+        <v>-4.9856538183401966</v>
       </c>
       <c r="BE8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.538953308007299</v>
+        <v>-5.0496839947415602</v>
       </c>
       <c r="BF8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.6100666583201564</v>
+        <v>-5.1135554786895021</v>
       </c>
       <c r="BG8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.6811461839669679</v>
+        <v>-5.1768943216846441</v>
       </c>
       <c r="BH8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.7521787639958966</v>
+        <v>-5.2396944642549297</v>
       </c>
       <c r="BI8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.8230693764018344</v>
+        <v>-5.3018812932491333</v>
       </c>
       <c r="BJ8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.8937551804897019</v>
+        <v>-5.3634251937807242</v>
       </c>
       <c r="BK8" s="2">
         <f t="shared" si="4"/>
-        <v>-5.9627310400813149</v>
+        <v>-5.4228491107412014</v>
       </c>
       <c r="BL8" s="2">
         <f t="shared" si="4"/>
-        <v>-6.0312211491092116</v>
+        <v>-5.4814252718631273</v>
       </c>
       <c r="BM8" s="2">
         <f t="shared" si="4"/>
-        <v>-6.0993719673605673</v>
+        <v>-5.5393356659288457</v>
       </c>
       <c r="BN8" s="2">
         <f t="shared" si="4"/>
-        <v>-6.1673530177726921</v>
+        <v>-5.5967782693270181</v>
       </c>
       <c r="BO8" s="2">
         <f t="shared" ref="BO8:CI8" si="5">BO3</f>
-        <v>-6.2352915712644119</v>
+        <v>-5.6539004613156525</v>
       </c>
       <c r="BP8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.2985615324749666</v>
+        <v>-5.7059328359795654</v>
       </c>
       <c r="BQ8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.3604577669279738</v>
+        <v>-5.7561970177342321</v>
       </c>
       <c r="BR8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.4213119370468359</v>
+        <v>-5.8050176666765152</v>
       </c>
       <c r="BS8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.4814497093279027</v>
+        <v>-5.8527213604684825</v>
       </c>
       <c r="BT8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.5411000815981835</v>
+        <v>-5.8995375439617082</v>
       </c>
       <c r="BU8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.597973463650475</v>
+        <v>-5.9431609779408863</v>
       </c>
       <c r="BV8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.6540575869920682</v>
+        <v>-5.9855825034606625</v>
       </c>
       <c r="BW8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.7095267408472932</v>
+        <v>-6.026967531817462</v>
       </c>
       <c r="BX8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.7645730315837538</v>
+        <v>-6.0674985976995055</v>
       </c>
       <c r="BY8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.8193461873122807</v>
+        <v>-6.1073155763356919</v>
       </c>
       <c r="BZ8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.8700194906914147</v>
+        <v>-6.142432726395997</v>
       </c>
       <c r="CA8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.9194266938419453</v>
+        <v>-6.1757107375436604</v>
       </c>
       <c r="CB8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.9678909725079947</v>
+        <v>-6.2074651022600573</v>
       </c>
       <c r="CC8" s="2">
         <f t="shared" si="5"/>
-        <v>-7.0157234307819056</v>
+        <v>-6.2380089345567491</v>
       </c>
       <c r="CD8" s="2">
         <f t="shared" si="5"/>
-        <v>-7.063148609647496</v>
+        <v>-6.267569340326407</v>
       </c>
       <c r="CE8" s="2">
         <f t="shared" si="5"/>
-        <v>-7.109622597534071</v>
+        <v>-6.2956097179621473</v>
       </c>
       <c r="CF8" s="2">
         <f t="shared" si="5"/>
-        <v>-7.1558280095632254</v>
+        <v>-6.3228054306053716</v>
       </c>
       <c r="CG8" s="2">
         <f t="shared" si="5"/>
-        <v>-7.1946536881305363</v>
+        <v>-6.3492498871058123</v>
       </c>
       <c r="CH8" s="2">
         <f t="shared" si="5"/>
-        <v>-7.2466119899013197</v>
+        <v>-6.3750187961419176</v>
       </c>
       <c r="CI8" s="2">
         <f t="shared" si="5"/>
-        <v>-6.8712948072433004</v>
+        <v>-9.2488478004404406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>